<commit_message>
learning to draw landscapes published
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20600" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20600" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;yes&quot;\,&quot;yes&quot;\,&quot;yes&quot;\,&quot;yes&quot;"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -145,7 +146,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -214,6 +215,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -615,7 +618,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C54"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
   <cols>
     <col width="21.83203125" customWidth="1" style="4" min="1" max="1"/>
     <col width="75.83203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1399,15 +1402,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y169"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <dimension ref="A1:Y189"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
   <cols>
     <col width="11.33203125" customWidth="1" style="7" min="1" max="1"/>
     <col width="13.33203125" customWidth="1" style="7" min="2" max="2"/>
     <col width="17" bestFit="1" customWidth="1" style="28" min="3" max="3"/>
-    <col width="22.6640625" customWidth="1" style="7" min="4" max="4"/>
-    <col width="31.6640625" customWidth="1" style="7" min="5" max="5"/>
-    <col width="27.6640625" customWidth="1" style="7" min="6" max="6"/>
+    <col width="29.1640625" bestFit="1" customWidth="1" style="7" min="4" max="4"/>
+    <col width="43.1640625" bestFit="1" customWidth="1" style="7" min="5" max="5"/>
+    <col width="72.83203125" bestFit="1" customWidth="1" style="7" min="6" max="6"/>
     <col width="13.1640625" customWidth="1" style="7" min="7" max="7"/>
     <col width="14" customWidth="1" style="7" min="8" max="8"/>
     <col width="10.83203125" customWidth="1" style="7" min="9" max="9"/>
@@ -1426,8 +1429,8 @@
     <col width="21.5" customWidth="1" style="7" min="23" max="23"/>
     <col width="26.83203125" customWidth="1" style="7" min="24" max="24"/>
     <col width="20.83203125" customWidth="1" style="7" min="25" max="25"/>
-    <col width="10.83203125" customWidth="1" style="7" min="26" max="43"/>
-    <col width="10.83203125" customWidth="1" style="7" min="44" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="26" max="46"/>
+    <col width="10.83203125" customWidth="1" style="7" min="47" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="6">
@@ -12369,6 +12372,1280 @@
         </is>
       </c>
       <c r="X169" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="22" t="inlineStr">
+        <is>
+          <t>00516</t>
+        </is>
+      </c>
+      <c r="B170" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C170" s="16" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D170" s="32" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="E170" s="7" t="inlineStr">
+        <is>
+          <t>landscape 1.jpg</t>
+        </is>
+      </c>
+      <c r="F170" s="7" t="inlineStr">
+        <is>
+          <t>landscape 1</t>
+        </is>
+      </c>
+      <c r="G170" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H170" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="I170" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J170" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K170" s="32" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="L170" s="7" t="inlineStr">
+        <is>
+          <t>digital print</t>
+        </is>
+      </c>
+      <c r="M170" s="7" t="inlineStr">
+        <is>
+          <t>digital c-type print</t>
+        </is>
+      </c>
+      <c r="X170" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="22" t="inlineStr">
+        <is>
+          <t>00517</t>
+        </is>
+      </c>
+      <c r="B171" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C171" s="16" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D171" s="32" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="E171" s="7" t="inlineStr">
+        <is>
+          <t>landscape 2.jpg</t>
+        </is>
+      </c>
+      <c r="F171" s="7" t="inlineStr">
+        <is>
+          <t>landscape 2</t>
+        </is>
+      </c>
+      <c r="G171" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H171" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="I171" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J171" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K171" s="32" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="L171" s="7" t="inlineStr">
+        <is>
+          <t>digital print</t>
+        </is>
+      </c>
+      <c r="M171" s="7" t="inlineStr">
+        <is>
+          <t>digital c-type print</t>
+        </is>
+      </c>
+      <c r="X171" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="22" t="inlineStr">
+        <is>
+          <t>00518</t>
+        </is>
+      </c>
+      <c r="B172" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C172" s="16" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D172" s="32" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="E172" s="7" t="inlineStr">
+        <is>
+          <t>landscape 2.1.jpg</t>
+        </is>
+      </c>
+      <c r="F172" s="7" t="inlineStr">
+        <is>
+          <t>landscape 2.1</t>
+        </is>
+      </c>
+      <c r="G172" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H172" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="I172" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J172" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K172" s="32" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="L172" s="7" t="inlineStr">
+        <is>
+          <t>digital print</t>
+        </is>
+      </c>
+      <c r="M172" s="7" t="inlineStr">
+        <is>
+          <t>digital c-type print</t>
+        </is>
+      </c>
+      <c r="X172" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="22" t="inlineStr">
+        <is>
+          <t>00114</t>
+        </is>
+      </c>
+      <c r="B173" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C173" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D173" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E173" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 1.jpg</t>
+        </is>
+      </c>
+      <c r="F173" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 1</t>
+        </is>
+      </c>
+      <c r="G173" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H173" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I173" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J173" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K173" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L173" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M173" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X173" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="22" t="inlineStr">
+        <is>
+          <t>00115</t>
+        </is>
+      </c>
+      <c r="B174" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C174" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D174" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E174" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 2.jpg</t>
+        </is>
+      </c>
+      <c r="F174" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 2</t>
+        </is>
+      </c>
+      <c r="G174" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H174" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I174" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J174" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K174" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L174" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M174" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X174" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="22" t="inlineStr">
+        <is>
+          <t>00116</t>
+        </is>
+      </c>
+      <c r="B175" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C175" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D175" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E175" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 3.jpg</t>
+        </is>
+      </c>
+      <c r="F175" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 3</t>
+        </is>
+      </c>
+      <c r="G175" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H175" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I175" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J175" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K175" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L175" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M175" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X175" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="22" t="inlineStr">
+        <is>
+          <t>00117</t>
+        </is>
+      </c>
+      <c r="B176" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C176" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D176" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E176" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 4.jpg</t>
+        </is>
+      </c>
+      <c r="F176" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 4</t>
+        </is>
+      </c>
+      <c r="G176" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H176" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I176" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J176" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K176" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L176" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M176" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X176" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="22" t="inlineStr">
+        <is>
+          <t>00118</t>
+        </is>
+      </c>
+      <c r="B177" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C177" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D177" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E177" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 5.jpg</t>
+        </is>
+      </c>
+      <c r="F177" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 5</t>
+        </is>
+      </c>
+      <c r="G177" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H177" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I177" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J177" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K177" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L177" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M177" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X177" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="22" t="inlineStr">
+        <is>
+          <t>00119</t>
+        </is>
+      </c>
+      <c r="B178" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C178" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D178" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E178" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 6.jpg</t>
+        </is>
+      </c>
+      <c r="F178" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 6</t>
+        </is>
+      </c>
+      <c r="G178" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H178" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I178" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J178" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K178" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L178" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M178" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X178" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="22" t="inlineStr">
+        <is>
+          <t>00120</t>
+        </is>
+      </c>
+      <c r="B179" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C179" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D179" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E179" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 7.jpg</t>
+        </is>
+      </c>
+      <c r="F179" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 7</t>
+        </is>
+      </c>
+      <c r="G179" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H179" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I179" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J179" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K179" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L179" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M179" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X179" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="22" t="inlineStr">
+        <is>
+          <t>00121</t>
+        </is>
+      </c>
+      <c r="B180" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C180" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D180" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E180" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 8.jpg</t>
+        </is>
+      </c>
+      <c r="F180" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 8</t>
+        </is>
+      </c>
+      <c r="G180" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H180" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I180" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J180" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K180" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L180" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M180" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X180" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="22" t="inlineStr">
+        <is>
+          <t>00122</t>
+        </is>
+      </c>
+      <c r="B181" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C181" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D181" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E181" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 9.jpg</t>
+        </is>
+      </c>
+      <c r="F181" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 9</t>
+        </is>
+      </c>
+      <c r="G181" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H181" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I181" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J181" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K181" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L181" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M181" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X181" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="22" t="inlineStr">
+        <is>
+          <t>00123</t>
+        </is>
+      </c>
+      <c r="B182" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C182" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D182" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E182" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 10.jpg</t>
+        </is>
+      </c>
+      <c r="F182" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 10</t>
+        </is>
+      </c>
+      <c r="G182" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H182" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I182" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J182" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K182" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L182" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M182" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X182" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="22" t="inlineStr">
+        <is>
+          <t>00124</t>
+        </is>
+      </c>
+      <c r="B183" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C183" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D183" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E183" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 11.jpg</t>
+        </is>
+      </c>
+      <c r="F183" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 11</t>
+        </is>
+      </c>
+      <c r="G183" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H183" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I183" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J183" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K183" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L183" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M183" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X183" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="22" t="inlineStr">
+        <is>
+          <t>00125</t>
+        </is>
+      </c>
+      <c r="B184" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C184" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D184" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 12.jpg</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 12</t>
+        </is>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H184" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I184" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J184" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K184" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L184" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M184" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X184" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="22" t="inlineStr">
+        <is>
+          <t>00126</t>
+        </is>
+      </c>
+      <c r="B185" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C185" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D185" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E185" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 13.jpg</t>
+        </is>
+      </c>
+      <c r="F185" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 13</t>
+        </is>
+      </c>
+      <c r="G185" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H185" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I185" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J185" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K185" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L185" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M185" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X185" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="22" t="inlineStr">
+        <is>
+          <t>00127</t>
+        </is>
+      </c>
+      <c r="B186" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C186" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D186" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 14.jpg</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 14</t>
+        </is>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H186" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I186" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J186" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K186" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L186" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M186" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X186" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="22" t="inlineStr">
+        <is>
+          <t>00128</t>
+        </is>
+      </c>
+      <c r="B187" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C187" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D187" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E187" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 15.jpg</t>
+        </is>
+      </c>
+      <c r="F187" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 15</t>
+        </is>
+      </c>
+      <c r="G187" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H187" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I187" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J187" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K187" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L187" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M187" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X187" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="22" t="inlineStr">
+        <is>
+          <t>00129</t>
+        </is>
+      </c>
+      <c r="B188" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C188" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D188" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 16.jpg</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes 16</t>
+        </is>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H188" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I188" s="7" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J188" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?</t>
+        </is>
+      </c>
+      <c r="K188" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L188" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M188" s="7" t="inlineStr">
+        <is>
+          <t>pencil on paper</t>
+        </is>
+      </c>
+      <c r="X188" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B189" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C189" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D189" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="E189" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes (versions).jpg</t>
+        </is>
+      </c>
+      <c r="F189" s="7" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes (versions)</t>
+        </is>
+      </c>
+      <c r="G189" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="H189" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="I189" s="7" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J189" s="7" t="inlineStr">
+        <is>
+          <t>c. 2022?</t>
+        </is>
+      </c>
+      <c r="K189" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="L189" s="7" t="inlineStr">
+        <is>
+          <t>digital print</t>
+        </is>
+      </c>
+      <c r="M189" s="7" t="inlineStr">
+        <is>
+          <t>digital c-type print</t>
+        </is>
+      </c>
+      <c r="X189" s="22" t="inlineStr">
         <is>
           <t>Michael Davies</t>
         </is>
@@ -12386,11 +13663,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
   <cols>
-    <col width="25.83203125" customWidth="1" style="1" min="1" max="1"/>
-    <col width="24.83203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
+    <col width="31.83203125" customWidth="1" style="1" min="1" max="1"/>
+    <col width="43.1640625" customWidth="1" style="1" min="2" max="2"/>
     <col width="20.83203125" customWidth="1" style="1" min="3" max="3"/>
     <col width="17" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
     <col width="10.83203125" customWidth="1" style="1" min="5" max="5"/>
@@ -12398,8 +13675,8 @@
     <col width="21" customWidth="1" style="7" min="7" max="7"/>
     <col width="28.1640625" customWidth="1" style="7" min="8" max="8"/>
     <col width="51" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
-    <col width="10.83203125" customWidth="1" style="1" min="10" max="28"/>
-    <col width="10.83203125" customWidth="1" style="1" min="29" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="1" min="10" max="31"/>
+    <col width="10.83203125" customWidth="1" style="1" min="32" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="3">
@@ -12890,6 +14167,80 @@
       <c r="I13" s="1" t="inlineStr">
         <is>
           <t>add dall-e versions</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>landscapes</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>46071</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>00516</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>landscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>learning-to-draw-landscapes</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>learning to draw landscapes</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>c. 2010?, 2022</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>00127</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>landscape,drawing</t>
         </is>
       </c>
     </row>
@@ -12904,8 +14255,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J372"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <dimension ref="A1:J447"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
   <cols>
     <col width="9.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="9.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -28186,6 +29537,3081 @@
         <v>4429</v>
       </c>
     </row>
+    <row r="373">
+      <c r="A373" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B373" s="5" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F373" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G373" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H373" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I373" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B374" s="5" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.1.jpg</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.1</t>
+        </is>
+      </c>
+      <c r="F374" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G374" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H374" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I374" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B375" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.2.jpg</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.2</t>
+        </is>
+      </c>
+      <c r="F375" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G375" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H375" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I375" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B376" s="5" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.3.jpg</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.3</t>
+        </is>
+      </c>
+      <c r="F376" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G376" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H376" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I376" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B377" s="5" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.4.jpg</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>version dall-e - 1.4</t>
+        </is>
+      </c>
+      <c r="F377" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G377" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H377" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I377" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B378" s="5" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F378" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G378" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H378" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I378" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B379" s="5" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.1.jpg</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.1</t>
+        </is>
+      </c>
+      <c r="F379" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G379" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H379" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I379" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B380" s="5" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.2.jpg</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.2</t>
+        </is>
+      </c>
+      <c r="F380" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G380" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H380" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I380" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B381" s="5" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.3.jpg</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.3</t>
+        </is>
+      </c>
+      <c r="F381" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G381" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H381" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I381" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B382" s="5" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.4.jpg</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>version dall-e - 2.4</t>
+        </is>
+      </c>
+      <c r="F382" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G382" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H382" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I382" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B383" s="5" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F383" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G383" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H383" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I383" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B384" s="5" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.1.jpg</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.1</t>
+        </is>
+      </c>
+      <c r="F384" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G384" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H384" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I384" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B385" s="5" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.2.jpg</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.2</t>
+        </is>
+      </c>
+      <c r="F385" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G385" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H385" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I385" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B386" s="5" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.3.jpg</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.3</t>
+        </is>
+      </c>
+      <c r="F386" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G386" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H386" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I386" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B387" s="5" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.4.jpg</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>version dall-e - 3.4</t>
+        </is>
+      </c>
+      <c r="F387" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G387" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H387" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I387" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B388" s="5" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F388" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G388" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H388" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I388" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B389" s="5" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.1.jpg</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.1</t>
+        </is>
+      </c>
+      <c r="F389" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G389" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H389" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I389" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B390" s="5" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.2.jpg</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.2</t>
+        </is>
+      </c>
+      <c r="F390" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G390" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H390" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I390" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B391" s="5" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.3.jpg</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.3</t>
+        </is>
+      </c>
+      <c r="F391" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G391" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H391" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I391" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B392" s="5" t="inlineStr">
+        <is>
+          <t>020</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.4.jpg</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>version dall-e - 4.4</t>
+        </is>
+      </c>
+      <c r="F392" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G392" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H392" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I392" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B393" s="5" t="inlineStr">
+        <is>
+          <t>021</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F393" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G393" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H393" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I393" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B394" s="5" t="inlineStr">
+        <is>
+          <t>022</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.1.jpg</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.1</t>
+        </is>
+      </c>
+      <c r="F394" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G394" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H394" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I394" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B395" s="5" t="inlineStr">
+        <is>
+          <t>023</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.2.jpg</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.2</t>
+        </is>
+      </c>
+      <c r="F395" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G395" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H395" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I395" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B396" s="5" t="inlineStr">
+        <is>
+          <t>024</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.3.jpg</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.3</t>
+        </is>
+      </c>
+      <c r="F396" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G396" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H396" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I396" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B397" s="5" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.4.jpg</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>version dall-e - 5.4</t>
+        </is>
+      </c>
+      <c r="F397" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G397" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H397" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I397" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B398" s="5" t="inlineStr">
+        <is>
+          <t>026</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F398" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G398" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H398" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I398" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B399" s="5" t="inlineStr">
+        <is>
+          <t>027</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.1.jpg</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.1</t>
+        </is>
+      </c>
+      <c r="F399" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G399" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H399" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I399" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B400" s="5" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.2.jpg</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.2</t>
+        </is>
+      </c>
+      <c r="F400" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G400" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H400" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I400" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B401" s="5" t="inlineStr">
+        <is>
+          <t>029</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.3.jpg</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.3</t>
+        </is>
+      </c>
+      <c r="F401" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G401" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H401" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I401" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B402" s="5" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.4.jpg</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>version dall-e - 6.4</t>
+        </is>
+      </c>
+      <c r="F402" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G402" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H402" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I402" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B403" s="5" t="inlineStr">
+        <is>
+          <t>031</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F403" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G403" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H403" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I403" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B404" s="5" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.1.jpg</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.1</t>
+        </is>
+      </c>
+      <c r="F404" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G404" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H404" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I404" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B405" s="5" t="inlineStr">
+        <is>
+          <t>033</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.2.jpg</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.2</t>
+        </is>
+      </c>
+      <c r="F405" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G405" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H405" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I405" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B406" s="5" t="inlineStr">
+        <is>
+          <t>034</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.3.jpg</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.3</t>
+        </is>
+      </c>
+      <c r="F406" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G406" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H406" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I406" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B407" s="5" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.4.jpg</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>version dall-e - 7.4</t>
+        </is>
+      </c>
+      <c r="F407" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G407" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H407" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I407" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B408" s="5" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F408" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G408" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H408" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I408" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B409" s="5" t="inlineStr">
+        <is>
+          <t>037</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.1.jpg</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.1</t>
+        </is>
+      </c>
+      <c r="F409" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G409" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H409" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I409" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B410" s="5" t="inlineStr">
+        <is>
+          <t>038</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.2.jpg</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.2</t>
+        </is>
+      </c>
+      <c r="F410" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G410" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H410" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I410" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B411" s="5" t="inlineStr">
+        <is>
+          <t>039</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.3.jpg</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.3</t>
+        </is>
+      </c>
+      <c r="F411" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G411" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H411" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I411" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B412" s="5" t="inlineStr">
+        <is>
+          <t>040</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.4.jpg</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>version dall-e - 8.4</t>
+        </is>
+      </c>
+      <c r="F412" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G412" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H412" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I412" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B413" s="5" t="inlineStr">
+        <is>
+          <t>041</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F413" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G413" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H413" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I413" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B414" s="5" t="inlineStr">
+        <is>
+          <t>042</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.1.jpg</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.1</t>
+        </is>
+      </c>
+      <c r="F414" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G414" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H414" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I414" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B415" s="5" t="inlineStr">
+        <is>
+          <t>043</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.2.jpg</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.2</t>
+        </is>
+      </c>
+      <c r="F415" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G415" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H415" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I415" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B416" s="5" t="inlineStr">
+        <is>
+          <t>044</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.3.jpg</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.3</t>
+        </is>
+      </c>
+      <c r="F416" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G416" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H416" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I416" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B417" s="5" t="inlineStr">
+        <is>
+          <t>045</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.4.jpg</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>version dall-e - 9.4</t>
+        </is>
+      </c>
+      <c r="F417" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G417" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H417" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I417" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B418" s="5" t="inlineStr">
+        <is>
+          <t>046</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F418" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G418" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H418" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I418" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B419" s="5" t="inlineStr">
+        <is>
+          <t>047</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.1.jpg</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.1</t>
+        </is>
+      </c>
+      <c r="F419" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G419" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H419" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I419" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B420" s="5" t="inlineStr">
+        <is>
+          <t>048</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.2.jpg</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.2</t>
+        </is>
+      </c>
+      <c r="F420" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G420" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H420" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I420" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B421" s="5" t="inlineStr">
+        <is>
+          <t>049</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.3.jpg</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.3</t>
+        </is>
+      </c>
+      <c r="F421" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G421" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H421" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I421" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B422" s="5" t="inlineStr">
+        <is>
+          <t>050</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.4.jpg</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>version dall-e - 10.4</t>
+        </is>
+      </c>
+      <c r="F422" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G422" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H422" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I422" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B423" s="5" t="inlineStr">
+        <is>
+          <t>051</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F423" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G423" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H423" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I423" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B424" s="5" t="inlineStr">
+        <is>
+          <t>052</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.1.jpg</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.1</t>
+        </is>
+      </c>
+      <c r="F424" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G424" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H424" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I424" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B425" s="5" t="inlineStr">
+        <is>
+          <t>053</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.2.jpg</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.2</t>
+        </is>
+      </c>
+      <c r="F425" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G425" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H425" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I425" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B426" s="5" t="inlineStr">
+        <is>
+          <t>054</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.3.jpg</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.3</t>
+        </is>
+      </c>
+      <c r="F426" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G426" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H426" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I426" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B427" s="5" t="inlineStr">
+        <is>
+          <t>055</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.4.jpg</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>version dall-e - 11.4</t>
+        </is>
+      </c>
+      <c r="F427" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G427" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H427" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I427" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B428" s="5" t="inlineStr">
+        <is>
+          <t>056</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F428" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G428" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H428" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I428" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B429" s="5" t="inlineStr">
+        <is>
+          <t>057</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.1.jpg</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.1</t>
+        </is>
+      </c>
+      <c r="F429" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G429" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H429" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I429" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B430" s="5" t="inlineStr">
+        <is>
+          <t>058</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.2.jpg</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.2</t>
+        </is>
+      </c>
+      <c r="F430" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G430" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H430" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I430" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B431" s="5" t="inlineStr">
+        <is>
+          <t>059</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.3.jpg</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.3</t>
+        </is>
+      </c>
+      <c r="F431" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G431" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H431" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I431" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B432" s="5" t="inlineStr">
+        <is>
+          <t>060</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.4.jpg</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>version dall-e - 12.4</t>
+        </is>
+      </c>
+      <c r="F432" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G432" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H432" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I432" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B433" s="5" t="inlineStr">
+        <is>
+          <t>061</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F433" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G433" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H433" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I433" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B434" s="5" t="inlineStr">
+        <is>
+          <t>062</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.1.jpg</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.1</t>
+        </is>
+      </c>
+      <c r="F434" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G434" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H434" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I434" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B435" s="5" t="inlineStr">
+        <is>
+          <t>063</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.2.jpg</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.2</t>
+        </is>
+      </c>
+      <c r="F435" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G435" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H435" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I435" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B436" s="5" t="inlineStr">
+        <is>
+          <t>064</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.3.jpg</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.3</t>
+        </is>
+      </c>
+      <c r="F436" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G436" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H436" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I436" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B437" s="5" t="inlineStr">
+        <is>
+          <t>065</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.4.jpg</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>version dall-e - 13.4</t>
+        </is>
+      </c>
+      <c r="F437" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G437" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H437" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I437" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B438" s="5" t="inlineStr">
+        <is>
+          <t>066</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F438" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G438" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H438" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I438" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B439" s="5" t="inlineStr">
+        <is>
+          <t>067</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.1.jpg</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.1</t>
+        </is>
+      </c>
+      <c r="F439" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G439" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H439" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I439" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B440" s="5" t="inlineStr">
+        <is>
+          <t>068</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.2.jpg</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.2</t>
+        </is>
+      </c>
+      <c r="F440" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G440" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H440" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I440" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B441" s="5" t="inlineStr">
+        <is>
+          <t>069</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.3.jpg</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.3</t>
+        </is>
+      </c>
+      <c r="F441" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G441" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H441" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I441" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B442" s="5" t="inlineStr">
+        <is>
+          <t>070</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.4.jpg</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>version dall-e - 14.4</t>
+        </is>
+      </c>
+      <c r="F442" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G442" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H442" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I442" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B443" s="5" t="inlineStr">
+        <is>
+          <t>071</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.0 (run source).jpg</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.0 (run source)</t>
+        </is>
+      </c>
+      <c r="F443" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G443" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H443" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I443" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B444" s="5" t="inlineStr">
+        <is>
+          <t>072</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.1.jpg</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.1</t>
+        </is>
+      </c>
+      <c r="F444" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G444" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H444" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I444" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B445" s="5" t="inlineStr">
+        <is>
+          <t>073</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.2.jpg</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.2</t>
+        </is>
+      </c>
+      <c r="F445" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G445" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H445" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I445" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B446" s="5" t="inlineStr">
+        <is>
+          <t>074</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.3.jpg</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.3</t>
+        </is>
+      </c>
+      <c r="F446" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G446" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H446" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I446" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="22" t="inlineStr">
+        <is>
+          <t>00519</t>
+        </is>
+      </c>
+      <c r="B447" s="5" t="inlineStr">
+        <is>
+          <t>075</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>versions</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.4.jpg</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>version dall-e - 15.4</t>
+        </is>
+      </c>
+      <c r="F447" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G447" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="H447" t="n">
+        <v>3543</v>
+      </c>
+      <c r="I447" t="n">
+        <v>3543</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28198,7 +32624,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19" outlineLevelCol="0"/>
   <cols>
     <col width="24.1640625" customWidth="1" style="19" min="1" max="1"/>
     <col width="34.83203125" customWidth="1" style="19" min="2" max="2"/>
@@ -28211,8 +32637,8 @@
     <col width="11.33203125" bestFit="1" customWidth="1" style="19" min="9" max="9"/>
     <col width="12.1640625" bestFit="1" customWidth="1" style="19" min="10" max="10"/>
     <col width="33.6640625" customWidth="1" style="19" min="11" max="11"/>
-    <col width="10.83203125" customWidth="1" style="19" min="12" max="21"/>
-    <col width="10.83203125" customWidth="1" style="19" min="22" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="19" min="12" max="24"/>
+    <col width="10.83203125" customWidth="1" style="19" min="25" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -30374,7 +34800,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G839"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
   <cols>
     <col width="41.6640625" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
     <col width="9.33203125" customWidth="1" style="10" min="2" max="2"/>
@@ -30384,8 +34810,8 @@
     <col width="20.1640625" bestFit="1" customWidth="1" style="10" min="6" max="6"/>
     <col width="48.1640625" bestFit="1" customWidth="1" style="10" min="7" max="7"/>
     <col width="21.83203125" customWidth="1" style="10" min="8" max="256"/>
-    <col width="21.83203125" customWidth="1" style="14" min="257" max="271"/>
-    <col width="21.83203125" customWidth="1" style="14" min="272" max="16384"/>
+    <col width="21.83203125" customWidth="1" style="14" min="257" max="274"/>
+    <col width="21.83203125" customWidth="1" style="14" min="275" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">

</xml_diff>

<commit_message>
leaf now replaced nerve as 00458
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -618,7 +618,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C54"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="21.83203125" customWidth="1" style="4" min="1" max="1"/>
     <col width="77.33203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1402,8 +1402,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y197"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <dimension ref="A1:Y250"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="11.33203125" customWidth="1" style="7" min="1" max="1"/>
     <col width="13.33203125" customWidth="1" style="7" min="2" max="2"/>
@@ -1429,8 +1429,8 @@
     <col width="21.5" customWidth="1" style="7" min="23" max="23"/>
     <col width="26.83203125" customWidth="1" style="7" min="24" max="24"/>
     <col width="20.83203125" customWidth="1" style="7" min="25" max="25"/>
-    <col width="10.83203125" customWidth="1" style="7" min="26" max="50"/>
-    <col width="10.83203125" customWidth="1" style="7" min="51" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="26" max="52"/>
+    <col width="10.83203125" customWidth="1" style="7" min="53" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="6">
@@ -9547,8 +9547,13 @@
           <t>00454</t>
         </is>
       </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
       <c r="C124" s="28" t="n">
-        <v>46066</v>
+        <v>46071</v>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
@@ -9808,55 +9813,48 @@
         </is>
       </c>
       <c r="C128" s="30" t="n">
-        <v>46068</v>
+        <v>46071</v>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>nerve</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>nerve.jpg</t>
+          <t>leaf.jpg</t>
         </is>
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>nerve</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="G128" s="7" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="H128" s="7" t="n">
-        <v>29.7</v>
+        <v>30</v>
       </c>
       <c r="I128" s="7" t="n">
-        <v>1995</v>
-      </c>
-      <c r="J128" s="7" t="inlineStr">
-        <is>
-          <t>July 1990 – January 1995</t>
-        </is>
+        <v>2016</v>
+      </c>
+      <c r="J128" s="7" t="n">
+        <v>2016</v>
       </c>
       <c r="K128" s="7" t="inlineStr">
         <is>
-          <t>nerve</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="L128" s="7" t="inlineStr">
         <is>
-          <t>writing</t>
+          <t>digital print</t>
         </is>
       </c>
       <c r="M128" s="7" t="inlineStr">
         <is>
-          <t>loose bound book, 48p</t>
-        </is>
-      </c>
-      <c r="R128" s="7" t="inlineStr">
-        <is>
-          <t>nerve.pdf</t>
+          <t>digital c-type print</t>
         </is>
       </c>
       <c r="X128" s="22" t="inlineStr">
@@ -13894,7 +13892,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C194" s="33" t="n">
+      <c r="C194" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="D194" s="7" t="inlineStr">
@@ -13956,7 +13954,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C195" s="33" t="n">
+      <c r="C195" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="D195" s="7" t="inlineStr">
@@ -14018,7 +14016,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C196" s="33" t="n">
+      <c r="C196" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="D196" s="7" t="inlineStr">
@@ -14080,7 +14078,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C197" s="33" t="n">
+      <c r="C197" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="D197" s="7" t="inlineStr">
@@ -14130,6 +14128,344 @@
           <t>box 1 (A4)</t>
         </is>
       </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="22" t="inlineStr">
+        <is>
+          <t>00005</t>
+        </is>
+      </c>
+      <c r="D198" s="7" t="inlineStr">
+        <is>
+          <t>collected 1989-1998</t>
+        </is>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>00005 untitled forms.jpg</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="inlineStr">
+        <is>
+          <t>untitled forms</t>
+        </is>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H198" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="I198" s="7" t="n">
+        <v>1998</v>
+      </c>
+      <c r="J198" s="7" t="inlineStr">
+        <is>
+          <t>c. 1989-98</t>
+        </is>
+      </c>
+      <c r="K198" s="7" t="inlineStr">
+        <is>
+          <t>collected-1989-1998</t>
+        </is>
+      </c>
+      <c r="L198" s="7" t="inlineStr">
+        <is>
+          <t>painting</t>
+        </is>
+      </c>
+      <c r="M198" s="7" t="inlineStr">
+        <is>
+          <t>mixed meda</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="22" t="inlineStr">
+        <is>
+          <t>00006</t>
+        </is>
+      </c>
+      <c r="E199" s="7" t="inlineStr">
+        <is>
+          <t>00006 gesture in grey.jpg</t>
+        </is>
+      </c>
+      <c r="F199" s="7" t="inlineStr">
+        <is>
+          <t>gesture in grey</t>
+        </is>
+      </c>
+      <c r="G199" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="H199" s="7" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="I199" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J199" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="L199" s="7" t="inlineStr">
+        <is>
+          <t>painting</t>
+        </is>
+      </c>
+      <c r="M199" s="7" t="inlineStr">
+        <is>
+          <t>acrylic on paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="22" t="inlineStr">
+        <is>
+          <t>00007</t>
+        </is>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>00007 skeletal.jpg</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="inlineStr">
+        <is>
+          <t>skeletal</t>
+        </is>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="H200" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I200" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J200" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="L200" s="7" t="inlineStr">
+        <is>
+          <t>painting</t>
+        </is>
+      </c>
+      <c r="M200" s="7" t="inlineStr">
+        <is>
+          <t>acrylic on paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="22" t="inlineStr">
+        <is>
+          <t>00008</t>
+        </is>
+      </c>
+      <c r="C201" s="30" t="n"/>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t>nerve</t>
+        </is>
+      </c>
+      <c r="E201" s="7" t="inlineStr">
+        <is>
+          <t>nerve.jpg</t>
+        </is>
+      </c>
+      <c r="F201" s="7" t="inlineStr">
+        <is>
+          <t>nerve</t>
+        </is>
+      </c>
+      <c r="G201" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="H201" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I201" s="7" t="n">
+        <v>1995</v>
+      </c>
+      <c r="J201" s="7" t="inlineStr">
+        <is>
+          <t>July 1990 – January 1995</t>
+        </is>
+      </c>
+      <c r="K201" s="7" t="inlineStr">
+        <is>
+          <t>nerve</t>
+        </is>
+      </c>
+      <c r="L201" s="7" t="inlineStr">
+        <is>
+          <t>writing</t>
+        </is>
+      </c>
+      <c r="M201" s="7" t="inlineStr">
+        <is>
+          <t>loose bound book, 48p</t>
+        </is>
+      </c>
+      <c r="R201" s="7" t="inlineStr">
+        <is>
+          <t>nerve.pdf</t>
+        </is>
+      </c>
+      <c r="X201" s="22" t="inlineStr">
+        <is>
+          <t>Michael Davies</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="22" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="22" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="22" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="22" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="22" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="22" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="22" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="22" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="22" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="22" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="22" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="22" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="22" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="22" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="22" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="22" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="22" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="22" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="22" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="22" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="22" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="22" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="22" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="22" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="22" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="22" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="22" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="22" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="22" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="22" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="22" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="22" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="22" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="22" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="22" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="22" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="22" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="22" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="22" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="22" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="22" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="22" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="22" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="22" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="22" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="22" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="22" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="22" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="22" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14143,8 +14479,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="31.83203125" customWidth="1" style="1" min="1" max="1"/>
     <col width="43.1640625" customWidth="1" style="1" min="2" max="2"/>
@@ -14155,8 +14491,8 @@
     <col width="21" customWidth="1" style="7" min="7" max="7"/>
     <col width="28.1640625" customWidth="1" style="7" min="8" max="8"/>
     <col width="51" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
-    <col width="10.83203125" customWidth="1" style="1" min="10" max="35"/>
-    <col width="10.83203125" customWidth="1" style="1" min="36" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="1" min="10" max="37"/>
+    <col width="10.83203125" customWidth="1" style="1" min="38" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="3">
@@ -14776,7 +15112,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="D17" s="33" t="n">
+      <c r="D17" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="E17" s="1" t="n">
@@ -14798,6 +15134,67 @@
       <c r="I17" s="1" t="inlineStr">
         <is>
           <t>details attached to 00001</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>collected-1989-1998</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>collected 1989-1998</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>1998</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>c. 1989-98</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>collected</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="D19" s="33" t="n">
+        <v>46071</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>leaf,nature</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>add details</t>
         </is>
       </c>
     </row>
@@ -14813,7 +15210,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J480"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="9.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="9.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -33856,7 +34253,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G464" s="33" t="n">
+      <c r="G464" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H464" t="n">
@@ -33897,7 +34294,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G465" s="33" t="n">
+      <c r="G465" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H465" t="n">
@@ -33938,7 +34335,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G466" s="33" t="n">
+      <c r="G466" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H466" t="n">
@@ -33979,7 +34376,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G467" s="33" t="n">
+      <c r="G467" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H467" t="n">
@@ -34020,7 +34417,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G468" s="33" t="n">
+      <c r="G468" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H468" t="n">
@@ -34061,7 +34458,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G469" s="33" t="n">
+      <c r="G469" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H469" t="n">
@@ -34102,7 +34499,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G470" s="33" t="n">
+      <c r="G470" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H470" t="n">
@@ -34143,7 +34540,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G471" s="33" t="n">
+      <c r="G471" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H471" t="n">
@@ -34184,7 +34581,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G472" s="33" t="n">
+      <c r="G472" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H472" t="n">
@@ -34225,7 +34622,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G473" s="33" t="n">
+      <c r="G473" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H473" t="n">
@@ -34266,7 +34663,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G474" s="33" t="n">
+      <c r="G474" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H474" t="n">
@@ -34307,7 +34704,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G475" s="33" t="n">
+      <c r="G475" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H475" t="n">
@@ -34348,7 +34745,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G476" s="33" t="n">
+      <c r="G476" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H476" t="n">
@@ -34389,7 +34786,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G477" s="33" t="n">
+      <c r="G477" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H477" t="n">
@@ -34430,7 +34827,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G478" s="33" t="n">
+      <c r="G478" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H478" t="n">
@@ -34471,7 +34868,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G479" s="33" t="n">
+      <c r="G479" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H479" t="n">
@@ -34512,7 +34909,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G480" s="33" t="n">
+      <c r="G480" s="16" t="n">
         <v>46071</v>
       </c>
       <c r="H480" t="n">
@@ -34534,7 +34931,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="19" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
   <cols>
     <col width="24.1640625" customWidth="1" style="19" min="1" max="1"/>
     <col width="34.83203125" customWidth="1" style="19" min="2" max="2"/>
@@ -34547,8 +34944,8 @@
     <col width="11.33203125" bestFit="1" customWidth="1" style="19" min="9" max="9"/>
     <col width="12.1640625" bestFit="1" customWidth="1" style="19" min="10" max="10"/>
     <col width="33.6640625" customWidth="1" style="19" min="11" max="11"/>
-    <col width="10.83203125" customWidth="1" style="19" min="12" max="28"/>
-    <col width="10.83203125" customWidth="1" style="19" min="29" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="19" min="12" max="30"/>
+    <col width="10.83203125" customWidth="1" style="19" min="31" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -36710,7 +37107,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G839"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="41.6640625" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
     <col width="9.33203125" customWidth="1" style="10" min="2" max="2"/>
@@ -36720,8 +37117,8 @@
     <col width="20.1640625" bestFit="1" customWidth="1" style="10" min="6" max="6"/>
     <col width="48.1640625" bestFit="1" customWidth="1" style="10" min="7" max="7"/>
     <col width="21.83203125" customWidth="1" style="10" min="8" max="256"/>
-    <col width="21.83203125" customWidth="1" style="14" min="257" max="278"/>
-    <col width="21.83203125" customWidth="1" style="14" min="279" max="16384"/>
+    <col width="21.83203125" customWidth="1" style="14" min="257" max="280"/>
+    <col width="21.83203125" customWidth="1" style="14" min="281" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">

</xml_diff>

<commit_message>
republished series pages and json following series_sort= work_id change
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -618,7 +618,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C54"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="21.83203125" customWidth="1" style="4" min="1" max="1"/>
     <col width="77.33203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1403,7 +1403,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Y306"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="11.33203125" customWidth="1" style="7" min="1" max="1"/>
     <col width="13.33203125" customWidth="1" style="7" min="2" max="2"/>
@@ -21112,7 +21112,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="31.83203125" customWidth="1" style="1" min="1" max="1"/>
     <col width="43.1640625" customWidth="1" style="1" min="2" max="2"/>
@@ -21191,7 +21191,7 @@
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>46067</v>
+        <v>46072</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>2025</v>
@@ -21234,7 +21234,7 @@
         </is>
       </c>
       <c r="D3" s="15" t="n">
-        <v>46067</v>
+        <v>46072</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>2025</v>
@@ -21277,7 +21277,7 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>46067</v>
+        <v>46072</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>2021</v>
@@ -21313,7 +21313,7 @@
         </is>
       </c>
       <c r="D5" s="15" t="n">
-        <v>46067</v>
+        <v>46072</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>2010</v>
@@ -21349,7 +21349,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>46067</v>
+        <v>46072</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>2020</v>
@@ -21387,7 +21387,7 @@
         </is>
       </c>
       <c r="D7" s="16" t="n">
-        <v>46068</v>
+        <v>46072</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1995</v>
@@ -21425,7 +21425,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>46069</v>
+        <v>46072</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>2013</v>
@@ -21461,7 +21461,7 @@
         </is>
       </c>
       <c r="D9" s="15" t="n">
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>2004</v>
@@ -21494,7 +21494,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>2023</v>
@@ -21525,7 +21525,7 @@
         </is>
       </c>
       <c r="D11" s="16" t="n">
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>2023</v>
@@ -21561,7 +21561,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>2011</v>
@@ -21592,7 +21592,7 @@
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>2009</v>
@@ -21635,7 +21635,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>2023</v>
@@ -21671,7 +21671,7 @@
         </is>
       </c>
       <c r="D15" s="16" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>2010</v>
@@ -21709,7 +21709,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>2023</v>
@@ -21745,7 +21745,7 @@
         </is>
       </c>
       <c r="D17" s="16" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>2025</v>
@@ -21786,7 +21786,7 @@
         </is>
       </c>
       <c r="D18" s="33" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>1998</v>
@@ -21824,7 +21824,7 @@
         </is>
       </c>
       <c r="D19" s="16" t="n">
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>2016</v>
@@ -21855,7 +21855,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J480"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="9.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="9.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -41576,7 +41576,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="19" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
   <cols>
     <col width="24.1640625" customWidth="1" style="19" min="1" max="1"/>
     <col width="34.83203125" customWidth="1" style="19" min="2" max="2"/>
@@ -43752,7 +43752,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G839"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="41.6640625" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
     <col width="9.33203125" customWidth="1" style="10" min="2" max="2"/>

</xml_diff>

<commit_message>
published new collected work
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -17,19 +17,18 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'index - old version'!$A$1:$G$803</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;yes&quot;\,&quot;yes&quot;\,&quot;yes&quot;\,&quot;yes&quot;"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -110,12 +109,6 @@
       <color rgb="FF000000"/>
       <sz val="13"/>
     </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -147,7 +140,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -217,7 +210,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,7 +611,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C54"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="21.83203125" customWidth="1" style="4" min="1" max="1"/>
     <col width="77.33203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1403,8 +1395,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y403"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <dimension ref="A1:Y406"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="11.33203125" customWidth="1" style="7" min="1" max="1"/>
     <col width="13.33203125" customWidth="1" style="7" min="2" max="2"/>
@@ -1430,8 +1422,8 @@
     <col width="21.5" customWidth="1" style="7" min="23" max="23"/>
     <col width="26.83203125" customWidth="1" style="7" min="24" max="24"/>
     <col width="20.83203125" customWidth="1" style="7" min="25" max="25"/>
-    <col width="10.83203125" customWidth="1" style="7" min="26" max="56"/>
-    <col width="10.83203125" customWidth="1" style="7" min="57" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="26" max="58"/>
+    <col width="10.83203125" customWidth="1" style="7" min="59" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="6">
@@ -21189,7 +21181,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C307" s="33" t="n">
+      <c r="C307" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D307" s="7" t="inlineStr">
@@ -21251,7 +21243,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C308" s="33" t="n">
+      <c r="C308" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D308" s="7" t="inlineStr">
@@ -21315,7 +21307,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C309" s="33" t="n">
+      <c r="C309" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D309" s="7" t="inlineStr">
@@ -21377,7 +21369,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C310" s="33" t="n">
+      <c r="C310" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D310" s="7" t="inlineStr">
@@ -21439,7 +21431,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C311" s="33" t="n">
+      <c r="C311" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D311" s="7" t="inlineStr">
@@ -21501,7 +21493,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C312" s="33" t="n">
+      <c r="C312" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D312" s="7" t="inlineStr">
@@ -21563,7 +21555,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C313" s="33" t="n">
+      <c r="C313" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D313" s="7" t="inlineStr">
@@ -21625,7 +21617,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C314" s="33" t="n">
+      <c r="C314" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D314" s="7" t="inlineStr">
@@ -21687,7 +21679,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C315" s="33" t="n">
+      <c r="C315" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D315" s="7" t="inlineStr">
@@ -21749,7 +21741,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C316" s="33" t="n">
+      <c r="C316" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D316" s="7" t="inlineStr">
@@ -21811,7 +21803,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C317" s="33" t="n">
+      <c r="C317" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D317" s="7" t="inlineStr">
@@ -21873,7 +21865,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C318" s="33" t="n">
+      <c r="C318" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D318" s="7" t="inlineStr">
@@ -21935,7 +21927,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C319" s="33" t="n">
+      <c r="C319" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D319" s="7" t="inlineStr">
@@ -21997,7 +21989,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C320" s="33" t="n">
+      <c r="C320" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D320" s="7" t="inlineStr">
@@ -22059,7 +22051,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C321" s="33" t="n">
+      <c r="C321" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D321" s="7" t="inlineStr">
@@ -22121,7 +22113,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C322" s="33" t="n">
+      <c r="C322" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D322" s="7" t="inlineStr">
@@ -22183,7 +22175,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C323" s="33" t="n">
+      <c r="C323" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D323" s="7" t="inlineStr">
@@ -22245,7 +22237,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C324" s="33" t="n">
+      <c r="C324" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D324" s="7" t="inlineStr">
@@ -22307,7 +22299,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C325" s="33" t="n">
+      <c r="C325" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D325" s="7" t="inlineStr">
@@ -22369,7 +22361,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C326" s="33" t="n">
+      <c r="C326" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D326" s="7" t="inlineStr">
@@ -22431,7 +22423,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C327" s="33" t="n">
+      <c r="C327" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D327" s="7" t="inlineStr">
@@ -22493,7 +22485,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C328" s="33" t="n">
+      <c r="C328" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D328" s="7" t="inlineStr">
@@ -22555,7 +22547,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C329" s="33" t="n">
+      <c r="C329" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D329" s="7" t="inlineStr">
@@ -22617,7 +22609,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C330" s="33" t="n">
+      <c r="C330" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D330" s="7" t="inlineStr">
@@ -22679,7 +22671,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C331" s="33" t="n">
+      <c r="C331" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D331" s="7" t="inlineStr">
@@ -22741,7 +22733,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C332" s="33" t="n">
+      <c r="C332" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D332" s="7" t="inlineStr">
@@ -22803,7 +22795,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C333" s="33" t="n">
+      <c r="C333" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D333" s="7" t="inlineStr">
@@ -22865,7 +22857,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C334" s="33" t="n">
+      <c r="C334" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D334" s="7" t="inlineStr">
@@ -22927,7 +22919,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C335" s="33" t="n">
+      <c r="C335" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D335" s="7" t="inlineStr">
@@ -22989,7 +22981,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C336" s="33" t="n">
+      <c r="C336" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D336" s="7" t="inlineStr">
@@ -23051,7 +23043,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C337" s="33" t="n">
+      <c r="C337" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D337" s="7" t="inlineStr">
@@ -23115,7 +23107,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C338" s="33" t="n">
+      <c r="C338" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D338" s="7" t="inlineStr">
@@ -23182,7 +23174,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C339" s="33" t="n">
+      <c r="C339" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D339" s="7" t="inlineStr">
@@ -23249,7 +23241,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C340" s="33" t="n">
+      <c r="C340" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D340" s="7" t="inlineStr">
@@ -23313,7 +23305,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C341" s="33" t="n">
+      <c r="C341" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D341" s="7" t="inlineStr">
@@ -23382,7 +23374,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C342" s="33" t="n">
+      <c r="C342" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D342" s="7" t="inlineStr">
@@ -23444,7 +23436,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C343" s="33" t="n">
+      <c r="C343" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D343" s="7" t="inlineStr">
@@ -23508,7 +23500,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C344" s="33" t="n">
+      <c r="C344" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D344" s="7" t="inlineStr">
@@ -23570,7 +23562,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C345" s="33" t="n">
+      <c r="C345" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D345" s="7" t="inlineStr">
@@ -23632,7 +23624,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C346" s="33" t="n">
+      <c r="C346" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D346" s="7" t="inlineStr">
@@ -23694,7 +23686,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C347" s="33" t="n">
+      <c r="C347" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D347" s="7" t="inlineStr">
@@ -23756,7 +23748,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C348" s="33" t="n">
+      <c r="C348" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D348" s="7" t="inlineStr">
@@ -23818,7 +23810,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C349" s="33" t="n">
+      <c r="C349" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D349" s="7" t="inlineStr">
@@ -23880,7 +23872,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C350" s="33" t="n">
+      <c r="C350" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D350" s="7" t="inlineStr">
@@ -23944,7 +23936,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C351" s="33" t="n">
+      <c r="C351" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D351" s="7" t="inlineStr">
@@ -24008,7 +24000,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C352" s="33" t="n">
+      <c r="C352" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D352" s="7" t="inlineStr">
@@ -24072,7 +24064,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C353" s="33" t="n">
+      <c r="C353" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D353" s="7" t="inlineStr">
@@ -24136,7 +24128,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C354" s="33" t="n">
+      <c r="C354" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D354" s="7" t="inlineStr">
@@ -24200,7 +24192,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C355" s="33" t="n">
+      <c r="C355" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D355" s="7" t="inlineStr">
@@ -24264,7 +24256,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C356" s="33" t="n">
+      <c r="C356" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D356" s="7" t="inlineStr">
@@ -24328,7 +24320,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C357" s="33" t="n">
+      <c r="C357" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D357" s="7" t="inlineStr">
@@ -24392,7 +24384,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C358" s="33" t="n">
+      <c r="C358" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D358" s="7" t="inlineStr">
@@ -24456,7 +24448,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C359" s="33" t="n">
+      <c r="C359" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D359" s="7" t="inlineStr">
@@ -24520,7 +24512,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C360" s="33" t="n">
+      <c r="C360" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D360" s="7" t="inlineStr">
@@ -24584,7 +24576,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C361" s="33" t="n">
+      <c r="C361" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D361" s="7" t="inlineStr">
@@ -24648,7 +24640,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C362" s="33" t="n">
+      <c r="C362" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D362" s="7" t="inlineStr">
@@ -24712,7 +24704,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C363" s="33" t="n">
+      <c r="C363" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D363" s="7" t="inlineStr">
@@ -24776,7 +24768,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C364" s="33" t="n">
+      <c r="C364" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D364" s="7" t="inlineStr">
@@ -24840,7 +24832,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C365" s="33" t="n">
+      <c r="C365" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D365" s="7" t="inlineStr">
@@ -24904,7 +24896,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C366" s="33" t="n">
+      <c r="C366" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D366" s="7" t="inlineStr">
@@ -24968,7 +24960,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C367" s="33" t="n">
+      <c r="C367" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D367" s="7" t="inlineStr">
@@ -25032,7 +25024,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C368" s="33" t="n">
+      <c r="C368" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D368" s="7" t="inlineStr">
@@ -25096,7 +25088,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C369" s="33" t="n">
+      <c r="C369" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D369" s="7" t="inlineStr">
@@ -25158,7 +25150,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C370" s="33" t="n">
+      <c r="C370" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D370" s="7" t="inlineStr">
@@ -25220,7 +25212,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C371" s="33" t="n">
+      <c r="C371" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D371" s="7" t="inlineStr">
@@ -25282,7 +25274,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C372" s="33" t="n">
+      <c r="C372" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D372" s="7" t="inlineStr">
@@ -25344,7 +25336,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C373" s="33" t="n">
+      <c r="C373" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D373" s="7" t="inlineStr">
@@ -25406,7 +25398,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C374" s="33" t="n">
+      <c r="C374" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D374" s="7" t="inlineStr">
@@ -25468,7 +25460,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C375" s="33" t="n">
+      <c r="C375" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D375" s="7" t="inlineStr">
@@ -25530,7 +25522,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C376" s="33" t="n">
+      <c r="C376" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D376" s="7" t="inlineStr">
@@ -25592,7 +25584,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C377" s="33" t="n">
+      <c r="C377" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D377" s="7" t="inlineStr">
@@ -25654,7 +25646,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C378" s="33" t="n">
+      <c r="C378" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D378" s="7" t="inlineStr">
@@ -25716,7 +25708,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C379" s="33" t="n">
+      <c r="C379" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D379" s="7" t="inlineStr">
@@ -25778,7 +25770,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C380" s="33" t="n">
+      <c r="C380" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D380" s="7" t="inlineStr">
@@ -25840,7 +25832,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C381" s="33" t="n">
+      <c r="C381" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D381" s="7" t="inlineStr">
@@ -25902,7 +25894,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C382" s="33" t="n">
+      <c r="C382" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D382" s="7" t="inlineStr">
@@ -25964,7 +25956,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C383" s="33" t="n">
+      <c r="C383" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D383" s="7" t="inlineStr">
@@ -26026,7 +26018,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C384" s="33" t="n">
+      <c r="C384" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D384" s="7" t="inlineStr">
@@ -26088,7 +26080,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C385" s="33" t="n">
+      <c r="C385" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D385" s="7" t="inlineStr">
@@ -26150,7 +26142,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C386" s="33" t="n">
+      <c r="C386" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D386" s="7" t="inlineStr">
@@ -26212,7 +26204,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C387" s="33" t="n">
+      <c r="C387" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D387" s="7" t="inlineStr">
@@ -26276,7 +26268,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C388" s="33" t="n">
+      <c r="C388" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D388" s="7" t="inlineStr">
@@ -26340,7 +26332,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C389" s="33" t="n">
+      <c r="C389" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D389" s="7" t="inlineStr">
@@ -26404,7 +26396,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C390" s="33" t="n">
+      <c r="C390" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D390" s="7" t="inlineStr">
@@ -26468,7 +26460,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C391" s="33" t="n">
+      <c r="C391" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D391" s="7" t="inlineStr">
@@ -26532,7 +26524,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C392" s="33" t="n">
+      <c r="C392" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D392" s="7" t="inlineStr">
@@ -26596,7 +26588,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C393" s="33" t="n">
+      <c r="C393" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D393" s="7" t="inlineStr">
@@ -26660,7 +26652,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C394" s="33" t="n">
+      <c r="C394" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D394" s="7" t="inlineStr">
@@ -26722,7 +26714,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C395" s="33" t="n">
+      <c r="C395" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D395" s="7" t="inlineStr">
@@ -26784,7 +26776,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C396" s="33" t="n">
+      <c r="C396" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D396" s="7" t="inlineStr">
@@ -26846,7 +26838,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C397" s="33" t="n">
+      <c r="C397" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D397" s="7" t="inlineStr">
@@ -26908,7 +26900,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C398" s="33" t="n">
+      <c r="C398" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D398" s="7" t="inlineStr">
@@ -26970,7 +26962,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C399" s="33" t="n">
+      <c r="C399" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D399" s="7" t="inlineStr">
@@ -27032,7 +27024,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C400" s="33" t="n">
+      <c r="C400" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D400" s="7" t="inlineStr">
@@ -27094,7 +27086,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C401" s="33" t="n">
+      <c r="C401" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D401" s="7" t="inlineStr">
@@ -27156,7 +27148,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C402" s="33" t="n">
+      <c r="C402" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D402" s="7" t="inlineStr">
@@ -27218,7 +27210,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="C403" s="33" t="n">
+      <c r="C403" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="D403" s="7" t="inlineStr">
@@ -27264,6 +27256,198 @@
         </is>
       </c>
       <c r="S403" s="7" t="inlineStr">
+        <is>
+          <t>box 1 (A4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="22" t="inlineStr">
+        <is>
+          <t>00233</t>
+        </is>
+      </c>
+      <c r="B404" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C404" s="16" t="n">
+        <v>46074</v>
+      </c>
+      <c r="D404" s="7" t="inlineStr">
+        <is>
+          <t>collected 1989-1998</t>
+        </is>
+      </c>
+      <c r="E404" s="7" t="inlineStr">
+        <is>
+          <t>untitled [0233].jpg</t>
+        </is>
+      </c>
+      <c r="F404" s="7" t="inlineStr">
+        <is>
+          <t>untitled [0233]</t>
+        </is>
+      </c>
+      <c r="G404" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="H404" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I404" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J404" s="7" t="inlineStr">
+        <is>
+          <t>c. 1989-98</t>
+        </is>
+      </c>
+      <c r="K404" s="7" t="inlineStr">
+        <is>
+          <t>collected-1989-1998</t>
+        </is>
+      </c>
+      <c r="L404" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M404" s="7" t="inlineStr">
+        <is>
+          <t>pen on paper</t>
+        </is>
+      </c>
+      <c r="S404" s="7" t="inlineStr">
+        <is>
+          <t>box 1 (A4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="22" t="inlineStr">
+        <is>
+          <t>00234</t>
+        </is>
+      </c>
+      <c r="B405" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C405" s="16" t="n">
+        <v>46074</v>
+      </c>
+      <c r="D405" s="7" t="inlineStr">
+        <is>
+          <t>collected 1989-1998</t>
+        </is>
+      </c>
+      <c r="E405" s="7" t="inlineStr">
+        <is>
+          <t>untitled [0234].jpg</t>
+        </is>
+      </c>
+      <c r="F405" s="7" t="inlineStr">
+        <is>
+          <t>untitled [0234]</t>
+        </is>
+      </c>
+      <c r="G405" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="H405" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I405" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J405" s="7" t="inlineStr">
+        <is>
+          <t>c. 1989-98</t>
+        </is>
+      </c>
+      <c r="K405" s="7" t="inlineStr">
+        <is>
+          <t>collected-1989-1998</t>
+        </is>
+      </c>
+      <c r="L405" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M405" s="7" t="inlineStr">
+        <is>
+          <t>pen on paper</t>
+        </is>
+      </c>
+      <c r="S405" s="7" t="inlineStr">
+        <is>
+          <t>box 1 (A4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="22" t="inlineStr">
+        <is>
+          <t>00247</t>
+        </is>
+      </c>
+      <c r="B406" s="7" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="C406" s="16" t="n">
+        <v>46074</v>
+      </c>
+      <c r="D406" s="7" t="inlineStr">
+        <is>
+          <t>collected 1989-1998</t>
+        </is>
+      </c>
+      <c r="E406" s="7" t="inlineStr">
+        <is>
+          <t>untitled [0247].jpg</t>
+        </is>
+      </c>
+      <c r="F406" s="7" t="inlineStr">
+        <is>
+          <t>untitled [0247]</t>
+        </is>
+      </c>
+      <c r="G406" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="H406" s="7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="I406" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J406" s="7" t="inlineStr">
+        <is>
+          <t>c. 1989-98</t>
+        </is>
+      </c>
+      <c r="K406" s="7" t="inlineStr">
+        <is>
+          <t>collected-1989-1998</t>
+        </is>
+      </c>
+      <c r="L406" s="7" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+      <c r="M406" s="7" t="inlineStr">
+        <is>
+          <t>pen on paper</t>
+        </is>
+      </c>
+      <c r="S406" s="7" t="inlineStr">
         <is>
           <t>box 1 (A4)</t>
         </is>
@@ -27282,7 +27466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="31.83203125" customWidth="1" style="1" min="1" max="1"/>
     <col width="43.1640625" customWidth="1" style="1" min="2" max="2"/>
@@ -27293,8 +27477,8 @@
     <col width="21" customWidth="1" style="7" min="7" max="7"/>
     <col width="28.1640625" customWidth="1" style="7" min="8" max="8"/>
     <col width="51" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
-    <col width="10.83203125" customWidth="1" style="1" min="10" max="41"/>
-    <col width="10.83203125" customWidth="1" style="1" min="42" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="1" min="10" max="43"/>
+    <col width="10.83203125" customWidth="1" style="1" min="44" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="3">
@@ -28029,7 +28213,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="D20" s="33" t="n">
+      <c r="D20" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="E20" s="1" t="n">
@@ -28065,7 +28249,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="D21" s="33" t="n">
+      <c r="D21" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="E21" s="1" t="n">
@@ -28096,7 +28280,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="D22" s="33" t="n">
+      <c r="D22" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="E22" s="1" t="n">
@@ -28134,7 +28318,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="D23" s="33" t="n">
+      <c r="D23" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="E23" s="1" t="n">
@@ -28166,7 +28350,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J530"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="9.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="9.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -47906,7 +48090,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G481" s="33" t="n">
+      <c r="G481" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H481" t="n">
@@ -47947,7 +48131,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G482" s="33" t="n">
+      <c r="G482" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H482" t="n">
@@ -47988,7 +48172,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G483" s="33" t="n">
+      <c r="G483" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H483" t="n">
@@ -48029,7 +48213,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G484" s="33" t="n">
+      <c r="G484" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H484" t="n">
@@ -48070,7 +48254,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G485" s="33" t="n">
+      <c r="G485" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H485" t="n">
@@ -48111,7 +48295,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G486" s="33" t="n">
+      <c r="G486" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H486" t="n">
@@ -48152,7 +48336,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G487" s="33" t="n">
+      <c r="G487" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H487" t="n">
@@ -48193,7 +48377,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G488" s="33" t="n">
+      <c r="G488" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H488" t="n">
@@ -48234,7 +48418,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G489" s="33" t="n">
+      <c r="G489" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H489" t="n">
@@ -48275,7 +48459,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G490" s="33" t="n">
+      <c r="G490" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H490" t="n">
@@ -48316,7 +48500,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G491" s="33" t="n">
+      <c r="G491" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H491" t="n">
@@ -48357,7 +48541,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G492" s="33" t="n">
+      <c r="G492" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H492" t="n">
@@ -48398,7 +48582,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G493" s="33" t="n">
+      <c r="G493" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H493" t="n">
@@ -48439,7 +48623,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G494" s="33" t="n">
+      <c r="G494" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H494" t="n">
@@ -48480,7 +48664,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G495" s="33" t="n">
+      <c r="G495" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H495" t="n">
@@ -48521,7 +48705,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G496" s="33" t="n">
+      <c r="G496" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H496" t="n">
@@ -48562,7 +48746,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G497" s="33" t="n">
+      <c r="G497" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H497" t="n">
@@ -48603,7 +48787,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G498" s="33" t="n">
+      <c r="G498" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H498" t="n">
@@ -48644,7 +48828,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G499" s="33" t="n">
+      <c r="G499" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H499" t="n">
@@ -48685,7 +48869,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G500" s="33" t="n">
+      <c r="G500" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H500" t="n">
@@ -48726,7 +48910,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G501" s="33" t="n">
+      <c r="G501" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H501" t="n">
@@ -48767,7 +48951,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G502" s="33" t="n">
+      <c r="G502" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H502" t="n">
@@ -48808,7 +48992,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G503" s="33" t="n">
+      <c r="G503" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H503" t="n">
@@ -48849,7 +49033,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G504" s="33" t="n">
+      <c r="G504" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H504" t="n">
@@ -48890,7 +49074,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G505" s="33" t="n">
+      <c r="G505" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H505" t="n">
@@ -48931,7 +49115,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G506" s="33" t="n">
+      <c r="G506" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H506" t="n">
@@ -48972,7 +49156,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G507" s="33" t="n">
+      <c r="G507" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H507" t="n">
@@ -49013,7 +49197,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G508" s="33" t="n">
+      <c r="G508" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H508" t="n">
@@ -49054,7 +49238,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G509" s="33" t="n">
+      <c r="G509" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H509" t="n">
@@ -49095,7 +49279,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G510" s="33" t="n">
+      <c r="G510" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H510" t="n">
@@ -49136,7 +49320,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G511" s="33" t="n">
+      <c r="G511" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H511" t="n">
@@ -49177,7 +49361,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G512" s="33" t="n">
+      <c r="G512" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H512" t="n">
@@ -49218,7 +49402,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G513" s="33" t="n">
+      <c r="G513" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H513" t="n">
@@ -49259,7 +49443,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G514" s="33" t="n">
+      <c r="G514" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H514" t="n">
@@ -49300,7 +49484,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G515" s="33" t="n">
+      <c r="G515" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H515" t="n">
@@ -49341,7 +49525,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G516" s="33" t="n">
+      <c r="G516" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H516" t="n">
@@ -49382,7 +49566,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G517" s="33" t="n">
+      <c r="G517" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H517" t="n">
@@ -49423,7 +49607,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G518" s="33" t="n">
+      <c r="G518" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H518" t="n">
@@ -49464,7 +49648,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G519" s="33" t="n">
+      <c r="G519" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H519" t="n">
@@ -49505,7 +49689,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G520" s="33" t="n">
+      <c r="G520" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H520" t="n">
@@ -49546,7 +49730,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G521" s="33" t="n">
+      <c r="G521" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H521" t="n">
@@ -49587,7 +49771,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G522" s="33" t="n">
+      <c r="G522" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H522" t="n">
@@ -49628,7 +49812,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G523" s="33" t="n">
+      <c r="G523" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H523" t="n">
@@ -49669,7 +49853,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G524" s="33" t="n">
+      <c r="G524" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H524" t="n">
@@ -49710,7 +49894,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G525" s="33" t="n">
+      <c r="G525" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H525" t="n">
@@ -49751,7 +49935,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G526" s="33" t="n">
+      <c r="G526" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H526" t="n">
@@ -49792,7 +49976,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G527" s="33" t="n">
+      <c r="G527" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H527" t="n">
@@ -49833,7 +50017,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G528" s="33" t="n">
+      <c r="G528" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H528" t="n">
@@ -49874,7 +50058,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G529" s="33" t="n">
+      <c r="G529" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H529" t="n">
@@ -49915,7 +50099,7 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G530" s="33" t="n">
+      <c r="G530" s="16" t="n">
         <v>46074</v>
       </c>
       <c r="H530" t="n">
@@ -49937,7 +50121,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="19" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
   <cols>
     <col width="24.1640625" customWidth="1" style="19" min="1" max="1"/>
     <col width="34.83203125" customWidth="1" style="19" min="2" max="2"/>
@@ -49950,8 +50134,8 @@
     <col width="11.33203125" bestFit="1" customWidth="1" style="19" min="9" max="9"/>
     <col width="12.1640625" bestFit="1" customWidth="1" style="19" min="10" max="10"/>
     <col width="33.6640625" customWidth="1" style="19" min="11" max="11"/>
-    <col width="10.83203125" customWidth="1" style="19" min="12" max="34"/>
-    <col width="10.83203125" customWidth="1" style="19" min="35" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="19" min="12" max="36"/>
+    <col width="10.83203125" customWidth="1" style="19" min="37" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -52113,7 +52297,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="26.33203125" customWidth="1" min="1" max="1"/>
     <col width="38.5" customWidth="1" min="2" max="2"/>
@@ -52155,7 +52339,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G839"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="21.83203125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="41.6640625" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
     <col width="9.33203125" customWidth="1" style="10" min="2" max="2"/>
@@ -52165,8 +52349,8 @@
     <col width="20.1640625" bestFit="1" customWidth="1" style="10" min="6" max="6"/>
     <col width="48.1640625" bestFit="1" customWidth="1" style="10" min="7" max="7"/>
     <col width="21.83203125" customWidth="1" style="10" min="8" max="256"/>
-    <col width="21.83203125" customWidth="1" style="14" min="257" max="284"/>
-    <col width="21.83203125" customWidth="1" style="14" min="285" max="16384"/>
+    <col width="21.83203125" customWidth="1" style="14" min="257" max="286"/>
+    <col width="21.83203125" customWidth="1" style="14" min="287" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">

</xml_diff>

<commit_message>
changed title of 00164 (note: this causes series_sort to change across most of the series, so lots of commits)
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -1422,8 +1422,8 @@
     <col width="21.5" customWidth="1" style="7" min="23" max="23"/>
     <col width="26.83203125" customWidth="1" style="7" min="24" max="24"/>
     <col width="20.83203125" customWidth="1" style="7" min="25" max="25"/>
-    <col width="10.83203125" customWidth="1" style="7" min="26" max="58"/>
-    <col width="10.83203125" customWidth="1" style="7" min="59" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="26" max="59"/>
+    <col width="10.83203125" customWidth="1" style="7" min="60" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="6">
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="C6" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="C8" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="C10" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="C12" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
       <c r="C18" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="C19" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="C20" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="C21" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="C22" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="C23" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="C24" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
         </is>
       </c>
       <c r="C25" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="C26" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="C27" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
         </is>
       </c>
       <c r="C28" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
         </is>
       </c>
       <c r="C29" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="C30" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="C31" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C32" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
@@ -3535,7 +3535,7 @@
         </is>
       </c>
       <c r="C33" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
@@ -3599,7 +3599,7 @@
         </is>
       </c>
       <c r="C34" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="C35" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="C36" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
@@ -3791,7 +3791,7 @@
         </is>
       </c>
       <c r="C37" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
@@ -3855,7 +3855,7 @@
         </is>
       </c>
       <c r="C38" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="C39" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         </is>
       </c>
       <c r="C40" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
@@ -4047,7 +4047,7 @@
         </is>
       </c>
       <c r="C41" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
@@ -4111,7 +4111,7 @@
         </is>
       </c>
       <c r="C42" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="C43" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="C44" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
@@ -4303,7 +4303,7 @@
         </is>
       </c>
       <c r="C45" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="C46" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="C47" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
@@ -4495,7 +4495,7 @@
         </is>
       </c>
       <c r="C48" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
@@ -4559,7 +4559,7 @@
         </is>
       </c>
       <c r="C49" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
         </is>
       </c>
       <c r="C50" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="C51" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="C52" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="C53" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
@@ -4879,7 +4879,7 @@
         </is>
       </c>
       <c r="C54" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
@@ -4943,7 +4943,7 @@
         </is>
       </c>
       <c r="C55" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
@@ -5007,7 +5007,7 @@
         </is>
       </c>
       <c r="C56" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
@@ -5071,7 +5071,7 @@
         </is>
       </c>
       <c r="C57" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="C58" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
@@ -5199,7 +5199,7 @@
         </is>
       </c>
       <c r="C59" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
@@ -5263,7 +5263,7 @@
         </is>
       </c>
       <c r="C60" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
@@ -5327,7 +5327,7 @@
         </is>
       </c>
       <c r="C61" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="C62" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
@@ -5455,7 +5455,7 @@
         </is>
       </c>
       <c r="C63" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
         </is>
       </c>
       <c r="C64" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
         </is>
       </c>
       <c r="C65" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="C66" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
@@ -5711,7 +5711,7 @@
         </is>
       </c>
       <c r="C67" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
@@ -5775,7 +5775,7 @@
         </is>
       </c>
       <c r="C68" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="C69" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
@@ -5903,7 +5903,7 @@
         </is>
       </c>
       <c r="C70" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
@@ -5967,7 +5967,7 @@
         </is>
       </c>
       <c r="C71" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
@@ -6031,7 +6031,7 @@
         </is>
       </c>
       <c r="C72" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
@@ -6095,7 +6095,7 @@
         </is>
       </c>
       <c r="C73" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         </is>
       </c>
       <c r="C74" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
         </is>
       </c>
       <c r="C75" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="C76" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
@@ -6351,7 +6351,7 @@
         </is>
       </c>
       <c r="C77" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
@@ -6415,7 +6415,7 @@
         </is>
       </c>
       <c r="C78" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
@@ -6479,7 +6479,7 @@
         </is>
       </c>
       <c r="C79" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C80" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
@@ -6607,7 +6607,7 @@
         </is>
       </c>
       <c r="C81" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
@@ -6671,7 +6671,7 @@
         </is>
       </c>
       <c r="C82" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
         </is>
       </c>
       <c r="C83" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
@@ -6799,7 +6799,7 @@
         </is>
       </c>
       <c r="C84" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
@@ -6863,7 +6863,7 @@
         </is>
       </c>
       <c r="C85" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
@@ -6927,7 +6927,7 @@
         </is>
       </c>
       <c r="C86" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
@@ -6991,7 +6991,7 @@
         </is>
       </c>
       <c r="C87" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="C88" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
@@ -7119,7 +7119,7 @@
         </is>
       </c>
       <c r="C89" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="C90" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
@@ -7247,7 +7247,7 @@
         </is>
       </c>
       <c r="C91" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
@@ -7311,7 +7311,7 @@
         </is>
       </c>
       <c r="C92" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
         </is>
       </c>
       <c r="C93" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         </is>
       </c>
       <c r="C94" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
@@ -7503,7 +7503,7 @@
         </is>
       </c>
       <c r="C95" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
@@ -7567,7 +7567,7 @@
         </is>
       </c>
       <c r="C96" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
@@ -7631,7 +7631,7 @@
         </is>
       </c>
       <c r="C97" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
@@ -7695,7 +7695,7 @@
         </is>
       </c>
       <c r="C98" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
@@ -7759,7 +7759,7 @@
         </is>
       </c>
       <c r="C99" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
         </is>
       </c>
       <c r="C100" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
@@ -7887,7 +7887,7 @@
         </is>
       </c>
       <c r="C101" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
@@ -7951,7 +7951,7 @@
         </is>
       </c>
       <c r="C102" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
@@ -8015,7 +8015,7 @@
         </is>
       </c>
       <c r="C103" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
@@ -8079,7 +8079,7 @@
         </is>
       </c>
       <c r="C104" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         </is>
       </c>
       <c r="C105" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
@@ -8207,7 +8207,7 @@
         </is>
       </c>
       <c r="C106" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
@@ -8271,7 +8271,7 @@
         </is>
       </c>
       <c r="C107" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
@@ -8335,7 +8335,7 @@
         </is>
       </c>
       <c r="C108" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
@@ -8399,7 +8399,7 @@
         </is>
       </c>
       <c r="C109" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
@@ -8463,7 +8463,7 @@
         </is>
       </c>
       <c r="C110" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
@@ -8527,7 +8527,7 @@
         </is>
       </c>
       <c r="C111" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
@@ -8591,7 +8591,7 @@
         </is>
       </c>
       <c r="C112" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
@@ -8653,7 +8653,7 @@
         </is>
       </c>
       <c r="C113" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
@@ -8717,7 +8717,7 @@
         </is>
       </c>
       <c r="C114" s="16" t="n">
-        <v>46071</v>
+        <v>46074</v>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
@@ -23389,7 +23389,7 @@
       </c>
       <c r="F342" s="7" t="inlineStr">
         <is>
-          <t>3 commentaries</t>
+          <t>unrelated commentaries</t>
         </is>
       </c>
       <c r="G342" s="7" t="n">
@@ -27477,8 +27477,8 @@
     <col width="21" customWidth="1" style="7" min="7" max="7"/>
     <col width="28.1640625" customWidth="1" style="7" min="8" max="8"/>
     <col width="51" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
-    <col width="10.83203125" customWidth="1" style="1" min="10" max="43"/>
-    <col width="10.83203125" customWidth="1" style="1" min="44" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="1" min="10" max="44"/>
+    <col width="10.83203125" customWidth="1" style="1" min="45" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="3">
@@ -28140,7 +28140,7 @@
         </is>
       </c>
       <c r="D18" s="16" t="n">
-        <v>46072</v>
+        <v>46074</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>1998</v>
@@ -50134,8 +50134,8 @@
     <col width="11.33203125" bestFit="1" customWidth="1" style="19" min="9" max="9"/>
     <col width="12.1640625" bestFit="1" customWidth="1" style="19" min="10" max="10"/>
     <col width="33.6640625" customWidth="1" style="19" min="11" max="11"/>
-    <col width="10.83203125" customWidth="1" style="19" min="12" max="36"/>
-    <col width="10.83203125" customWidth="1" style="19" min="37" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="19" min="12" max="37"/>
+    <col width="10.83203125" customWidth="1" style="19" min="38" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -52349,8 +52349,8 @@
     <col width="20.1640625" bestFit="1" customWidth="1" style="10" min="6" max="6"/>
     <col width="48.1640625" bestFit="1" customWidth="1" style="10" min="7" max="7"/>
     <col width="21.83203125" customWidth="1" style="10" min="8" max="256"/>
-    <col width="21.83203125" customWidth="1" style="14" min="257" max="286"/>
-    <col width="21.83203125" customWidth="1" style="14" min="287" max="16384"/>
+    <col width="21.83203125" customWidth="1" style="14" min="257" max="287"/>
+    <col width="21.83203125" customWidth="1" style="14" min="288" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">

</xml_diff>

<commit_message>
republished tag studio pages
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -36495,7 +36495,7 @@
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>2025</v>
@@ -36555,7 +36555,7 @@
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>1998</v>
@@ -36588,7 +36588,7 @@
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1998</v>
@@ -36616,7 +36616,7 @@
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1996</v>
@@ -36703,7 +36703,7 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>2021</v>
@@ -36734,7 +36734,7 @@
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>2010</v>
@@ -36765,7 +36765,7 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>2025</v>
@@ -36809,7 +36809,7 @@
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>2023</v>
@@ -36835,7 +36835,7 @@
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>2023</v>
@@ -36878,7 +36878,7 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>2025</v>
@@ -36928,7 +36928,7 @@
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>2011</v>
@@ -36954,7 +36954,7 @@
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>2020</v>
@@ -36987,7 +36987,7 @@
         </is>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>2023</v>
@@ -37018,7 +37018,7 @@
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>2023</v>
@@ -37049,7 +37049,7 @@
         </is>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>2016</v>
@@ -37080,7 +37080,7 @@
         </is>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>2010</v>
@@ -37131,7 +37131,7 @@
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>2004</v>
@@ -37159,7 +37159,7 @@
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E28" s="1" t="n">
         <v>2009</v>
@@ -37197,7 +37197,7 @@
         </is>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>1994</v>
@@ -37223,7 +37223,7 @@
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>2013</v>
@@ -37266,7 +37266,7 @@
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E32" s="1" t="n">
         <v>1993</v>
@@ -37299,7 +37299,7 @@
         </is>
       </c>
       <c r="D33" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>1995</v>
@@ -37387,7 +37387,7 @@
         </is>
       </c>
       <c r="D37" s="10" t="n">
-        <v>46081</v>
+        <v>46082</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>2001</v>

</xml_diff>

<commit_message>
Rewrote 24 published _series/*.md files as lightweight stubs.
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -36489,7 +36489,7 @@
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>2025</v>
@@ -36549,7 +36549,7 @@
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>1998</v>
@@ -36582,7 +36582,7 @@
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1998</v>
@@ -36610,7 +36610,7 @@
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1996</v>
@@ -36659,7 +36659,7 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>2025</v>
@@ -36697,7 +36697,7 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>2021</v>
@@ -36728,7 +36728,7 @@
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>2010</v>
@@ -36759,7 +36759,7 @@
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>2025</v>
@@ -36803,7 +36803,7 @@
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>2023</v>
@@ -36829,7 +36829,7 @@
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>2023</v>
@@ -36872,7 +36872,7 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>2025</v>
@@ -36922,7 +36922,7 @@
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>2011</v>
@@ -36948,7 +36948,7 @@
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>2020</v>
@@ -36981,7 +36981,7 @@
         </is>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>2023</v>
@@ -37012,7 +37012,7 @@
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>2023</v>
@@ -37043,7 +37043,7 @@
         </is>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>2016</v>
@@ -37074,7 +37074,7 @@
         </is>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>2010</v>
@@ -37125,7 +37125,7 @@
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>2004</v>
@@ -37153,7 +37153,7 @@
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E28" s="1" t="n">
         <v>2009</v>
@@ -37191,7 +37191,7 @@
         </is>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>1994</v>
@@ -37217,7 +37217,7 @@
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>2013</v>
@@ -37260,7 +37260,7 @@
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E32" s="1" t="n">
         <v>1993</v>
@@ -37293,7 +37293,7 @@
         </is>
       </c>
       <c r="D33" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>1995</v>
@@ -37381,7 +37381,7 @@
         </is>
       </c>
       <c r="D37" s="10" t="n">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>2001</v>

</xml_diff>

<commit_message>
Rewrote 24 published _series/*.md files as lightweight stubs. Rewrote 24 _studio_series/*.md files (existing coupled behavior of series-pages). Updated Series.published_date for 24 rows in data/works.xlsx.
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -37570,7 +37570,7 @@
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="H2" s="5" t="n">
         <v>5906</v>
@@ -37612,7 +37612,7 @@
         </is>
       </c>
       <c r="G3" s="9" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="H3" s="5" t="n">
         <v>5906</v>
@@ -37654,7 +37654,7 @@
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="H4" s="5" t="n">
         <v>5906</v>
@@ -37696,7 +37696,7 @@
         </is>
       </c>
       <c r="G5" s="9" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="H5" s="5" t="n">
         <v>5906</v>
@@ -37738,7 +37738,7 @@
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="H6" s="5" t="n">
         <v>5906</v>
@@ -37780,7 +37780,7 @@
         </is>
       </c>
       <c r="G7" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H7" s="1" t="n">
         <v>4724</v>
@@ -37821,7 +37821,7 @@
         </is>
       </c>
       <c r="G8" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H8" s="1" t="n">
         <v>4724</v>
@@ -37862,7 +37862,7 @@
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>4724</v>
@@ -37903,7 +37903,7 @@
         </is>
       </c>
       <c r="G10" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H10" s="1" t="n">
         <v>4724</v>
@@ -37944,7 +37944,7 @@
         </is>
       </c>
       <c r="G11" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>4724</v>
@@ -37985,7 +37985,7 @@
         </is>
       </c>
       <c r="G12" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H12" s="1" t="n">
         <v>4724</v>
@@ -38026,7 +38026,7 @@
         </is>
       </c>
       <c r="G13" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H13" s="1" t="n">
         <v>4724</v>
@@ -38067,7 +38067,7 @@
         </is>
       </c>
       <c r="G14" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H14" s="1" t="n">
         <v>4724</v>
@@ -38108,7 +38108,7 @@
         </is>
       </c>
       <c r="G15" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H15" s="1" t="n">
         <v>4724</v>
@@ -38149,7 +38149,7 @@
         </is>
       </c>
       <c r="G16" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H16" s="1" t="n">
         <v>4724</v>
@@ -38190,7 +38190,7 @@
         </is>
       </c>
       <c r="G17" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H17" s="1" t="n">
         <v>4724</v>
@@ -38231,7 +38231,7 @@
         </is>
       </c>
       <c r="G18" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H18" s="1" t="n">
         <v>4724</v>
@@ -38272,7 +38272,7 @@
         </is>
       </c>
       <c r="G19" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H19" s="1" t="n">
         <v>4724</v>
@@ -38313,7 +38313,7 @@
         </is>
       </c>
       <c r="G20" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H20" s="1" t="n">
         <v>4724</v>
@@ -38354,7 +38354,7 @@
         </is>
       </c>
       <c r="G21" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H21" s="1" t="n">
         <v>4724</v>
@@ -38395,7 +38395,7 @@
         </is>
       </c>
       <c r="G22" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H22" s="1" t="n">
         <v>4724</v>
@@ -38436,7 +38436,7 @@
         </is>
       </c>
       <c r="G23" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>4724</v>
@@ -38477,7 +38477,7 @@
         </is>
       </c>
       <c r="G24" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H24" s="1" t="n">
         <v>4724</v>
@@ -38518,7 +38518,7 @@
         </is>
       </c>
       <c r="G25" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H25" s="1" t="n">
         <v>4724</v>
@@ -38559,7 +38559,7 @@
         </is>
       </c>
       <c r="G26" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>4724</v>
@@ -38600,7 +38600,7 @@
         </is>
       </c>
       <c r="G27" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H27" s="1" t="n">
         <v>4724</v>
@@ -38641,7 +38641,7 @@
         </is>
       </c>
       <c r="G28" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H28" s="1" t="n">
         <v>4724</v>
@@ -38682,7 +38682,7 @@
         </is>
       </c>
       <c r="G29" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H29" s="1" t="n">
         <v>4724</v>
@@ -38723,7 +38723,7 @@
         </is>
       </c>
       <c r="G30" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H30" s="1" t="n">
         <v>4724</v>
@@ -38764,7 +38764,7 @@
         </is>
       </c>
       <c r="G31" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H31" s="1" t="n">
         <v>4724</v>
@@ -38805,7 +38805,7 @@
         </is>
       </c>
       <c r="G32" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H32" s="1" t="n">
         <v>4724</v>
@@ -38846,7 +38846,7 @@
         </is>
       </c>
       <c r="G33" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H33" s="1" t="n">
         <v>4724</v>
@@ -38887,7 +38887,7 @@
         </is>
       </c>
       <c r="G34" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H34" s="1" t="n">
         <v>4724</v>
@@ -38928,7 +38928,7 @@
         </is>
       </c>
       <c r="G35" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H35" s="1" t="n">
         <v>4724</v>
@@ -38969,7 +38969,7 @@
         </is>
       </c>
       <c r="G36" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H36" s="1" t="n">
         <v>4724</v>
@@ -39010,7 +39010,7 @@
         </is>
       </c>
       <c r="G37" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H37" s="1" t="n">
         <v>4724</v>
@@ -39051,7 +39051,7 @@
         </is>
       </c>
       <c r="G38" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H38" s="1" t="n">
         <v>4724</v>
@@ -39092,7 +39092,7 @@
         </is>
       </c>
       <c r="G39" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H39" s="1" t="n">
         <v>4724</v>
@@ -39133,7 +39133,7 @@
         </is>
       </c>
       <c r="G40" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H40" s="1" t="n">
         <v>4724</v>
@@ -39174,7 +39174,7 @@
         </is>
       </c>
       <c r="G41" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H41" s="1" t="n">
         <v>4724</v>
@@ -39215,7 +39215,7 @@
         </is>
       </c>
       <c r="G42" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H42" s="1" t="n">
         <v>4724</v>
@@ -39256,7 +39256,7 @@
         </is>
       </c>
       <c r="G43" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H43" s="1" t="n">
         <v>4724</v>
@@ -39297,7 +39297,7 @@
         </is>
       </c>
       <c r="G44" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H44" s="1" t="n">
         <v>4724</v>
@@ -39338,7 +39338,7 @@
         </is>
       </c>
       <c r="G45" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H45" s="1" t="n">
         <v>4724</v>
@@ -39379,7 +39379,7 @@
         </is>
       </c>
       <c r="G46" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H46" s="1" t="n">
         <v>4724</v>
@@ -39420,7 +39420,7 @@
         </is>
       </c>
       <c r="G47" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H47" s="1" t="n">
         <v>4724</v>
@@ -39461,7 +39461,7 @@
         </is>
       </c>
       <c r="G48" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H48" s="1" t="n">
         <v>4724</v>
@@ -39502,7 +39502,7 @@
         </is>
       </c>
       <c r="G49" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H49" s="1" t="n">
         <v>4724</v>
@@ -39543,7 +39543,7 @@
         </is>
       </c>
       <c r="G50" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H50" s="1" t="n">
         <v>4724</v>
@@ -39584,7 +39584,7 @@
         </is>
       </c>
       <c r="G51" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H51" s="1" t="n">
         <v>4724</v>
@@ -39625,7 +39625,7 @@
         </is>
       </c>
       <c r="G52" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H52" s="1" t="n">
         <v>4724</v>
@@ -39666,7 +39666,7 @@
         </is>
       </c>
       <c r="G53" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H53" s="1" t="n">
         <v>4724</v>
@@ -39707,7 +39707,7 @@
         </is>
       </c>
       <c r="G54" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H54" s="1" t="n">
         <v>4724</v>
@@ -39748,7 +39748,7 @@
         </is>
       </c>
       <c r="G55" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H55" s="1" t="n">
         <v>4724</v>
@@ -39789,7 +39789,7 @@
         </is>
       </c>
       <c r="G56" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H56" s="1" t="n">
         <v>4724</v>
@@ -39830,7 +39830,7 @@
         </is>
       </c>
       <c r="G57" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H57" s="1" t="n">
         <v>4724</v>
@@ -39871,7 +39871,7 @@
         </is>
       </c>
       <c r="G58" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H58" s="1" t="n">
         <v>4724</v>
@@ -39912,7 +39912,7 @@
         </is>
       </c>
       <c r="G59" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H59" s="1" t="n">
         <v>4724</v>
@@ -39953,7 +39953,7 @@
         </is>
       </c>
       <c r="G60" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H60" s="1" t="n">
         <v>4724</v>
@@ -39994,7 +39994,7 @@
         </is>
       </c>
       <c r="G61" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H61" s="1" t="n">
         <v>4724</v>
@@ -40035,7 +40035,7 @@
         </is>
       </c>
       <c r="G62" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H62" s="1" t="n">
         <v>4724</v>
@@ -40076,7 +40076,7 @@
         </is>
       </c>
       <c r="G63" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H63" s="1" t="n">
         <v>4724</v>
@@ -40117,7 +40117,7 @@
         </is>
       </c>
       <c r="G64" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H64" s="1" t="n">
         <v>4724</v>
@@ -40158,7 +40158,7 @@
         </is>
       </c>
       <c r="G65" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H65" s="1" t="n">
         <v>4724</v>
@@ -40199,7 +40199,7 @@
         </is>
       </c>
       <c r="G66" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H66" s="1" t="n">
         <v>4724</v>
@@ -40240,7 +40240,7 @@
         </is>
       </c>
       <c r="G67" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H67" s="1" t="n">
         <v>4724</v>
@@ -40281,7 +40281,7 @@
         </is>
       </c>
       <c r="G68" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H68" s="1" t="n">
         <v>4724</v>
@@ -40322,7 +40322,7 @@
         </is>
       </c>
       <c r="G69" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H69" s="1" t="n">
         <v>4724</v>
@@ -40363,7 +40363,7 @@
         </is>
       </c>
       <c r="G70" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H70" s="1" t="n">
         <v>4724</v>
@@ -40404,7 +40404,7 @@
         </is>
       </c>
       <c r="G71" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H71" s="1" t="n">
         <v>4724</v>
@@ -40445,7 +40445,7 @@
         </is>
       </c>
       <c r="G72" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H72" s="1" t="n">
         <v>4724</v>
@@ -40486,7 +40486,7 @@
         </is>
       </c>
       <c r="G73" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H73" s="1" t="n">
         <v>4724</v>
@@ -40527,7 +40527,7 @@
         </is>
       </c>
       <c r="G74" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H74" s="1" t="n">
         <v>4724</v>
@@ -40568,7 +40568,7 @@
         </is>
       </c>
       <c r="G75" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H75" s="1" t="n">
         <v>4724</v>
@@ -40609,7 +40609,7 @@
         </is>
       </c>
       <c r="G76" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H76" s="1" t="n">
         <v>4724</v>
@@ -40650,7 +40650,7 @@
         </is>
       </c>
       <c r="G77" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H77" s="1" t="n">
         <v>4724</v>
@@ -40691,7 +40691,7 @@
         </is>
       </c>
       <c r="G78" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H78" s="1" t="n">
         <v>4724</v>
@@ -40732,7 +40732,7 @@
         </is>
       </c>
       <c r="G79" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H79" s="1" t="n">
         <v>4724</v>
@@ -40773,7 +40773,7 @@
         </is>
       </c>
       <c r="G80" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H80" s="1" t="n">
         <v>4724</v>
@@ -40814,7 +40814,7 @@
         </is>
       </c>
       <c r="G81" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H81" s="1" t="n">
         <v>4724</v>
@@ -40855,7 +40855,7 @@
         </is>
       </c>
       <c r="G82" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H82" s="1" t="n">
         <v>4724</v>
@@ -40896,7 +40896,7 @@
         </is>
       </c>
       <c r="G83" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H83" s="1" t="n">
         <v>4724</v>
@@ -40937,7 +40937,7 @@
         </is>
       </c>
       <c r="G84" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H84" s="1" t="n">
         <v>4724</v>
@@ -40978,7 +40978,7 @@
         </is>
       </c>
       <c r="G85" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H85" s="1" t="n">
         <v>4724</v>
@@ -41019,7 +41019,7 @@
         </is>
       </c>
       <c r="G86" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H86" s="1" t="n">
         <v>4724</v>
@@ -41060,7 +41060,7 @@
         </is>
       </c>
       <c r="G87" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H87" s="1" t="n">
         <v>4724</v>
@@ -41101,7 +41101,7 @@
         </is>
       </c>
       <c r="G88" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H88" s="1" t="n">
         <v>4724</v>
@@ -41142,7 +41142,7 @@
         </is>
       </c>
       <c r="G89" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H89" s="1" t="n">
         <v>4724</v>
@@ -41183,7 +41183,7 @@
         </is>
       </c>
       <c r="G90" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H90" s="1" t="n">
         <v>4724</v>
@@ -41224,7 +41224,7 @@
         </is>
       </c>
       <c r="G91" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H91" s="1" t="n">
         <v>4724</v>
@@ -41265,7 +41265,7 @@
         </is>
       </c>
       <c r="G92" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H92" s="1" t="n">
         <v>4724</v>
@@ -41306,7 +41306,7 @@
         </is>
       </c>
       <c r="G93" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H93" s="1" t="n">
         <v>4724</v>
@@ -41347,7 +41347,7 @@
         </is>
       </c>
       <c r="G94" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H94" s="1" t="n">
         <v>4724</v>
@@ -41388,7 +41388,7 @@
         </is>
       </c>
       <c r="G95" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H95" s="1" t="n">
         <v>4724</v>
@@ -41429,7 +41429,7 @@
         </is>
       </c>
       <c r="G96" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H96" s="1" t="n">
         <v>4724</v>
@@ -41470,7 +41470,7 @@
         </is>
       </c>
       <c r="G97" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H97" s="1" t="n">
         <v>4724</v>
@@ -41511,7 +41511,7 @@
         </is>
       </c>
       <c r="G98" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H98" s="1" t="n">
         <v>4724</v>
@@ -41552,7 +41552,7 @@
         </is>
       </c>
       <c r="G99" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H99" s="1" t="n">
         <v>4724</v>
@@ -41593,7 +41593,7 @@
         </is>
       </c>
       <c r="G100" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H100" s="1" t="n">
         <v>4724</v>
@@ -41634,7 +41634,7 @@
         </is>
       </c>
       <c r="G101" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H101" s="1" t="n">
         <v>4724</v>
@@ -41675,7 +41675,7 @@
         </is>
       </c>
       <c r="G102" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H102" s="1" t="n">
         <v>4724</v>
@@ -41716,7 +41716,7 @@
         </is>
       </c>
       <c r="G103" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H103" s="1" t="n">
         <v>4724</v>
@@ -41757,7 +41757,7 @@
         </is>
       </c>
       <c r="G104" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H104" s="1" t="n">
         <v>4724</v>
@@ -41798,7 +41798,7 @@
         </is>
       </c>
       <c r="G105" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H105" s="1" t="n">
         <v>4724</v>
@@ -41839,7 +41839,7 @@
         </is>
       </c>
       <c r="G106" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H106" s="1" t="n">
         <v>4724</v>
@@ -41880,7 +41880,7 @@
         </is>
       </c>
       <c r="G107" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H107" s="1" t="n">
         <v>4724</v>
@@ -41921,7 +41921,7 @@
         </is>
       </c>
       <c r="G108" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H108" s="1" t="n">
         <v>4724</v>
@@ -41962,7 +41962,7 @@
         </is>
       </c>
       <c r="G109" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H109" s="1" t="n">
         <v>4724</v>
@@ -42003,7 +42003,7 @@
         </is>
       </c>
       <c r="G110" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H110" s="1" t="n">
         <v>4724</v>
@@ -42044,7 +42044,7 @@
         </is>
       </c>
       <c r="G111" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H111" s="1" t="n">
         <v>4724</v>
@@ -42085,7 +42085,7 @@
         </is>
       </c>
       <c r="G112" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H112" s="1" t="n">
         <v>4724</v>
@@ -42126,7 +42126,7 @@
         </is>
       </c>
       <c r="G113" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H113" s="1" t="n">
         <v>4724</v>
@@ -42167,7 +42167,7 @@
         </is>
       </c>
       <c r="G114" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H114" s="1" t="n">
         <v>4724</v>
@@ -42208,7 +42208,7 @@
         </is>
       </c>
       <c r="G115" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H115" s="1" t="n">
         <v>4724</v>
@@ -42249,7 +42249,7 @@
         </is>
       </c>
       <c r="G116" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H116" s="1" t="n">
         <v>4724</v>
@@ -42290,7 +42290,7 @@
         </is>
       </c>
       <c r="G117" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H117" s="1" t="n">
         <v>4724</v>
@@ -42331,7 +42331,7 @@
         </is>
       </c>
       <c r="G118" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H118" s="1" t="n">
         <v>4724</v>
@@ -42372,7 +42372,7 @@
         </is>
       </c>
       <c r="G119" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H119" s="1" t="n">
         <v>4724</v>
@@ -42413,7 +42413,7 @@
         </is>
       </c>
       <c r="G120" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H120" s="1" t="n">
         <v>4724</v>
@@ -42454,7 +42454,7 @@
         </is>
       </c>
       <c r="G121" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H121" s="1" t="n">
         <v>4724</v>
@@ -42495,7 +42495,7 @@
         </is>
       </c>
       <c r="G122" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H122" s="1" t="n">
         <v>4724</v>
@@ -42536,7 +42536,7 @@
         </is>
       </c>
       <c r="G123" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H123" s="1" t="n">
         <v>4724</v>
@@ -42577,7 +42577,7 @@
         </is>
       </c>
       <c r="G124" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H124" s="1" t="n">
         <v>4724</v>
@@ -42618,7 +42618,7 @@
         </is>
       </c>
       <c r="G125" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H125" s="1" t="n">
         <v>4724</v>
@@ -42659,7 +42659,7 @@
         </is>
       </c>
       <c r="G126" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H126" s="1" t="n">
         <v>4724</v>
@@ -42700,7 +42700,7 @@
         </is>
       </c>
       <c r="G127" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H127" s="1" t="n">
         <v>4724</v>
@@ -42741,7 +42741,7 @@
         </is>
       </c>
       <c r="G128" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H128" s="1" t="n">
         <v>4724</v>
@@ -42782,7 +42782,7 @@
         </is>
       </c>
       <c r="G129" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H129" s="1" t="n">
         <v>4724</v>
@@ -42823,7 +42823,7 @@
         </is>
       </c>
       <c r="G130" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H130" s="1" t="n">
         <v>4724</v>
@@ -42864,7 +42864,7 @@
         </is>
       </c>
       <c r="G131" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H131" s="1" t="n">
         <v>4724</v>
@@ -42905,7 +42905,7 @@
         </is>
       </c>
       <c r="G132" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H132" s="1" t="n">
         <v>4724</v>
@@ -42946,7 +42946,7 @@
         </is>
       </c>
       <c r="G133" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H133" s="1" t="n">
         <v>4724</v>
@@ -42987,7 +42987,7 @@
         </is>
       </c>
       <c r="G134" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H134" s="1" t="n">
         <v>4724</v>
@@ -43028,7 +43028,7 @@
         </is>
       </c>
       <c r="G135" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H135" s="1" t="n">
         <v>4724</v>
@@ -43069,7 +43069,7 @@
         </is>
       </c>
       <c r="G136" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H136" s="1" t="n">
         <v>4724</v>
@@ -43110,7 +43110,7 @@
         </is>
       </c>
       <c r="G137" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H137" s="1" t="n">
         <v>4724</v>
@@ -43151,7 +43151,7 @@
         </is>
       </c>
       <c r="G138" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H138" s="1" t="n">
         <v>4724</v>
@@ -43192,7 +43192,7 @@
         </is>
       </c>
       <c r="G139" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H139" s="1" t="n">
         <v>4724</v>
@@ -43233,7 +43233,7 @@
         </is>
       </c>
       <c r="G140" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H140" s="1" t="n">
         <v>4724</v>
@@ -43274,7 +43274,7 @@
         </is>
       </c>
       <c r="G141" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H141" s="1" t="n">
         <v>4724</v>
@@ -43315,7 +43315,7 @@
         </is>
       </c>
       <c r="G142" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H142" s="1" t="n">
         <v>4724</v>
@@ -43356,7 +43356,7 @@
         </is>
       </c>
       <c r="G143" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H143" s="1" t="n">
         <v>4724</v>
@@ -43397,7 +43397,7 @@
         </is>
       </c>
       <c r="G144" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H144" s="1" t="n">
         <v>4724</v>
@@ -43438,7 +43438,7 @@
         </is>
       </c>
       <c r="G145" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H145" s="1" t="n">
         <v>4724</v>
@@ -43479,7 +43479,7 @@
         </is>
       </c>
       <c r="G146" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H146" s="1" t="n">
         <v>4724</v>
@@ -43520,7 +43520,7 @@
         </is>
       </c>
       <c r="G147" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H147" s="1" t="n">
         <v>4724</v>
@@ -43561,7 +43561,7 @@
         </is>
       </c>
       <c r="G148" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H148" s="1" t="n">
         <v>4724</v>
@@ -43602,7 +43602,7 @@
         </is>
       </c>
       <c r="G149" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H149" s="1" t="n">
         <v>4724</v>
@@ -43643,7 +43643,7 @@
         </is>
       </c>
       <c r="G150" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H150" s="1" t="n">
         <v>4724</v>
@@ -43684,7 +43684,7 @@
         </is>
       </c>
       <c r="G151" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H151" s="1" t="n">
         <v>4724</v>
@@ -43725,7 +43725,7 @@
         </is>
       </c>
       <c r="G152" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H152" s="1" t="n">
         <v>4724</v>
@@ -43766,7 +43766,7 @@
         </is>
       </c>
       <c r="G153" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H153" s="1" t="n">
         <v>4724</v>
@@ -43807,7 +43807,7 @@
         </is>
       </c>
       <c r="G154" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H154" s="1" t="n">
         <v>4724</v>
@@ -43848,7 +43848,7 @@
         </is>
       </c>
       <c r="G155" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H155" s="1" t="n">
         <v>4724</v>
@@ -43889,7 +43889,7 @@
         </is>
       </c>
       <c r="G156" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H156" s="1" t="n">
         <v>4724</v>
@@ -43930,7 +43930,7 @@
         </is>
       </c>
       <c r="G157" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H157" s="1" t="n">
         <v>4724</v>
@@ -43971,7 +43971,7 @@
         </is>
       </c>
       <c r="G158" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H158" s="1" t="n">
         <v>4724</v>
@@ -44012,7 +44012,7 @@
         </is>
       </c>
       <c r="G159" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H159" s="1" t="n">
         <v>4724</v>
@@ -44053,7 +44053,7 @@
         </is>
       </c>
       <c r="G160" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H160" s="1" t="n">
         <v>4724</v>
@@ -44094,7 +44094,7 @@
         </is>
       </c>
       <c r="G161" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H161" s="1" t="n">
         <v>4724</v>
@@ -44135,7 +44135,7 @@
         </is>
       </c>
       <c r="G162" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H162" s="1" t="n">
         <v>4724</v>
@@ -44176,7 +44176,7 @@
         </is>
       </c>
       <c r="G163" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H163" s="1" t="n">
         <v>4724</v>
@@ -44217,7 +44217,7 @@
         </is>
       </c>
       <c r="G164" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H164" s="1" t="n">
         <v>4724</v>
@@ -44258,7 +44258,7 @@
         </is>
       </c>
       <c r="G165" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H165" s="1" t="n">
         <v>4724</v>
@@ -44299,7 +44299,7 @@
         </is>
       </c>
       <c r="G166" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H166" s="1" t="n">
         <v>4724</v>
@@ -44340,7 +44340,7 @@
         </is>
       </c>
       <c r="G167" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H167" s="1" t="n">
         <v>4724</v>
@@ -44381,7 +44381,7 @@
         </is>
       </c>
       <c r="G168" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H168" s="1" t="n">
         <v>4724</v>
@@ -44422,7 +44422,7 @@
         </is>
       </c>
       <c r="G169" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H169" s="1" t="n">
         <v>4724</v>
@@ -44463,7 +44463,7 @@
         </is>
       </c>
       <c r="G170" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H170" s="1" t="n">
         <v>4724</v>
@@ -44504,7 +44504,7 @@
         </is>
       </c>
       <c r="G171" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H171" s="1" t="n">
         <v>4724</v>
@@ -44545,7 +44545,7 @@
         </is>
       </c>
       <c r="G172" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H172" s="1" t="n">
         <v>4724</v>
@@ -44586,7 +44586,7 @@
         </is>
       </c>
       <c r="G173" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H173" s="1" t="n">
         <v>4724</v>
@@ -44627,7 +44627,7 @@
         </is>
       </c>
       <c r="G174" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H174" s="1" t="n">
         <v>4724</v>
@@ -44668,7 +44668,7 @@
         </is>
       </c>
       <c r="G175" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H175" s="1" t="n">
         <v>4724</v>
@@ -44709,7 +44709,7 @@
         </is>
       </c>
       <c r="G176" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H176" s="1" t="n">
         <v>4724</v>
@@ -44750,7 +44750,7 @@
         </is>
       </c>
       <c r="G177" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H177" s="1" t="n">
         <v>4724</v>
@@ -44791,7 +44791,7 @@
         </is>
       </c>
       <c r="G178" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H178" s="1" t="n">
         <v>4724</v>
@@ -44832,7 +44832,7 @@
         </is>
       </c>
       <c r="G179" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H179" s="1" t="n">
         <v>4724</v>
@@ -44873,7 +44873,7 @@
         </is>
       </c>
       <c r="G180" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H180" s="1" t="n">
         <v>4724</v>
@@ -44914,7 +44914,7 @@
         </is>
       </c>
       <c r="G181" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H181" s="1" t="n">
         <v>4724</v>
@@ -44955,7 +44955,7 @@
         </is>
       </c>
       <c r="G182" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H182" s="1" t="n">
         <v>4724</v>
@@ -44996,7 +44996,7 @@
         </is>
       </c>
       <c r="G183" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H183" s="1" t="n">
         <v>4724</v>
@@ -45037,7 +45037,7 @@
         </is>
       </c>
       <c r="G184" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H184" s="1" t="n">
         <v>4724</v>
@@ -45078,7 +45078,7 @@
         </is>
       </c>
       <c r="G185" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H185" s="1" t="n">
         <v>4724</v>
@@ -45119,7 +45119,7 @@
         </is>
       </c>
       <c r="G186" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H186" s="1" t="n">
         <v>4724</v>
@@ -45160,7 +45160,7 @@
         </is>
       </c>
       <c r="G187" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H187" s="1" t="n">
         <v>4724</v>
@@ -45201,7 +45201,7 @@
         </is>
       </c>
       <c r="G188" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H188" s="1" t="n">
         <v>4724</v>
@@ -45242,7 +45242,7 @@
         </is>
       </c>
       <c r="G189" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H189" s="1" t="n">
         <v>4724</v>
@@ -45283,7 +45283,7 @@
         </is>
       </c>
       <c r="G190" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H190" s="1" t="n">
         <v>4724</v>
@@ -45324,7 +45324,7 @@
         </is>
       </c>
       <c r="G191" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H191" s="1" t="n">
         <v>4724</v>
@@ -45365,7 +45365,7 @@
         </is>
       </c>
       <c r="G192" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H192" s="1" t="n">
         <v>4724</v>
@@ -45406,7 +45406,7 @@
         </is>
       </c>
       <c r="G193" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H193" s="1" t="n">
         <v>4724</v>
@@ -45447,7 +45447,7 @@
         </is>
       </c>
       <c r="G194" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H194" s="1" t="n">
         <v>4724</v>
@@ -45488,7 +45488,7 @@
         </is>
       </c>
       <c r="G195" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H195" s="1" t="n">
         <v>4724</v>
@@ -45529,7 +45529,7 @@
         </is>
       </c>
       <c r="G196" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H196" s="1" t="n">
         <v>4724</v>
@@ -45570,7 +45570,7 @@
         </is>
       </c>
       <c r="G197" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H197" s="1" t="n">
         <v>4724</v>
@@ -45611,7 +45611,7 @@
         </is>
       </c>
       <c r="G198" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H198" s="1" t="n">
         <v>4724</v>
@@ -45652,7 +45652,7 @@
         </is>
       </c>
       <c r="G199" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H199" s="1" t="n">
         <v>4724</v>
@@ -45693,7 +45693,7 @@
         </is>
       </c>
       <c r="G200" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H200" s="1" t="n">
         <v>4724</v>
@@ -45734,7 +45734,7 @@
         </is>
       </c>
       <c r="G201" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H201" s="1" t="n">
         <v>4724</v>
@@ -45775,7 +45775,7 @@
         </is>
       </c>
       <c r="G202" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H202" s="1" t="n">
         <v>4724</v>
@@ -45816,7 +45816,7 @@
         </is>
       </c>
       <c r="G203" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H203" s="1" t="n">
         <v>4724</v>
@@ -45857,7 +45857,7 @@
         </is>
       </c>
       <c r="G204" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H204" s="1" t="n">
         <v>4724</v>
@@ -45898,7 +45898,7 @@
         </is>
       </c>
       <c r="G205" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H205" s="1" t="n">
         <v>4724</v>
@@ -45939,7 +45939,7 @@
         </is>
       </c>
       <c r="G206" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H206" s="1" t="n">
         <v>4724</v>
@@ -45980,7 +45980,7 @@
         </is>
       </c>
       <c r="G207" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H207" s="1" t="n">
         <v>4724</v>
@@ -46021,7 +46021,7 @@
         </is>
       </c>
       <c r="G208" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H208" s="1" t="n">
         <v>4724</v>
@@ -46062,7 +46062,7 @@
         </is>
       </c>
       <c r="G209" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H209" s="1" t="n">
         <v>4724</v>
@@ -46103,7 +46103,7 @@
         </is>
       </c>
       <c r="G210" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H210" s="1" t="n">
         <v>4724</v>
@@ -46144,7 +46144,7 @@
         </is>
       </c>
       <c r="G211" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H211" s="1" t="n">
         <v>4724</v>
@@ -46185,7 +46185,7 @@
         </is>
       </c>
       <c r="G212" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H212" s="1" t="n">
         <v>4724</v>
@@ -46226,7 +46226,7 @@
         </is>
       </c>
       <c r="G213" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H213" s="1" t="n">
         <v>4724</v>
@@ -46267,7 +46267,7 @@
         </is>
       </c>
       <c r="G214" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H214" s="1" t="n">
         <v>4724</v>
@@ -46308,7 +46308,7 @@
         </is>
       </c>
       <c r="G215" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H215" s="1" t="n">
         <v>4724</v>
@@ -46349,7 +46349,7 @@
         </is>
       </c>
       <c r="G216" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H216" s="1" t="n">
         <v>4724</v>
@@ -46390,7 +46390,7 @@
         </is>
       </c>
       <c r="G217" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H217" s="1" t="n">
         <v>4724</v>
@@ -46431,7 +46431,7 @@
         </is>
       </c>
       <c r="G218" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H218" s="1" t="n">
         <v>4724</v>
@@ -46472,7 +46472,7 @@
         </is>
       </c>
       <c r="G219" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H219" s="1" t="n">
         <v>4724</v>
@@ -46513,7 +46513,7 @@
         </is>
       </c>
       <c r="G220" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H220" s="1" t="n">
         <v>4724</v>
@@ -46554,7 +46554,7 @@
         </is>
       </c>
       <c r="G221" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H221" s="1" t="n">
         <v>4724</v>
@@ -46595,7 +46595,7 @@
         </is>
       </c>
       <c r="G222" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H222" s="1" t="n">
         <v>4724</v>
@@ -46636,7 +46636,7 @@
         </is>
       </c>
       <c r="G223" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H223" s="1" t="n">
         <v>4724</v>
@@ -46677,7 +46677,7 @@
         </is>
       </c>
       <c r="G224" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H224" s="1" t="n">
         <v>4724</v>
@@ -46718,7 +46718,7 @@
         </is>
       </c>
       <c r="G225" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H225" s="1" t="n">
         <v>4724</v>
@@ -46759,7 +46759,7 @@
         </is>
       </c>
       <c r="G226" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H226" s="1" t="n">
         <v>4724</v>
@@ -46800,7 +46800,7 @@
         </is>
       </c>
       <c r="G227" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H227" s="1" t="n">
         <v>4724</v>
@@ -46841,7 +46841,7 @@
         </is>
       </c>
       <c r="G228" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H228" s="1" t="n">
         <v>4724</v>
@@ -46882,7 +46882,7 @@
         </is>
       </c>
       <c r="G229" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H229" s="1" t="n">
         <v>4724</v>
@@ -46923,7 +46923,7 @@
         </is>
       </c>
       <c r="G230" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H230" s="1" t="n">
         <v>4724</v>
@@ -46964,7 +46964,7 @@
         </is>
       </c>
       <c r="G231" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H231" s="1" t="n">
         <v>4724</v>
@@ -47005,7 +47005,7 @@
         </is>
       </c>
       <c r="G232" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H232" s="1" t="n">
         <v>4724</v>
@@ -47046,7 +47046,7 @@
         </is>
       </c>
       <c r="G233" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H233" s="1" t="n">
         <v>4724</v>
@@ -47087,7 +47087,7 @@
         </is>
       </c>
       <c r="G234" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H234" s="1" t="n">
         <v>4724</v>
@@ -47128,7 +47128,7 @@
         </is>
       </c>
       <c r="G235" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H235" s="1" t="n">
         <v>4724</v>
@@ -47169,7 +47169,7 @@
         </is>
       </c>
       <c r="G236" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H236" s="1" t="n">
         <v>4724</v>
@@ -47210,7 +47210,7 @@
         </is>
       </c>
       <c r="G237" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H237" s="1" t="n">
         <v>4724</v>
@@ -47251,7 +47251,7 @@
         </is>
       </c>
       <c r="G238" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H238" s="1" t="n">
         <v>4724</v>
@@ -47292,7 +47292,7 @@
         </is>
       </c>
       <c r="G239" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H239" s="1" t="n">
         <v>4724</v>
@@ -47333,7 +47333,7 @@
         </is>
       </c>
       <c r="G240" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H240" s="1" t="n">
         <v>4724</v>
@@ -47374,7 +47374,7 @@
         </is>
       </c>
       <c r="G241" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H241" s="1" t="n">
         <v>4724</v>
@@ -47415,7 +47415,7 @@
         </is>
       </c>
       <c r="G242" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H242" s="1" t="n">
         <v>4724</v>
@@ -47456,7 +47456,7 @@
         </is>
       </c>
       <c r="G243" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H243" s="1" t="n">
         <v>4724</v>
@@ -47497,7 +47497,7 @@
         </is>
       </c>
       <c r="G244" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H244" s="1" t="n">
         <v>4724</v>
@@ -47538,7 +47538,7 @@
         </is>
       </c>
       <c r="G245" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H245" s="1" t="n">
         <v>4724</v>
@@ -47579,7 +47579,7 @@
         </is>
       </c>
       <c r="G246" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H246" s="1" t="n">
         <v>4724</v>
@@ -47620,7 +47620,7 @@
         </is>
       </c>
       <c r="G247" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H247" s="1" t="n">
         <v>4724</v>
@@ -47661,7 +47661,7 @@
         </is>
       </c>
       <c r="G248" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H248" s="1" t="n">
         <v>4724</v>
@@ -47702,7 +47702,7 @@
         </is>
       </c>
       <c r="G249" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H249" s="1" t="n">
         <v>4724</v>
@@ -47743,7 +47743,7 @@
         </is>
       </c>
       <c r="G250" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H250" s="1" t="n">
         <v>4724</v>
@@ -47784,7 +47784,7 @@
         </is>
       </c>
       <c r="G251" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H251" s="1" t="n">
         <v>4724</v>
@@ -47825,7 +47825,7 @@
         </is>
       </c>
       <c r="G252" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H252" s="1" t="n">
         <v>4724</v>
@@ -47866,7 +47866,7 @@
         </is>
       </c>
       <c r="G253" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H253" s="1" t="n">
         <v>4724</v>
@@ -47907,7 +47907,7 @@
         </is>
       </c>
       <c r="G254" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H254" s="1" t="n">
         <v>4724</v>
@@ -47948,7 +47948,7 @@
         </is>
       </c>
       <c r="G255" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H255" s="1" t="n">
         <v>4724</v>
@@ -47989,7 +47989,7 @@
         </is>
       </c>
       <c r="G256" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H256" s="1" t="n">
         <v>4724</v>
@@ -48030,7 +48030,7 @@
         </is>
       </c>
       <c r="G257" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H257" s="1" t="n">
         <v>4724</v>
@@ -48071,7 +48071,7 @@
         </is>
       </c>
       <c r="G258" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H258" s="1" t="n">
         <v>4724</v>
@@ -48112,7 +48112,7 @@
         </is>
       </c>
       <c r="G259" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H259" s="1" t="n">
         <v>4724</v>
@@ -48153,7 +48153,7 @@
         </is>
       </c>
       <c r="G260" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H260" s="1" t="n">
         <v>4724</v>
@@ -48194,7 +48194,7 @@
         </is>
       </c>
       <c r="G261" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H261" s="1" t="n">
         <v>4724</v>
@@ -48235,7 +48235,7 @@
         </is>
       </c>
       <c r="G262" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H262" s="1" t="n">
         <v>4724</v>
@@ -48276,7 +48276,7 @@
         </is>
       </c>
       <c r="G263" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H263" s="1" t="n">
         <v>9000</v>
@@ -48317,7 +48317,7 @@
         </is>
       </c>
       <c r="G264" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H264" s="1" t="n">
         <v>9000</v>
@@ -48358,7 +48358,7 @@
         </is>
       </c>
       <c r="G265" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H265" s="1" t="n">
         <v>9000</v>
@@ -48399,7 +48399,7 @@
         </is>
       </c>
       <c r="G266" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H266" s="1" t="n">
         <v>9000</v>
@@ -48440,7 +48440,7 @@
         </is>
       </c>
       <c r="G267" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H267" s="1" t="n">
         <v>3543</v>
@@ -48481,7 +48481,7 @@
         </is>
       </c>
       <c r="G268" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H268" s="1" t="n">
         <v>3543</v>
@@ -48522,7 +48522,7 @@
         </is>
       </c>
       <c r="G269" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H269" s="1" t="n">
         <v>3543</v>
@@ -48563,7 +48563,7 @@
         </is>
       </c>
       <c r="G270" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H270" s="1" t="n">
         <v>3543</v>
@@ -48604,7 +48604,7 @@
         </is>
       </c>
       <c r="G271" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H271" s="1" t="n">
         <v>3543</v>
@@ -48645,7 +48645,7 @@
         </is>
       </c>
       <c r="G272" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H272" s="1" t="n">
         <v>3543</v>
@@ -48686,7 +48686,7 @@
         </is>
       </c>
       <c r="G273" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H273" s="1" t="n">
         <v>3543</v>
@@ -48727,7 +48727,7 @@
         </is>
       </c>
       <c r="G274" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H274" s="1" t="n">
         <v>3543</v>
@@ -48768,7 +48768,7 @@
         </is>
       </c>
       <c r="G275" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H275" s="1" t="n">
         <v>3543</v>
@@ -48809,7 +48809,7 @@
         </is>
       </c>
       <c r="G276" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H276" s="1" t="n">
         <v>3543</v>
@@ -48850,7 +48850,7 @@
         </is>
       </c>
       <c r="G277" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H277" s="1" t="n">
         <v>3543</v>
@@ -48891,7 +48891,7 @@
         </is>
       </c>
       <c r="G278" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H278" s="1" t="n">
         <v>3543</v>
@@ -48932,7 +48932,7 @@
         </is>
       </c>
       <c r="G279" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H279" s="1" t="n">
         <v>3543</v>
@@ -48973,7 +48973,7 @@
         </is>
       </c>
       <c r="G280" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H280" s="1" t="n">
         <v>3543</v>
@@ -49014,7 +49014,7 @@
         </is>
       </c>
       <c r="G281" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H281" s="1" t="n">
         <v>3543</v>
@@ -49055,7 +49055,7 @@
         </is>
       </c>
       <c r="G282" s="10" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="H282" s="1" t="n">
         <v>3543</v>
@@ -49096,7 +49096,7 @@
         </is>
       </c>
       <c r="G283" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H283" s="1" t="n">
         <v>2169</v>
@@ -49137,7 +49137,7 @@
         </is>
       </c>
       <c r="G284" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H284" s="1" t="n">
         <v>5315</v>
@@ -49178,7 +49178,7 @@
         </is>
       </c>
       <c r="G285" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H285" s="1" t="n">
         <v>7087</v>
@@ -49219,7 +49219,7 @@
         </is>
       </c>
       <c r="G286" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H286" s="1" t="n">
         <v>7087</v>
@@ -49260,7 +49260,7 @@
         </is>
       </c>
       <c r="G287" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H287" s="1" t="n">
         <v>1400</v>
@@ -49301,7 +49301,7 @@
         </is>
       </c>
       <c r="G288" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H288" s="1" t="n">
         <v>7087</v>
@@ -49342,7 +49342,7 @@
         </is>
       </c>
       <c r="G289" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H289" s="1" t="n">
         <v>1400</v>
@@ -49383,7 +49383,7 @@
         </is>
       </c>
       <c r="G290" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H290" t="n">
         <v>8268</v>
@@ -49424,7 +49424,7 @@
         </is>
       </c>
       <c r="G291" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H291" t="n">
         <v>8268</v>
@@ -49465,7 +49465,7 @@
         </is>
       </c>
       <c r="G292" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H292" t="n">
         <v>8268</v>
@@ -49506,7 +49506,7 @@
         </is>
       </c>
       <c r="G293" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H293" t="n">
         <v>4000</v>
@@ -49547,7 +49547,7 @@
         </is>
       </c>
       <c r="G294" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H294" t="n">
         <v>2362</v>
@@ -49588,7 +49588,7 @@
         </is>
       </c>
       <c r="G295" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H295" t="n">
         <v>2362</v>
@@ -49629,7 +49629,7 @@
         </is>
       </c>
       <c r="G296" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H296" t="n">
         <v>2362</v>
@@ -49670,7 +49670,7 @@
         </is>
       </c>
       <c r="G297" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H297" t="n">
         <v>2362</v>
@@ -49711,7 +49711,7 @@
         </is>
       </c>
       <c r="G298" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H298" t="n">
         <v>2362</v>
@@ -49752,7 +49752,7 @@
         </is>
       </c>
       <c r="G299" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H299" t="n">
         <v>2362</v>
@@ -49793,7 +49793,7 @@
         </is>
       </c>
       <c r="G300" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H300" t="n">
         <v>2362</v>
@@ -49834,7 +49834,7 @@
         </is>
       </c>
       <c r="G301" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H301" t="n">
         <v>2362</v>
@@ -49875,7 +49875,7 @@
         </is>
       </c>
       <c r="G302" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H302" t="n">
         <v>2362</v>
@@ -49916,7 +49916,7 @@
         </is>
       </c>
       <c r="G303" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H303" t="n">
         <v>2362</v>
@@ -49957,7 +49957,7 @@
         </is>
       </c>
       <c r="G304" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H304" t="n">
         <v>2362</v>
@@ -49998,7 +49998,7 @@
         </is>
       </c>
       <c r="G305" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H305" t="n">
         <v>2362</v>
@@ -50039,7 +50039,7 @@
         </is>
       </c>
       <c r="G306" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H306" t="n">
         <v>2362</v>
@@ -50080,7 +50080,7 @@
         </is>
       </c>
       <c r="G307" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H307" t="n">
         <v>2362</v>
@@ -50121,7 +50121,7 @@
         </is>
       </c>
       <c r="G308" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H308" t="n">
         <v>2362</v>
@@ -50162,7 +50162,7 @@
         </is>
       </c>
       <c r="G309" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H309" t="n">
         <v>2362</v>
@@ -50203,7 +50203,7 @@
         </is>
       </c>
       <c r="G310" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H310" t="n">
         <v>2362</v>
@@ -50244,7 +50244,7 @@
         </is>
       </c>
       <c r="G311" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H311" t="n">
         <v>2362</v>
@@ -50285,7 +50285,7 @@
         </is>
       </c>
       <c r="G312" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H312" t="n">
         <v>2362</v>
@@ -50326,7 +50326,7 @@
         </is>
       </c>
       <c r="G313" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H313" t="n">
         <v>2362</v>
@@ -50367,7 +50367,7 @@
         </is>
       </c>
       <c r="G314" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H314" t="n">
         <v>2362</v>
@@ -50408,7 +50408,7 @@
         </is>
       </c>
       <c r="G315" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H315" t="n">
         <v>2362</v>
@@ -50449,7 +50449,7 @@
         </is>
       </c>
       <c r="G316" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H316" t="n">
         <v>2362</v>
@@ -50490,7 +50490,7 @@
         </is>
       </c>
       <c r="G317" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H317" t="n">
         <v>2362</v>
@@ -50531,7 +50531,7 @@
         </is>
       </c>
       <c r="G318" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H318" t="n">
         <v>2362</v>
@@ -50572,7 +50572,7 @@
         </is>
       </c>
       <c r="G319" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H319" t="n">
         <v>2362</v>
@@ -50613,7 +50613,7 @@
         </is>
       </c>
       <c r="G320" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H320" t="n">
         <v>2362</v>
@@ -50654,7 +50654,7 @@
         </is>
       </c>
       <c r="G321" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H321" t="n">
         <v>2362</v>
@@ -50695,7 +50695,7 @@
         </is>
       </c>
       <c r="G322" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H322" t="n">
         <v>2362</v>
@@ -50736,7 +50736,7 @@
         </is>
       </c>
       <c r="G323" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H323" t="n">
         <v>2362</v>
@@ -50777,7 +50777,7 @@
         </is>
       </c>
       <c r="G324" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H324" t="n">
         <v>2362</v>
@@ -50818,7 +50818,7 @@
         </is>
       </c>
       <c r="G325" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H325" t="n">
         <v>2362</v>
@@ -50859,7 +50859,7 @@
         </is>
       </c>
       <c r="G326" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H326" t="n">
         <v>2362</v>
@@ -50900,7 +50900,7 @@
         </is>
       </c>
       <c r="G327" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H327" t="n">
         <v>2362</v>
@@ -50941,7 +50941,7 @@
         </is>
       </c>
       <c r="G328" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H328" t="n">
         <v>2362</v>
@@ -50982,7 +50982,7 @@
         </is>
       </c>
       <c r="G329" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H329" t="n">
         <v>2362</v>
@@ -51023,7 +51023,7 @@
         </is>
       </c>
       <c r="G330" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H330" t="n">
         <v>2362</v>
@@ -51064,7 +51064,7 @@
         </is>
       </c>
       <c r="G331" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H331" t="n">
         <v>2362</v>
@@ -51105,7 +51105,7 @@
         </is>
       </c>
       <c r="G332" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H332" t="n">
         <v>2362</v>
@@ -51146,7 +51146,7 @@
         </is>
       </c>
       <c r="G333" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H333" t="n">
         <v>2362</v>
@@ -51187,7 +51187,7 @@
         </is>
       </c>
       <c r="G334" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H334" t="n">
         <v>2362</v>
@@ -51228,7 +51228,7 @@
         </is>
       </c>
       <c r="G335" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H335" t="n">
         <v>2362</v>
@@ -51269,7 +51269,7 @@
         </is>
       </c>
       <c r="G336" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H336" t="n">
         <v>2362</v>
@@ -51310,7 +51310,7 @@
         </is>
       </c>
       <c r="G337" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H337" t="n">
         <v>2362</v>
@@ -51351,7 +51351,7 @@
         </is>
       </c>
       <c r="G338" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H338" t="n">
         <v>2362</v>
@@ -51392,7 +51392,7 @@
         </is>
       </c>
       <c r="G339" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H339" t="n">
         <v>2362</v>
@@ -51433,7 +51433,7 @@
         </is>
       </c>
       <c r="G340" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H340" t="n">
         <v>2362</v>
@@ -51474,7 +51474,7 @@
         </is>
       </c>
       <c r="G341" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H341" t="n">
         <v>2362</v>
@@ -51515,7 +51515,7 @@
         </is>
       </c>
       <c r="G342" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H342" t="n">
         <v>5906</v>
@@ -51556,7 +51556,7 @@
         </is>
       </c>
       <c r="G343" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H343" t="n">
         <v>5906</v>
@@ -51597,7 +51597,7 @@
         </is>
       </c>
       <c r="G344" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H344" t="n">
         <v>5906</v>
@@ -51638,7 +51638,7 @@
         </is>
       </c>
       <c r="G345" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H345" t="n">
         <v>5906</v>
@@ -51679,7 +51679,7 @@
         </is>
       </c>
       <c r="G346" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H346" t="n">
         <v>5906</v>
@@ -51720,7 +51720,7 @@
         </is>
       </c>
       <c r="G347" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H347" t="n">
         <v>5906</v>
@@ -51761,7 +51761,7 @@
         </is>
       </c>
       <c r="G348" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H348" t="n">
         <v>5906</v>
@@ -51802,7 +51802,7 @@
         </is>
       </c>
       <c r="G349" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H349" t="n">
         <v>5906</v>
@@ -51843,7 +51843,7 @@
         </is>
       </c>
       <c r="G350" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H350" t="n">
         <v>4000</v>
@@ -51884,7 +51884,7 @@
         </is>
       </c>
       <c r="G351" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H351" t="n">
         <v>4000</v>
@@ -51925,7 +51925,7 @@
         </is>
       </c>
       <c r="G352" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H352" t="n">
         <v>4000</v>
@@ -51966,7 +51966,7 @@
         </is>
       </c>
       <c r="G353" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H353" t="n">
         <v>4000</v>
@@ -52007,7 +52007,7 @@
         </is>
       </c>
       <c r="G354" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H354" t="n">
         <v>4000</v>
@@ -52048,7 +52048,7 @@
         </is>
       </c>
       <c r="G355" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H355" t="n">
         <v>4000</v>
@@ -52089,7 +52089,7 @@
         </is>
       </c>
       <c r="G356" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H356" t="n">
         <v>4000</v>
@@ -52130,7 +52130,7 @@
         </is>
       </c>
       <c r="G357" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H357" t="n">
         <v>4000</v>
@@ -52171,7 +52171,7 @@
         </is>
       </c>
       <c r="G358" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H358" t="n">
         <v>4000</v>
@@ -52212,7 +52212,7 @@
         </is>
       </c>
       <c r="G359" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H359" t="n">
         <v>2000</v>
@@ -52253,7 +52253,7 @@
         </is>
       </c>
       <c r="G360" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H360" t="n">
         <v>2000</v>
@@ -52294,7 +52294,7 @@
         </is>
       </c>
       <c r="G361" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H361" t="n">
         <v>2688</v>
@@ -52335,7 +52335,7 @@
         </is>
       </c>
       <c r="G362" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H362" t="n">
         <v>2688</v>
@@ -52376,7 +52376,7 @@
         </is>
       </c>
       <c r="G363" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H363" t="n">
         <v>2084</v>
@@ -52417,7 +52417,7 @@
         </is>
       </c>
       <c r="G364" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H364" t="n">
         <v>2084</v>
@@ -52458,7 +52458,7 @@
         </is>
       </c>
       <c r="G365" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H365" t="n">
         <v>7087</v>
@@ -52499,7 +52499,7 @@
         </is>
       </c>
       <c r="G366" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H366" t="n">
         <v>5906</v>
@@ -52540,7 +52540,7 @@
         </is>
       </c>
       <c r="G367" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H367" t="n">
         <v>5906</v>
@@ -52581,7 +52581,7 @@
         </is>
       </c>
       <c r="G368" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H368" t="n">
         <v>5906</v>
@@ -52622,7 +52622,7 @@
         </is>
       </c>
       <c r="G369" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H369" t="n">
         <v>7087</v>
@@ -52663,7 +52663,7 @@
         </is>
       </c>
       <c r="G370" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H370" t="n">
         <v>5906</v>
@@ -52704,7 +52704,7 @@
         </is>
       </c>
       <c r="G371" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H371" t="n">
         <v>5906</v>
@@ -52745,7 +52745,7 @@
         </is>
       </c>
       <c r="G372" s="10" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="H372" t="n">
         <v>5906</v>
@@ -52786,7 +52786,7 @@
         </is>
       </c>
       <c r="G373" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H373" t="n">
         <v>3543</v>
@@ -52827,7 +52827,7 @@
         </is>
       </c>
       <c r="G374" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H374" t="n">
         <v>3543</v>
@@ -52868,7 +52868,7 @@
         </is>
       </c>
       <c r="G375" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H375" t="n">
         <v>3543</v>
@@ -52909,7 +52909,7 @@
         </is>
       </c>
       <c r="G376" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H376" t="n">
         <v>3543</v>
@@ -52950,7 +52950,7 @@
         </is>
       </c>
       <c r="G377" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H377" t="n">
         <v>3543</v>
@@ -52991,7 +52991,7 @@
         </is>
       </c>
       <c r="G378" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H378" t="n">
         <v>3543</v>
@@ -53032,7 +53032,7 @@
         </is>
       </c>
       <c r="G379" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H379" t="n">
         <v>3543</v>
@@ -53073,7 +53073,7 @@
         </is>
       </c>
       <c r="G380" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H380" t="n">
         <v>3543</v>
@@ -53114,7 +53114,7 @@
         </is>
       </c>
       <c r="G381" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H381" t="n">
         <v>3543</v>
@@ -53155,7 +53155,7 @@
         </is>
       </c>
       <c r="G382" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H382" t="n">
         <v>3543</v>
@@ -53196,7 +53196,7 @@
         </is>
       </c>
       <c r="G383" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H383" t="n">
         <v>3543</v>
@@ -53237,7 +53237,7 @@
         </is>
       </c>
       <c r="G384" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H384" t="n">
         <v>3543</v>
@@ -53278,7 +53278,7 @@
         </is>
       </c>
       <c r="G385" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H385" t="n">
         <v>3543</v>
@@ -53319,7 +53319,7 @@
         </is>
       </c>
       <c r="G386" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H386" t="n">
         <v>3543</v>
@@ -53360,7 +53360,7 @@
         </is>
       </c>
       <c r="G387" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H387" t="n">
         <v>3543</v>
@@ -53401,7 +53401,7 @@
         </is>
       </c>
       <c r="G388" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H388" t="n">
         <v>3543</v>
@@ -53442,7 +53442,7 @@
         </is>
       </c>
       <c r="G389" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H389" t="n">
         <v>3543</v>
@@ -53483,7 +53483,7 @@
         </is>
       </c>
       <c r="G390" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H390" t="n">
         <v>3543</v>
@@ -53524,7 +53524,7 @@
         </is>
       </c>
       <c r="G391" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H391" t="n">
         <v>3543</v>
@@ -53565,7 +53565,7 @@
         </is>
       </c>
       <c r="G392" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H392" t="n">
         <v>3543</v>
@@ -53606,7 +53606,7 @@
         </is>
       </c>
       <c r="G393" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H393" t="n">
         <v>3543</v>
@@ -53647,7 +53647,7 @@
         </is>
       </c>
       <c r="G394" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H394" t="n">
         <v>3543</v>
@@ -53688,7 +53688,7 @@
         </is>
       </c>
       <c r="G395" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H395" t="n">
         <v>3543</v>
@@ -53729,7 +53729,7 @@
         </is>
       </c>
       <c r="G396" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H396" t="n">
         <v>3543</v>
@@ -53770,7 +53770,7 @@
         </is>
       </c>
       <c r="G397" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H397" t="n">
         <v>3543</v>
@@ -53811,7 +53811,7 @@
         </is>
       </c>
       <c r="G398" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H398" t="n">
         <v>3543</v>
@@ -53852,7 +53852,7 @@
         </is>
       </c>
       <c r="G399" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H399" t="n">
         <v>3543</v>
@@ -53893,7 +53893,7 @@
         </is>
       </c>
       <c r="G400" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H400" t="n">
         <v>3543</v>
@@ -53934,7 +53934,7 @@
         </is>
       </c>
       <c r="G401" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H401" t="n">
         <v>3543</v>
@@ -53975,7 +53975,7 @@
         </is>
       </c>
       <c r="G402" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H402" t="n">
         <v>3543</v>
@@ -54016,7 +54016,7 @@
         </is>
       </c>
       <c r="G403" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H403" t="n">
         <v>3543</v>
@@ -54057,7 +54057,7 @@
         </is>
       </c>
       <c r="G404" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H404" t="n">
         <v>3543</v>
@@ -54098,7 +54098,7 @@
         </is>
       </c>
       <c r="G405" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H405" t="n">
         <v>3543</v>
@@ -54139,7 +54139,7 @@
         </is>
       </c>
       <c r="G406" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H406" t="n">
         <v>3543</v>
@@ -54180,7 +54180,7 @@
         </is>
       </c>
       <c r="G407" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H407" t="n">
         <v>3543</v>
@@ -54221,7 +54221,7 @@
         </is>
       </c>
       <c r="G408" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H408" t="n">
         <v>3543</v>
@@ -54262,7 +54262,7 @@
         </is>
       </c>
       <c r="G409" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H409" t="n">
         <v>3543</v>
@@ -54303,7 +54303,7 @@
         </is>
       </c>
       <c r="G410" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H410" t="n">
         <v>3543</v>
@@ -54344,7 +54344,7 @@
         </is>
       </c>
       <c r="G411" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H411" t="n">
         <v>3543</v>
@@ -54385,7 +54385,7 @@
         </is>
       </c>
       <c r="G412" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H412" t="n">
         <v>3543</v>
@@ -54426,7 +54426,7 @@
         </is>
       </c>
       <c r="G413" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H413" t="n">
         <v>3543</v>
@@ -54467,7 +54467,7 @@
         </is>
       </c>
       <c r="G414" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H414" t="n">
         <v>3543</v>
@@ -54508,7 +54508,7 @@
         </is>
       </c>
       <c r="G415" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H415" t="n">
         <v>3543</v>
@@ -54549,7 +54549,7 @@
         </is>
       </c>
       <c r="G416" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H416" t="n">
         <v>3543</v>
@@ -54590,7 +54590,7 @@
         </is>
       </c>
       <c r="G417" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H417" t="n">
         <v>3543</v>
@@ -54631,7 +54631,7 @@
         </is>
       </c>
       <c r="G418" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H418" t="n">
         <v>3543</v>
@@ -54672,7 +54672,7 @@
         </is>
       </c>
       <c r="G419" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H419" t="n">
         <v>3543</v>
@@ -54713,7 +54713,7 @@
         </is>
       </c>
       <c r="G420" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H420" t="n">
         <v>3543</v>
@@ -54754,7 +54754,7 @@
         </is>
       </c>
       <c r="G421" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H421" t="n">
         <v>3543</v>
@@ -54795,7 +54795,7 @@
         </is>
       </c>
       <c r="G422" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H422" t="n">
         <v>3543</v>
@@ -54836,7 +54836,7 @@
         </is>
       </c>
       <c r="G423" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H423" t="n">
         <v>3543</v>
@@ -54877,7 +54877,7 @@
         </is>
       </c>
       <c r="G424" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H424" t="n">
         <v>3543</v>
@@ -54918,7 +54918,7 @@
         </is>
       </c>
       <c r="G425" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H425" t="n">
         <v>3543</v>
@@ -54959,7 +54959,7 @@
         </is>
       </c>
       <c r="G426" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H426" t="n">
         <v>3543</v>
@@ -55000,7 +55000,7 @@
         </is>
       </c>
       <c r="G427" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H427" t="n">
         <v>3543</v>
@@ -55041,7 +55041,7 @@
         </is>
       </c>
       <c r="G428" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H428" t="n">
         <v>3543</v>
@@ -55082,7 +55082,7 @@
         </is>
       </c>
       <c r="G429" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H429" t="n">
         <v>3543</v>
@@ -55123,7 +55123,7 @@
         </is>
       </c>
       <c r="G430" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H430" t="n">
         <v>3543</v>
@@ -55164,7 +55164,7 @@
         </is>
       </c>
       <c r="G431" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H431" t="n">
         <v>3543</v>
@@ -55205,7 +55205,7 @@
         </is>
       </c>
       <c r="G432" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H432" t="n">
         <v>3543</v>
@@ -55246,7 +55246,7 @@
         </is>
       </c>
       <c r="G433" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H433" t="n">
         <v>3543</v>
@@ -55287,7 +55287,7 @@
         </is>
       </c>
       <c r="G434" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H434" t="n">
         <v>3543</v>
@@ -55328,7 +55328,7 @@
         </is>
       </c>
       <c r="G435" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H435" t="n">
         <v>3543</v>
@@ -55369,7 +55369,7 @@
         </is>
       </c>
       <c r="G436" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H436" t="n">
         <v>3543</v>
@@ -55410,7 +55410,7 @@
         </is>
       </c>
       <c r="G437" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H437" t="n">
         <v>3543</v>
@@ -55451,7 +55451,7 @@
         </is>
       </c>
       <c r="G438" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H438" t="n">
         <v>3543</v>
@@ -55492,7 +55492,7 @@
         </is>
       </c>
       <c r="G439" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H439" t="n">
         <v>3543</v>
@@ -55533,7 +55533,7 @@
         </is>
       </c>
       <c r="G440" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H440" t="n">
         <v>3543</v>
@@ -55574,7 +55574,7 @@
         </is>
       </c>
       <c r="G441" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H441" t="n">
         <v>3543</v>
@@ -55615,7 +55615,7 @@
         </is>
       </c>
       <c r="G442" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H442" t="n">
         <v>3543</v>
@@ -55656,7 +55656,7 @@
         </is>
       </c>
       <c r="G443" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H443" t="n">
         <v>3543</v>
@@ -55697,7 +55697,7 @@
         </is>
       </c>
       <c r="G444" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H444" t="n">
         <v>3543</v>
@@ -55738,7 +55738,7 @@
         </is>
       </c>
       <c r="G445" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H445" t="n">
         <v>3543</v>
@@ -55779,7 +55779,7 @@
         </is>
       </c>
       <c r="G446" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H446" t="n">
         <v>3543</v>
@@ -55820,7 +55820,7 @@
         </is>
       </c>
       <c r="G447" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H447" t="n">
         <v>3543</v>
@@ -55861,7 +55861,7 @@
         </is>
       </c>
       <c r="G448" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H448" t="n">
         <v>2000</v>
@@ -55902,7 +55902,7 @@
         </is>
       </c>
       <c r="G449" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H449" t="n">
         <v>2000</v>
@@ -55943,7 +55943,7 @@
         </is>
       </c>
       <c r="G450" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H450" t="n">
         <v>2000</v>
@@ -55984,7 +55984,7 @@
         </is>
       </c>
       <c r="G451" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H451" t="n">
         <v>2000</v>
@@ -56025,7 +56025,7 @@
         </is>
       </c>
       <c r="G452" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H452" t="n">
         <v>2000</v>
@@ -56066,7 +56066,7 @@
         </is>
       </c>
       <c r="G453" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H453" t="n">
         <v>2000</v>
@@ -56107,7 +56107,7 @@
         </is>
       </c>
       <c r="G454" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H454" t="n">
         <v>2000</v>
@@ -56148,7 +56148,7 @@
         </is>
       </c>
       <c r="G455" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H455" t="n">
         <v>2000</v>
@@ -56189,7 +56189,7 @@
         </is>
       </c>
       <c r="G456" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H456" t="n">
         <v>2000</v>
@@ -56230,7 +56230,7 @@
         </is>
       </c>
       <c r="G457" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H457" t="n">
         <v>2000</v>
@@ -56271,7 +56271,7 @@
         </is>
       </c>
       <c r="G458" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H458" t="n">
         <v>2000</v>
@@ -56312,7 +56312,7 @@
         </is>
       </c>
       <c r="G459" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H459" t="n">
         <v>2000</v>
@@ -56353,7 +56353,7 @@
         </is>
       </c>
       <c r="G460" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H460" t="n">
         <v>3316</v>
@@ -56394,7 +56394,7 @@
         </is>
       </c>
       <c r="G461" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H461" t="n">
         <v>3316</v>
@@ -56435,7 +56435,7 @@
         </is>
       </c>
       <c r="G462" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H462" t="n">
         <v>2785</v>
@@ -56476,7 +56476,7 @@
         </is>
       </c>
       <c r="G463" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H463" t="n">
         <v>2785</v>
@@ -56517,7 +56517,7 @@
         </is>
       </c>
       <c r="G464" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H464" t="n">
         <v>4032</v>
@@ -56558,7 +56558,7 @@
         </is>
       </c>
       <c r="G465" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H465" t="n">
         <v>4032</v>
@@ -56599,7 +56599,7 @@
         </is>
       </c>
       <c r="G466" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H466" t="n">
         <v>3047</v>
@@ -56640,7 +56640,7 @@
         </is>
       </c>
       <c r="G467" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H467" t="n">
         <v>4032</v>
@@ -56681,7 +56681,7 @@
         </is>
       </c>
       <c r="G468" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H468" t="n">
         <v>4032</v>
@@ -56722,7 +56722,7 @@
         </is>
       </c>
       <c r="G469" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H469" t="n">
         <v>3661</v>
@@ -56763,7 +56763,7 @@
         </is>
       </c>
       <c r="G470" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H470" t="n">
         <v>3607</v>
@@ -56804,7 +56804,7 @@
         </is>
       </c>
       <c r="G471" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H471" t="n">
         <v>4028</v>
@@ -56845,7 +56845,7 @@
         </is>
       </c>
       <c r="G472" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H472" t="n">
         <v>4028</v>
@@ -56886,7 +56886,7 @@
         </is>
       </c>
       <c r="G473" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H473" t="n">
         <v>4028</v>
@@ -56927,7 +56927,7 @@
         </is>
       </c>
       <c r="G474" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H474" t="n">
         <v>4028</v>
@@ -56968,7 +56968,7 @@
         </is>
       </c>
       <c r="G475" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H475" t="n">
         <v>4028</v>
@@ -57009,7 +57009,7 @@
         </is>
       </c>
       <c r="G476" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H476" t="n">
         <v>4028</v>
@@ -57050,7 +57050,7 @@
         </is>
       </c>
       <c r="G477" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H477" t="n">
         <v>4028</v>
@@ -57091,7 +57091,7 @@
         </is>
       </c>
       <c r="G478" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H478" t="n">
         <v>3895</v>
@@ -57132,7 +57132,7 @@
         </is>
       </c>
       <c r="G479" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H479" t="n">
         <v>2784</v>
@@ -57173,7 +57173,7 @@
         </is>
       </c>
       <c r="G480" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="H480" t="n">
         <v>4028</v>
@@ -57214,7 +57214,7 @@
         </is>
       </c>
       <c r="G481" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H481" t="n">
         <v>2138</v>
@@ -57255,7 +57255,7 @@
         </is>
       </c>
       <c r="G482" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H482" t="n">
         <v>4038</v>
@@ -57296,7 +57296,7 @@
         </is>
       </c>
       <c r="G483" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H483" t="n">
         <v>4038</v>
@@ -57337,7 +57337,7 @@
         </is>
       </c>
       <c r="G484" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H484" t="n">
         <v>4038</v>
@@ -57378,7 +57378,7 @@
         </is>
       </c>
       <c r="G485" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H485" t="n">
         <v>4038</v>
@@ -57419,7 +57419,7 @@
         </is>
       </c>
       <c r="G486" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H486" t="n">
         <v>4038</v>
@@ -57460,7 +57460,7 @@
         </is>
       </c>
       <c r="G487" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H487" t="n">
         <v>4038</v>
@@ -57501,7 +57501,7 @@
         </is>
       </c>
       <c r="G488" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H488" t="n">
         <v>4038</v>
@@ -57542,7 +57542,7 @@
         </is>
       </c>
       <c r="G489" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H489" t="n">
         <v>4038</v>
@@ -57583,7 +57583,7 @@
         </is>
       </c>
       <c r="G490" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H490" t="n">
         <v>4038</v>
@@ -57624,7 +57624,7 @@
         </is>
       </c>
       <c r="G491" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H491" t="n">
         <v>5712</v>
@@ -57665,7 +57665,7 @@
         </is>
       </c>
       <c r="G492" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H492" t="n">
         <v>2472</v>
@@ -57706,7 +57706,7 @@
         </is>
       </c>
       <c r="G493" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H493" t="n">
         <v>2472</v>
@@ -57747,7 +57747,7 @@
         </is>
       </c>
       <c r="G494" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H494" t="n">
         <v>2472</v>
@@ -57788,7 +57788,7 @@
         </is>
       </c>
       <c r="G495" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H495" t="n">
         <v>2472</v>
@@ -57829,7 +57829,7 @@
         </is>
       </c>
       <c r="G496" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H496" t="n">
         <v>2472</v>
@@ -57870,7 +57870,7 @@
         </is>
       </c>
       <c r="G497" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H497" t="n">
         <v>5192</v>
@@ -57911,7 +57911,7 @@
         </is>
       </c>
       <c r="G498" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H498" t="n">
         <v>6525</v>
@@ -57952,7 +57952,7 @@
         </is>
       </c>
       <c r="G499" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H499" t="n">
         <v>2000</v>
@@ -57993,7 +57993,7 @@
         </is>
       </c>
       <c r="G500" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H500" t="n">
         <v>4179</v>
@@ -58034,7 +58034,7 @@
         </is>
       </c>
       <c r="G501" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H501" t="n">
         <v>5983</v>
@@ -58075,7 +58075,7 @@
         </is>
       </c>
       <c r="G502" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H502" t="n">
         <v>2242</v>
@@ -58116,7 +58116,7 @@
         </is>
       </c>
       <c r="G503" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H503" t="n">
         <v>3240</v>
@@ -58157,7 +58157,7 @@
         </is>
       </c>
       <c r="G504" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H504" t="n">
         <v>2869</v>
@@ -58198,7 +58198,7 @@
         </is>
       </c>
       <c r="G505" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H505" t="n">
         <v>2750</v>
@@ -58239,7 +58239,7 @@
         </is>
       </c>
       <c r="G506" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H506" t="n">
         <v>2665</v>
@@ -58280,7 +58280,7 @@
         </is>
       </c>
       <c r="G507" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H507" t="n">
         <v>2971</v>
@@ -58321,7 +58321,7 @@
         </is>
       </c>
       <c r="G508" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H508" t="n">
         <v>2979</v>
@@ -58362,7 +58362,7 @@
         </is>
       </c>
       <c r="G509" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H509" t="n">
         <v>2896</v>
@@ -58403,7 +58403,7 @@
         </is>
       </c>
       <c r="G510" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H510" t="n">
         <v>3015</v>
@@ -58444,7 +58444,7 @@
         </is>
       </c>
       <c r="G511" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H511" t="n">
         <v>1985</v>
@@ -58485,7 +58485,7 @@
         </is>
       </c>
       <c r="G512" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H512" t="n">
         <v>1859</v>
@@ -58526,7 +58526,7 @@
         </is>
       </c>
       <c r="G513" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H513" t="n">
         <v>3566</v>
@@ -58567,7 +58567,7 @@
         </is>
       </c>
       <c r="G514" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H514" t="n">
         <v>3566</v>
@@ -58608,7 +58608,7 @@
         </is>
       </c>
       <c r="G515" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H515" t="n">
         <v>3566</v>
@@ -58649,7 +58649,7 @@
         </is>
       </c>
       <c r="G516" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H516" t="n">
         <v>3566</v>
@@ -58690,7 +58690,7 @@
         </is>
       </c>
       <c r="G517" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H517" t="n">
         <v>3566</v>
@@ -58731,7 +58731,7 @@
         </is>
       </c>
       <c r="G518" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H518" t="n">
         <v>3566</v>
@@ -58772,7 +58772,7 @@
         </is>
       </c>
       <c r="G519" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H519" t="n">
         <v>3566</v>
@@ -58813,7 +58813,7 @@
         </is>
       </c>
       <c r="G520" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H520" t="n">
         <v>3566</v>
@@ -58854,7 +58854,7 @@
         </is>
       </c>
       <c r="G521" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H521" t="n">
         <v>3566</v>
@@ -58895,7 +58895,7 @@
         </is>
       </c>
       <c r="G522" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H522" t="n">
         <v>3566</v>
@@ -58936,7 +58936,7 @@
         </is>
       </c>
       <c r="G523" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H523" t="n">
         <v>3566</v>
@@ -58977,7 +58977,7 @@
         </is>
       </c>
       <c r="G524" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H524" t="n">
         <v>3566</v>
@@ -59018,7 +59018,7 @@
         </is>
       </c>
       <c r="G525" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H525" t="n">
         <v>3566</v>
@@ -59059,7 +59059,7 @@
         </is>
       </c>
       <c r="G526" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H526" t="n">
         <v>3566</v>
@@ -59100,7 +59100,7 @@
         </is>
       </c>
       <c r="G527" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H527" t="n">
         <v>3566</v>
@@ -59141,7 +59141,7 @@
         </is>
       </c>
       <c r="G528" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H528" t="n">
         <v>3566</v>
@@ -59182,7 +59182,7 @@
         </is>
       </c>
       <c r="G529" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H529" t="n">
         <v>3566</v>
@@ -59223,7 +59223,7 @@
         </is>
       </c>
       <c r="G530" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H530" t="n">
         <v>1828</v>
@@ -59264,7 +59264,7 @@
         </is>
       </c>
       <c r="G531" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="H531" t="n">
         <v>2480</v>

</xml_diff>

<commit_message>
republished works details .md + path fixes
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20580" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Works'!$A$1:$Y$550</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -1375,8 +1375,8 @@
     <col width="15.1640625" customWidth="1" style="7" min="23" max="23"/>
     <col width="21.5" customWidth="1" style="7" min="24" max="24"/>
     <col width="26.83203125" customWidth="1" style="7" min="25" max="25"/>
-    <col width="10.83203125" customWidth="1" style="7" min="27" max="64"/>
-    <col width="10.83203125" customWidth="1" style="7" min="65" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="7" min="27" max="66"/>
+    <col width="10.83203125" customWidth="1" style="7" min="67" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="6">
@@ -28216,7 +28216,7 @@
       </c>
       <c r="B429" s="7" t="inlineStr">
         <is>
-          <t>published</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="C429" s="24" t="n">
@@ -28224,12 +28224,12 @@
       </c>
       <c r="D429" s="7" t="inlineStr">
         <is>
-          <t>molecules</t>
+          <t>molecule-forms</t>
         </is>
       </c>
       <c r="E429" s="7" t="inlineStr">
         <is>
-          <t>molecules</t>
+          <t>molecule forms</t>
         </is>
       </c>
       <c r="F429" s="7" t="inlineStr">
@@ -36392,7 +36392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
     <col width="31.83203125" customWidth="1" style="1" min="1" max="1"/>
@@ -36403,8 +36403,8 @@
     <col width="21" bestFit="1" customWidth="1" style="7" min="6" max="6"/>
     <col width="21" customWidth="1" style="7" min="7" max="7"/>
     <col width="51" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
-    <col width="10.83203125" customWidth="1" style="1" min="9" max="47"/>
-    <col width="10.83203125" customWidth="1" style="1" min="48" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="1" min="9" max="49"/>
+    <col width="10.83203125" customWidth="1" style="1" min="50" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="3">
@@ -37203,12 +37203,12 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>molecules</t>
+          <t>molecule-forms</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>molecules</t>
+          <t>molecule forms</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
@@ -37225,66 +37225,59 @@
       <c r="F30" s="7" t="n">
         <v>2013</v>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>molecules</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>molecules</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>46086</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>2013</v>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>00460</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>monoprints-residues</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>monoprints and residues</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>mouse-story</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t>mouse story</t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="n">
-        <v>46086</v>
-      </c>
-      <c r="E32" s="1" t="n">
-        <v>1993</v>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>1991-93</t>
-        </is>
-      </c>
-      <c r="G32" s="16" t="inlineStr">
-        <is>
-          <t>00160</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>nerve</t>
+          <t>mouse-story</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>nerve</t>
+          <t>mouse story</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
@@ -37296,165 +37289,198 @@
         <v>46086</v>
       </c>
       <c r="E33" s="1" t="n">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>1990-95</t>
-        </is>
-      </c>
-      <c r="H33" s="1" t="inlineStr">
-        <is>
-          <t>works and details to publish</t>
+          <t>1991-93</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>00160</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>nerve-forms</t>
+          <t>nerve</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>nerve forms</t>
-        </is>
+          <t>nerve</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>46086</v>
       </c>
       <c r="E34" s="1" t="n">
-        <v>2004</v>
-      </c>
-      <c r="F34" s="7" t="n">
-        <v>2004</v>
+        <v>1995</v>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>1990-95</t>
+        </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>add remaining works and series text</t>
+          <t>works and details to publish</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>particle-theory</t>
+          <t>nerve-forms</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>particle theory</t>
+          <t>nerve forms</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>2004</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>2004</v>
+      </c>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>add remaining works and series text</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>qrnt</t>
+          <t>particle-theory</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>quantum random number theory</t>
-        </is>
-      </c>
-      <c r="E36" s="1" t="n">
-        <v>2015</v>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>2009, 2015</t>
+          <t>particle theory</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>qrnt</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>r</t>
-        </is>
-      </c>
-      <c r="C37" s="1" t="inlineStr">
-        <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="n">
-        <v>46086</v>
+          <t>quantum random number theory</t>
+        </is>
       </c>
       <c r="E37" s="1" t="n">
-        <v>2001</v>
-      </c>
-      <c r="F37" s="7" t="n">
-        <v>2001</v>
-      </c>
-      <c r="G37" s="16" t="inlineStr">
-        <is>
-          <t>00142</t>
+        <v>2015</v>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>2009, 2015</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>spiders</t>
+          <t>r</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>spiders</t>
-        </is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>46086</v>
       </c>
       <c r="E38" s="1" t="n">
-        <v>2006</v>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>2006, 2015</t>
+        <v>2001</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>2001</v>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>00142</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>string-theory</t>
+          <t>spiders</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>string theory</t>
+          <t>spiders</t>
         </is>
       </c>
       <c r="E39" s="1" t="n">
-        <v>2012</v>
+        <v>2006</v>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>2005-12</t>
-        </is>
-      </c>
-      <c r="G39" s="16" t="inlineStr">
-        <is>
-          <t>00573</t>
+          <t>2006, 2015</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
+          <t>string-theory</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>string theory</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>2005-12</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>00573</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
           <t>wa</t>
         </is>
       </c>
-      <c r="B40" s="1" t="inlineStr">
+      <c r="B41" s="1" t="inlineStr">
         <is>
           <t>wa</t>
         </is>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="E41" s="1" t="n">
         <v>2008</v>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>2008, 2011</t>
         </is>
@@ -51829,12 +51855,12 @@
       </c>
       <c r="D350" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 1 - detail 1.jpg</t>
+          <t>forest 1 - detail 1.jpg</t>
         </is>
       </c>
       <c r="E350" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 1 - detail 1</t>
+          <t>forest 1 - detail 1</t>
         </is>
       </c>
       <c r="F350" s="1" t="inlineStr">
@@ -51870,12 +51896,12 @@
       </c>
       <c r="D351" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 1 - detail 2.jpg</t>
+          <t>forest 1 - detail 2.jpg</t>
         </is>
       </c>
       <c r="E351" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 1 - detail 2</t>
+          <t>forest 1 - detail 2</t>
         </is>
       </c>
       <c r="F351" s="1" t="inlineStr">
@@ -51911,12 +51937,12 @@
       </c>
       <c r="D352" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 1 - detail 3.jpg</t>
+          <t>forest 1 - detail 3.jpg</t>
         </is>
       </c>
       <c r="E352" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 1 - detail 3</t>
+          <t>forest 1 - detail 3</t>
         </is>
       </c>
       <c r="F352" s="1" t="inlineStr">
@@ -51952,12 +51978,12 @@
       </c>
       <c r="D353" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 2 - detail 1.jpg</t>
+          <t>forest 2 - detail 1.jpg</t>
         </is>
       </c>
       <c r="E353" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 2 - detail 1</t>
+          <t>forest 2 - detail 1</t>
         </is>
       </c>
       <c r="F353" s="1" t="inlineStr">
@@ -51993,12 +52019,12 @@
       </c>
       <c r="D354" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 2 - detail 2.jpg</t>
+          <t>forest 2 - detail 2.jpg</t>
         </is>
       </c>
       <c r="E354" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 2 - detail 2</t>
+          <t>forest 2 - detail 2</t>
         </is>
       </c>
       <c r="F354" s="1" t="inlineStr">
@@ -52034,12 +52060,12 @@
       </c>
       <c r="D355" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 2 - detail 3.jpg</t>
+          <t>forest 2 - detail 3.jpg</t>
         </is>
       </c>
       <c r="E355" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 2 - detail 3</t>
+          <t>forest 2 - detail 3</t>
         </is>
       </c>
       <c r="F355" s="1" t="inlineStr">
@@ -52075,12 +52101,12 @@
       </c>
       <c r="D356" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 3 - detail 1.jpg</t>
+          <t>forest 3 - detail 1.jpg</t>
         </is>
       </c>
       <c r="E356" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 3 - detail 1</t>
+          <t>forest 3 - detail 1</t>
         </is>
       </c>
       <c r="F356" s="1" t="inlineStr">
@@ -52116,12 +52142,12 @@
       </c>
       <c r="D357" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 3 - detail 2.jpg</t>
+          <t>forest 3 - detail 2.jpg</t>
         </is>
       </c>
       <c r="E357" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 3 - detail 2</t>
+          <t>forest 3 - detail 2</t>
         </is>
       </c>
       <c r="F357" s="1" t="inlineStr">
@@ -52157,12 +52183,12 @@
       </c>
       <c r="D358" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 3 - detail 3.jpg</t>
+          <t>forest 3 - detail 3.jpg</t>
         </is>
       </c>
       <c r="E358" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 3 - detail 3</t>
+          <t>forest 3 - detail 3</t>
         </is>
       </c>
       <c r="F358" s="1" t="inlineStr">
@@ -52198,12 +52224,12 @@
       </c>
       <c r="D359" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 1.jpg</t>
+          <t>forest 4 - detail 1.jpg</t>
         </is>
       </c>
       <c r="E359" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 1</t>
+          <t>forest 4 - detail 1</t>
         </is>
       </c>
       <c r="F359" s="1" t="inlineStr">
@@ -52239,12 +52265,12 @@
       </c>
       <c r="D360" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 2.jpg</t>
+          <t>forest 4 - detail 2.jpg</t>
         </is>
       </c>
       <c r="E360" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 2</t>
+          <t>forest 4 - detail 2</t>
         </is>
       </c>
       <c r="F360" s="1" t="inlineStr">
@@ -52280,12 +52306,12 @@
       </c>
       <c r="D361" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 3.jpg</t>
+          <t>forest 4 - detail 3.jpg</t>
         </is>
       </c>
       <c r="E361" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 3</t>
+          <t>forest 4 - detail 3</t>
         </is>
       </c>
       <c r="F361" s="1" t="inlineStr">
@@ -52321,12 +52347,12 @@
       </c>
       <c r="D362" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 4.jpg</t>
+          <t>forest 4 - detail 4.jpg</t>
         </is>
       </c>
       <c r="E362" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 4</t>
+          <t>forest 4 - detail 4</t>
         </is>
       </c>
       <c r="F362" s="1" t="inlineStr">
@@ -52362,12 +52388,12 @@
       </c>
       <c r="D363" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 5.jpg</t>
+          <t>forest 4 - detail 5.jpg</t>
         </is>
       </c>
       <c r="E363" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 5</t>
+          <t>forest 4 - detail 5</t>
         </is>
       </c>
       <c r="F363" s="1" t="inlineStr">
@@ -52403,12 +52429,12 @@
       </c>
       <c r="D364" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 6.jpg</t>
+          <t>forest 4 - detail 6.jpg</t>
         </is>
       </c>
       <c r="E364" s="1" t="inlineStr">
         <is>
-          <t>forests (2023) - forest 4 - detail 6</t>
+          <t>forest 4 - detail 6</t>
         </is>
       </c>
       <c r="F364" s="1" t="inlineStr">
@@ -59298,8 +59324,8 @@
     <col width="11.33203125" bestFit="1" customWidth="1" style="13" min="9" max="9"/>
     <col width="12.1640625" bestFit="1" customWidth="1" style="13" min="10" max="10"/>
     <col width="33.6640625" customWidth="1" style="13" min="11" max="11"/>
-    <col width="10.83203125" customWidth="1" style="13" min="12" max="41"/>
-    <col width="10.83203125" customWidth="1" style="13" min="42" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="13" min="12" max="43"/>
+    <col width="10.83203125" customWidth="1" style="13" min="44" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
json-first: make _works/_work_details lightweight and render work pages from work JSON
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="C2" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
         </is>
       </c>
       <c r="C9" s="24" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
@@ -2078,7 +2078,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
@@ -2202,7 +2202,7 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
@@ -2386,7 +2386,7 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
         </is>
       </c>
       <c r="C18" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
@@ -2626,7 +2626,7 @@
         </is>
       </c>
       <c r="C20" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="C21" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="C22" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="C23" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
@@ -2868,7 +2868,7 @@
         </is>
       </c>
       <c r="C24" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
@@ -2992,7 +2992,7 @@
         </is>
       </c>
       <c r="C26" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="C27" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
@@ -3116,7 +3116,7 @@
         </is>
       </c>
       <c r="C28" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
@@ -3178,7 +3178,7 @@
         </is>
       </c>
       <c r="C29" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
@@ -3240,7 +3240,7 @@
         </is>
       </c>
       <c r="C30" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="C31" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
@@ -3364,7 +3364,7 @@
         </is>
       </c>
       <c r="C32" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
@@ -3426,7 +3426,7 @@
         </is>
       </c>
       <c r="C33" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
@@ -3488,7 +3488,7 @@
         </is>
       </c>
       <c r="C34" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
@@ -3550,7 +3550,7 @@
         </is>
       </c>
       <c r="C35" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="C36" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
@@ -3674,7 +3674,7 @@
         </is>
       </c>
       <c r="C37" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C38" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
         </is>
       </c>
       <c r="C39" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="C40" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="C41" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
@@ -3984,7 +3984,7 @@
         </is>
       </c>
       <c r="C42" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         </is>
       </c>
       <c r="C43" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="C44" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
@@ -4170,7 +4170,7 @@
         </is>
       </c>
       <c r="C45" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
@@ -4232,7 +4232,7 @@
         </is>
       </c>
       <c r="C46" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
@@ -4294,7 +4294,7 @@
         </is>
       </c>
       <c r="C47" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
@@ -4356,7 +4356,7 @@
         </is>
       </c>
       <c r="C48" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
@@ -4418,7 +4418,7 @@
         </is>
       </c>
       <c r="C49" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
@@ -4480,7 +4480,7 @@
         </is>
       </c>
       <c r="C50" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
@@ -4542,7 +4542,7 @@
         </is>
       </c>
       <c r="C51" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
@@ -4604,7 +4604,7 @@
         </is>
       </c>
       <c r="C52" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
@@ -4666,7 +4666,7 @@
         </is>
       </c>
       <c r="C53" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
@@ -4728,7 +4728,7 @@
         </is>
       </c>
       <c r="C54" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
@@ -4790,7 +4790,7 @@
         </is>
       </c>
       <c r="C55" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="C56" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
@@ -4914,7 +4914,7 @@
         </is>
       </c>
       <c r="C57" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
@@ -4976,7 +4976,7 @@
         </is>
       </c>
       <c r="C58" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
         </is>
       </c>
       <c r="C59" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
@@ -5100,7 +5100,7 @@
         </is>
       </c>
       <c r="C60" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="C61" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
@@ -5224,7 +5224,7 @@
         </is>
       </c>
       <c r="C62" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
@@ -5286,7 +5286,7 @@
         </is>
       </c>
       <c r="C63" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
         </is>
       </c>
       <c r="C64" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
@@ -5410,7 +5410,7 @@
         </is>
       </c>
       <c r="C65" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
@@ -5472,7 +5472,7 @@
         </is>
       </c>
       <c r="C66" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C67" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
@@ -5596,7 +5596,7 @@
         </is>
       </c>
       <c r="C68" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
         </is>
       </c>
       <c r="C69" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
@@ -5720,7 +5720,7 @@
         </is>
       </c>
       <c r="C70" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
@@ -5782,7 +5782,7 @@
         </is>
       </c>
       <c r="C71" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
@@ -5844,7 +5844,7 @@
         </is>
       </c>
       <c r="C72" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
@@ -5906,7 +5906,7 @@
         </is>
       </c>
       <c r="C73" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
@@ -5968,7 +5968,7 @@
         </is>
       </c>
       <c r="C74" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
@@ -6030,7 +6030,7 @@
         </is>
       </c>
       <c r="C75" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
@@ -6092,7 +6092,7 @@
         </is>
       </c>
       <c r="C76" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         </is>
       </c>
       <c r="C77" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
@@ -6216,7 +6216,7 @@
         </is>
       </c>
       <c r="C78" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
@@ -6278,7 +6278,7 @@
         </is>
       </c>
       <c r="C79" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="C80" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
@@ -6402,7 +6402,7 @@
         </is>
       </c>
       <c r="C81" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
         </is>
       </c>
       <c r="C82" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
@@ -6526,7 +6526,7 @@
         </is>
       </c>
       <c r="C83" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
@@ -6588,7 +6588,7 @@
         </is>
       </c>
       <c r="C84" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
@@ -6650,7 +6650,7 @@
         </is>
       </c>
       <c r="C85" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="C86" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
@@ -6774,7 +6774,7 @@
         </is>
       </c>
       <c r="C87" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
@@ -6836,7 +6836,7 @@
         </is>
       </c>
       <c r="C88" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         </is>
       </c>
       <c r="C89" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
@@ -6960,7 +6960,7 @@
         </is>
       </c>
       <c r="C90" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
@@ -7022,7 +7022,7 @@
         </is>
       </c>
       <c r="C91" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
@@ -7084,7 +7084,7 @@
         </is>
       </c>
       <c r="C92" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
@@ -7146,7 +7146,7 @@
         </is>
       </c>
       <c r="C93" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
@@ -7208,7 +7208,7 @@
         </is>
       </c>
       <c r="C94" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
@@ -7270,7 +7270,7 @@
         </is>
       </c>
       <c r="C95" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
@@ -7332,7 +7332,7 @@
         </is>
       </c>
       <c r="C96" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="C97" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
@@ -7456,7 +7456,7 @@
         </is>
       </c>
       <c r="C98" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
@@ -7518,7 +7518,7 @@
         </is>
       </c>
       <c r="C99" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
         </is>
       </c>
       <c r="C100" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
@@ -7642,7 +7642,7 @@
         </is>
       </c>
       <c r="C101" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
@@ -7704,7 +7704,7 @@
         </is>
       </c>
       <c r="C102" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
@@ -7766,7 +7766,7 @@
         </is>
       </c>
       <c r="C103" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
@@ -7828,7 +7828,7 @@
         </is>
       </c>
       <c r="C104" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="C105" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
@@ -7952,7 +7952,7 @@
         </is>
       </c>
       <c r="C106" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
@@ -8014,7 +8014,7 @@
         </is>
       </c>
       <c r="C107" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
@@ -8076,7 +8076,7 @@
         </is>
       </c>
       <c r="C108" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
@@ -8138,7 +8138,7 @@
         </is>
       </c>
       <c r="C109" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
@@ -8200,7 +8200,7 @@
         </is>
       </c>
       <c r="C110" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="C111" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
@@ -8324,7 +8324,7 @@
         </is>
       </c>
       <c r="C112" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
@@ -8384,7 +8384,7 @@
         </is>
       </c>
       <c r="C113" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
@@ -8446,7 +8446,7 @@
         </is>
       </c>
       <c r="C114" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
         </is>
       </c>
       <c r="C115" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
@@ -8575,7 +8575,7 @@
         </is>
       </c>
       <c r="C116" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
@@ -8642,7 +8642,7 @@
         </is>
       </c>
       <c r="C117" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
@@ -8709,7 +8709,7 @@
         </is>
       </c>
       <c r="C118" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
@@ -8776,7 +8776,7 @@
         </is>
       </c>
       <c r="C119" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
@@ -8843,7 +8843,7 @@
         </is>
       </c>
       <c r="C120" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
@@ -8910,7 +8910,7 @@
         </is>
       </c>
       <c r="C121" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
@@ -8977,7 +8977,7 @@
         </is>
       </c>
       <c r="C122" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
@@ -9044,7 +9044,7 @@
         </is>
       </c>
       <c r="C123" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
@@ -9111,7 +9111,7 @@
         </is>
       </c>
       <c r="C124" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
@@ -9178,7 +9178,7 @@
         </is>
       </c>
       <c r="C125" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
@@ -9245,7 +9245,7 @@
         </is>
       </c>
       <c r="C126" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
@@ -9312,7 +9312,7 @@
         </is>
       </c>
       <c r="C127" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
@@ -9379,7 +9379,7 @@
         </is>
       </c>
       <c r="C128" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
@@ -9446,7 +9446,7 @@
         </is>
       </c>
       <c r="C129" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
@@ -9513,7 +9513,7 @@
         </is>
       </c>
       <c r="C130" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
@@ -9580,7 +9580,7 @@
         </is>
       </c>
       <c r="C131" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
@@ -9642,7 +9642,7 @@
         </is>
       </c>
       <c r="C132" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
@@ -9702,7 +9702,7 @@
         </is>
       </c>
       <c r="C133" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
@@ -9762,7 +9762,7 @@
         </is>
       </c>
       <c r="C134" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
@@ -9822,7 +9822,7 @@
         </is>
       </c>
       <c r="C135" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
@@ -9882,7 +9882,7 @@
         </is>
       </c>
       <c r="C136" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
@@ -9942,7 +9942,7 @@
         </is>
       </c>
       <c r="C137" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
@@ -10002,7 +10002,7 @@
         </is>
       </c>
       <c r="C138" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
@@ -10062,7 +10062,7 @@
         </is>
       </c>
       <c r="C139" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
         </is>
       </c>
       <c r="C140" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="C141" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
@@ -10242,7 +10242,7 @@
         </is>
       </c>
       <c r="C142" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="C143" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
         </is>
       </c>
       <c r="C144" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="C145" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
@@ -10482,7 +10482,7 @@
         </is>
       </c>
       <c r="C146" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
@@ -10542,7 +10542,7 @@
         </is>
       </c>
       <c r="C147" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
@@ -10602,7 +10602,7 @@
         </is>
       </c>
       <c r="C148" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="C149" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
@@ -10722,7 +10722,7 @@
         </is>
       </c>
       <c r="C150" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="C151" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
@@ -10842,7 +10842,7 @@
         </is>
       </c>
       <c r="C152" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="C153" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
@@ -10962,7 +10962,7 @@
         </is>
       </c>
       <c r="C154" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
@@ -11022,7 +11022,7 @@
         </is>
       </c>
       <c r="C155" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
@@ -11082,7 +11082,7 @@
         </is>
       </c>
       <c r="C156" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="C157" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
@@ -11202,7 +11202,7 @@
         </is>
       </c>
       <c r="C158" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
@@ -11262,7 +11262,7 @@
         </is>
       </c>
       <c r="C159" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
@@ -11324,7 +11324,7 @@
         </is>
       </c>
       <c r="C160" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
@@ -11389,7 +11389,7 @@
         </is>
       </c>
       <c r="C161" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
@@ -11454,7 +11454,7 @@
         </is>
       </c>
       <c r="C162" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
@@ -11516,7 +11516,7 @@
         </is>
       </c>
       <c r="C163" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
@@ -11583,7 +11583,7 @@
         </is>
       </c>
       <c r="C164" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
@@ -11643,7 +11643,7 @@
         </is>
       </c>
       <c r="C165" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
@@ -11705,7 +11705,7 @@
         </is>
       </c>
       <c r="C166" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
@@ -11765,7 +11765,7 @@
         </is>
       </c>
       <c r="C167" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
@@ -11825,7 +11825,7 @@
         </is>
       </c>
       <c r="C168" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
         </is>
       </c>
       <c r="C169" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="C170" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
@@ -12005,7 +12005,7 @@
         </is>
       </c>
       <c r="C171" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
@@ -12065,7 +12065,7 @@
         </is>
       </c>
       <c r="C172" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D172" s="7" t="inlineStr">
         <is>
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="C173" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
@@ -12189,7 +12189,7 @@
         </is>
       </c>
       <c r="C174" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
@@ -12251,7 +12251,7 @@
         </is>
       </c>
       <c r="C175" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D175" s="7" t="inlineStr">
         <is>
@@ -12313,7 +12313,7 @@
         </is>
       </c>
       <c r="C176" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D176" s="7" t="inlineStr">
         <is>
@@ -12375,7 +12375,7 @@
         </is>
       </c>
       <c r="C177" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D177" s="7" t="inlineStr">
         <is>
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="C178" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D178" s="7" t="inlineStr">
         <is>
@@ -12499,7 +12499,7 @@
         </is>
       </c>
       <c r="C179" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D179" s="7" t="inlineStr">
         <is>
@@ -12561,7 +12561,7 @@
         </is>
       </c>
       <c r="C180" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
         </is>
       </c>
       <c r="C181" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
@@ -12685,7 +12685,7 @@
         </is>
       </c>
       <c r="C182" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
@@ -12747,7 +12747,7 @@
         </is>
       </c>
       <c r="C183" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
@@ -12809,7 +12809,7 @@
         </is>
       </c>
       <c r="C184" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D184" s="7" t="inlineStr">
         <is>
@@ -12871,7 +12871,7 @@
         </is>
       </c>
       <c r="C185" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D185" s="7" t="inlineStr">
         <is>
@@ -12933,7 +12933,7 @@
         </is>
       </c>
       <c r="C186" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D186" s="7" t="inlineStr">
         <is>
@@ -12995,7 +12995,7 @@
         </is>
       </c>
       <c r="C187" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D187" s="7" t="inlineStr">
         <is>
@@ -13057,7 +13057,7 @@
         </is>
       </c>
       <c r="C188" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D188" s="7" t="inlineStr">
         <is>
@@ -13119,7 +13119,7 @@
         </is>
       </c>
       <c r="C189" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D189" s="7" t="inlineStr">
         <is>
@@ -13181,7 +13181,7 @@
         </is>
       </c>
       <c r="C190" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D190" s="7" t="inlineStr">
         <is>
@@ -13243,7 +13243,7 @@
         </is>
       </c>
       <c r="C191" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D191" s="7" t="inlineStr">
         <is>
@@ -13303,7 +13303,7 @@
         </is>
       </c>
       <c r="C192" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D192" s="7" t="inlineStr">
         <is>
@@ -13363,7 +13363,7 @@
         </is>
       </c>
       <c r="C193" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D193" s="7" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         </is>
       </c>
       <c r="C194" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D194" s="7" t="inlineStr">
         <is>
@@ -13483,7 +13483,7 @@
         </is>
       </c>
       <c r="C195" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D195" s="7" t="inlineStr">
         <is>
@@ -13543,7 +13543,7 @@
         </is>
       </c>
       <c r="C196" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D196" s="7" t="inlineStr">
         <is>
@@ -13603,7 +13603,7 @@
         </is>
       </c>
       <c r="C197" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D197" s="7" t="inlineStr">
         <is>
@@ -13660,7 +13660,7 @@
         </is>
       </c>
       <c r="C198" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D198" s="7" t="inlineStr">
         <is>
@@ -13720,7 +13720,7 @@
         </is>
       </c>
       <c r="C199" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D199" s="7" t="inlineStr">
         <is>
@@ -13780,7 +13780,7 @@
         </is>
       </c>
       <c r="C200" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D200" s="7" t="inlineStr">
         <is>
@@ -13840,7 +13840,7 @@
         </is>
       </c>
       <c r="C201" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D201" s="7" t="inlineStr">
         <is>
@@ -13900,7 +13900,7 @@
         </is>
       </c>
       <c r="C202" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D202" s="7" t="inlineStr">
         <is>
@@ -13960,7 +13960,7 @@
         </is>
       </c>
       <c r="C203" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D203" s="7" t="inlineStr">
         <is>
@@ -14020,7 +14020,7 @@
         </is>
       </c>
       <c r="C204" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D204" s="7" t="inlineStr">
         <is>
@@ -14080,7 +14080,7 @@
         </is>
       </c>
       <c r="C205" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D205" s="7" t="inlineStr">
         <is>
@@ -14140,7 +14140,7 @@
         </is>
       </c>
       <c r="C206" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D206" s="7" t="inlineStr">
         <is>
@@ -14200,7 +14200,7 @@
         </is>
       </c>
       <c r="C207" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D207" s="7" t="inlineStr">
         <is>
@@ -14260,7 +14260,7 @@
         </is>
       </c>
       <c r="C208" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D208" s="7" t="inlineStr">
         <is>
@@ -14320,7 +14320,7 @@
         </is>
       </c>
       <c r="C209" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D209" s="7" t="inlineStr">
         <is>
@@ -14382,7 +14382,7 @@
         </is>
       </c>
       <c r="C210" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D210" s="7" t="inlineStr">
         <is>
@@ -14444,7 +14444,7 @@
         </is>
       </c>
       <c r="C211" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D211" s="7" t="inlineStr">
         <is>
@@ -14506,7 +14506,7 @@
         </is>
       </c>
       <c r="C212" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D212" s="7" t="inlineStr">
         <is>
@@ -14568,7 +14568,7 @@
         </is>
       </c>
       <c r="C213" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D213" s="7" t="inlineStr">
         <is>
@@ -14630,7 +14630,7 @@
         </is>
       </c>
       <c r="C214" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D214" s="7" t="inlineStr">
         <is>
@@ -14692,7 +14692,7 @@
         </is>
       </c>
       <c r="C215" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D215" s="7" t="inlineStr">
         <is>
@@ -14754,7 +14754,7 @@
         </is>
       </c>
       <c r="C216" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D216" s="7" t="inlineStr">
         <is>
@@ -14814,7 +14814,7 @@
         </is>
       </c>
       <c r="C217" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D217" s="7" t="inlineStr">
         <is>
@@ -14874,7 +14874,7 @@
         </is>
       </c>
       <c r="C218" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D218" s="7" t="inlineStr">
         <is>
@@ -14934,7 +14934,7 @@
         </is>
       </c>
       <c r="C219" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D219" s="7" t="inlineStr">
         <is>
@@ -14994,7 +14994,7 @@
         </is>
       </c>
       <c r="C220" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D220" s="7" t="inlineStr">
         <is>
@@ -15054,7 +15054,7 @@
         </is>
       </c>
       <c r="C221" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D221" s="7" t="inlineStr">
         <is>
@@ -15114,7 +15114,7 @@
         </is>
       </c>
       <c r="C222" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D222" s="7" t="inlineStr">
         <is>
@@ -15174,7 +15174,7 @@
         </is>
       </c>
       <c r="C223" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D223" s="7" t="inlineStr">
         <is>
@@ -15234,7 +15234,7 @@
         </is>
       </c>
       <c r="C224" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D224" s="7" t="inlineStr">
         <is>
@@ -15294,7 +15294,7 @@
         </is>
       </c>
       <c r="C225" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D225" s="7" t="inlineStr">
         <is>
@@ -15354,7 +15354,7 @@
         </is>
       </c>
       <c r="C226" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D226" s="1" t="inlineStr">
         <is>
@@ -15416,7 +15416,7 @@
         </is>
       </c>
       <c r="C227" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D227" s="1" t="inlineStr">
         <is>
@@ -15478,7 +15478,7 @@
         </is>
       </c>
       <c r="C228" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D228" s="1" t="inlineStr">
         <is>
@@ -15540,7 +15540,7 @@
         </is>
       </c>
       <c r="C229" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D229" s="1" t="inlineStr">
         <is>
@@ -15602,7 +15602,7 @@
         </is>
       </c>
       <c r="C230" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D230" s="1" t="inlineStr">
         <is>
@@ -15664,7 +15664,7 @@
         </is>
       </c>
       <c r="C231" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D231" s="1" t="inlineStr">
         <is>
@@ -15726,7 +15726,7 @@
         </is>
       </c>
       <c r="C232" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D232" s="1" t="inlineStr">
         <is>
@@ -15788,7 +15788,7 @@
         </is>
       </c>
       <c r="C233" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D233" s="7" t="inlineStr">
         <is>
@@ -15850,7 +15850,7 @@
         </is>
       </c>
       <c r="C234" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D234" s="7" t="inlineStr">
         <is>
@@ -15912,7 +15912,7 @@
         </is>
       </c>
       <c r="C235" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D235" s="1" t="inlineStr">
         <is>
@@ -15974,7 +15974,7 @@
         </is>
       </c>
       <c r="C236" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D236" s="1" t="inlineStr">
         <is>
@@ -16036,7 +16036,7 @@
         </is>
       </c>
       <c r="C237" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D237" s="1" t="inlineStr">
         <is>
@@ -16098,7 +16098,7 @@
         </is>
       </c>
       <c r="C238" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D238" s="1" t="inlineStr">
         <is>
@@ -16160,7 +16160,7 @@
         </is>
       </c>
       <c r="C239" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D239" s="1" t="inlineStr">
         <is>
@@ -16222,7 +16222,7 @@
         </is>
       </c>
       <c r="C240" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D240" s="1" t="inlineStr">
         <is>
@@ -16284,7 +16284,7 @@
         </is>
       </c>
       <c r="C241" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D241" s="1" t="inlineStr">
         <is>
@@ -16346,7 +16346,7 @@
         </is>
       </c>
       <c r="C242" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D242" s="1" t="inlineStr">
         <is>
@@ -16408,7 +16408,7 @@
         </is>
       </c>
       <c r="C243" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D243" s="1" t="inlineStr">
         <is>
@@ -16470,7 +16470,7 @@
         </is>
       </c>
       <c r="C244" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D244" s="1" t="inlineStr">
         <is>
@@ -16532,7 +16532,7 @@
         </is>
       </c>
       <c r="C245" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D245" s="1" t="inlineStr">
         <is>
@@ -16594,7 +16594,7 @@
         </is>
       </c>
       <c r="C246" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D246" s="1" t="inlineStr">
         <is>
@@ -16656,7 +16656,7 @@
         </is>
       </c>
       <c r="C247" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D247" s="7" t="inlineStr">
         <is>
@@ -16718,7 +16718,7 @@
         </is>
       </c>
       <c r="C248" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D248" s="1" t="inlineStr">
         <is>
@@ -16780,7 +16780,7 @@
         </is>
       </c>
       <c r="C249" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D249" s="1" t="inlineStr">
         <is>
@@ -16842,7 +16842,7 @@
         </is>
       </c>
       <c r="C250" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D250" s="1" t="inlineStr">
         <is>
@@ -16904,7 +16904,7 @@
         </is>
       </c>
       <c r="C251" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D251" s="1" t="inlineStr">
         <is>
@@ -16966,7 +16966,7 @@
         </is>
       </c>
       <c r="C252" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D252" s="1" t="inlineStr">
         <is>
@@ -17028,7 +17028,7 @@
         </is>
       </c>
       <c r="C253" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D253" s="1" t="inlineStr">
         <is>
@@ -17090,7 +17090,7 @@
         </is>
       </c>
       <c r="C254" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D254" s="1" t="inlineStr">
         <is>
@@ -17152,7 +17152,7 @@
         </is>
       </c>
       <c r="C255" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D255" s="1" t="inlineStr">
         <is>
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="C256" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D256" s="1" t="inlineStr">
         <is>
@@ -17276,7 +17276,7 @@
         </is>
       </c>
       <c r="C257" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D257" s="1" t="inlineStr">
         <is>
@@ -17338,7 +17338,7 @@
         </is>
       </c>
       <c r="C258" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D258" s="1" t="inlineStr">
         <is>
@@ -17400,7 +17400,7 @@
         </is>
       </c>
       <c r="C259" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D259" s="1" t="inlineStr">
         <is>
@@ -17462,7 +17462,7 @@
         </is>
       </c>
       <c r="C260" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D260" s="1" t="inlineStr">
         <is>
@@ -17524,7 +17524,7 @@
         </is>
       </c>
       <c r="C261" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D261" s="1" t="inlineStr">
         <is>
@@ -17586,7 +17586,7 @@
         </is>
       </c>
       <c r="C262" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D262" s="1" t="inlineStr">
         <is>
@@ -17648,7 +17648,7 @@
         </is>
       </c>
       <c r="C263" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D263" s="1" t="inlineStr">
         <is>
@@ -17710,7 +17710,7 @@
         </is>
       </c>
       <c r="C264" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D264" s="1" t="inlineStr">
         <is>
@@ -17772,7 +17772,7 @@
         </is>
       </c>
       <c r="C265" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D265" s="1" t="inlineStr">
         <is>
@@ -17834,7 +17834,7 @@
         </is>
       </c>
       <c r="C266" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D266" s="1" t="inlineStr">
         <is>
@@ -17896,7 +17896,7 @@
         </is>
       </c>
       <c r="C267" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D267" s="1" t="inlineStr">
         <is>
@@ -17958,7 +17958,7 @@
         </is>
       </c>
       <c r="C268" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D268" s="1" t="inlineStr">
         <is>
@@ -18020,7 +18020,7 @@
         </is>
       </c>
       <c r="C269" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
@@ -18082,7 +18082,7 @@
         </is>
       </c>
       <c r="C270" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D270" s="1" t="inlineStr">
         <is>
@@ -18144,7 +18144,7 @@
         </is>
       </c>
       <c r="C271" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
@@ -18206,7 +18206,7 @@
         </is>
       </c>
       <c r="C272" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
@@ -18268,7 +18268,7 @@
         </is>
       </c>
       <c r="C273" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D273" s="1" t="inlineStr">
         <is>
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="C274" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D274" s="1" t="inlineStr">
         <is>
@@ -18392,7 +18392,7 @@
         </is>
       </c>
       <c r="C275" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D275" s="1" t="inlineStr">
         <is>
@@ -18454,7 +18454,7 @@
         </is>
       </c>
       <c r="C276" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D276" s="1" t="inlineStr">
         <is>
@@ -18516,7 +18516,7 @@
         </is>
       </c>
       <c r="C277" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D277" s="1" t="inlineStr">
         <is>
@@ -18578,7 +18578,7 @@
         </is>
       </c>
       <c r="C278" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D278" s="1" t="inlineStr">
         <is>
@@ -18640,7 +18640,7 @@
         </is>
       </c>
       <c r="C279" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
@@ -18702,7 +18702,7 @@
         </is>
       </c>
       <c r="C280" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
@@ -18764,7 +18764,7 @@
         </is>
       </c>
       <c r="C281" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
@@ -18826,7 +18826,7 @@
         </is>
       </c>
       <c r="C282" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D282" s="1" t="inlineStr">
         <is>
@@ -18888,7 +18888,7 @@
         </is>
       </c>
       <c r="C283" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
@@ -18950,7 +18950,7 @@
         </is>
       </c>
       <c r="C284" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
@@ -19012,7 +19012,7 @@
         </is>
       </c>
       <c r="C285" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
@@ -19074,7 +19074,7 @@
         </is>
       </c>
       <c r="C286" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D286" s="7" t="inlineStr">
         <is>
@@ -19141,7 +19141,7 @@
         </is>
       </c>
       <c r="C287" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D287" s="7" t="inlineStr">
         <is>
@@ -19208,7 +19208,7 @@
         </is>
       </c>
       <c r="C288" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D288" s="7" t="inlineStr">
         <is>
@@ -19275,7 +19275,7 @@
         </is>
       </c>
       <c r="C289" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D289" s="7" t="inlineStr">
         <is>
@@ -19342,7 +19342,7 @@
         </is>
       </c>
       <c r="C290" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D290" s="7" t="inlineStr">
         <is>
@@ -19409,7 +19409,7 @@
         </is>
       </c>
       <c r="C291" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D291" s="7" t="inlineStr">
         <is>
@@ -19476,7 +19476,7 @@
         </is>
       </c>
       <c r="C292" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D292" s="7" t="inlineStr">
         <is>
@@ -19543,7 +19543,7 @@
         </is>
       </c>
       <c r="C293" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D293" s="7" t="inlineStr">
         <is>
@@ -19610,7 +19610,7 @@
         </is>
       </c>
       <c r="C294" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D294" s="7" t="inlineStr">
         <is>
@@ -19677,7 +19677,7 @@
         </is>
       </c>
       <c r="C295" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D295" s="7" t="inlineStr">
         <is>
@@ -19744,7 +19744,7 @@
         </is>
       </c>
       <c r="C296" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D296" s="7" t="inlineStr">
         <is>
@@ -19811,7 +19811,7 @@
         </is>
       </c>
       <c r="C297" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D297" s="7" t="inlineStr">
         <is>
@@ -19878,7 +19878,7 @@
         </is>
       </c>
       <c r="C298" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D298" s="7" t="inlineStr">
         <is>
@@ -19945,7 +19945,7 @@
         </is>
       </c>
       <c r="C299" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D299" s="7" t="inlineStr">
         <is>
@@ -20012,7 +20012,7 @@
         </is>
       </c>
       <c r="C300" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D300" s="7" t="inlineStr">
         <is>
@@ -20079,7 +20079,7 @@
         </is>
       </c>
       <c r="C301" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D301" s="7" t="inlineStr">
         <is>
@@ -20146,7 +20146,7 @@
         </is>
       </c>
       <c r="C302" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D302" s="7" t="inlineStr">
         <is>
@@ -20213,7 +20213,7 @@
         </is>
       </c>
       <c r="C303" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D303" s="7" t="inlineStr">
         <is>
@@ -20280,7 +20280,7 @@
         </is>
       </c>
       <c r="C304" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D304" s="7" t="inlineStr">
         <is>
@@ -20347,7 +20347,7 @@
         </is>
       </c>
       <c r="C305" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D305" s="7" t="inlineStr">
         <is>
@@ -20414,7 +20414,7 @@
         </is>
       </c>
       <c r="C306" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D306" s="7" t="inlineStr">
         <is>
@@ -20481,7 +20481,7 @@
         </is>
       </c>
       <c r="C307" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D307" s="7" t="inlineStr">
         <is>
@@ -20548,7 +20548,7 @@
         </is>
       </c>
       <c r="C308" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D308" s="7" t="inlineStr">
         <is>
@@ -20615,7 +20615,7 @@
         </is>
       </c>
       <c r="C309" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D309" s="7" t="inlineStr">
         <is>
@@ -20682,7 +20682,7 @@
         </is>
       </c>
       <c r="C310" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D310" s="7" t="inlineStr">
         <is>
@@ -20749,7 +20749,7 @@
         </is>
       </c>
       <c r="C311" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D311" s="7" t="inlineStr">
         <is>
@@ -20816,7 +20816,7 @@
         </is>
       </c>
       <c r="C312" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D312" s="7" t="inlineStr">
         <is>
@@ -20883,7 +20883,7 @@
         </is>
       </c>
       <c r="C313" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D313" s="7" t="inlineStr">
         <is>
@@ -20950,7 +20950,7 @@
         </is>
       </c>
       <c r="C314" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D314" s="7" t="inlineStr">
         <is>
@@ -21017,7 +21017,7 @@
         </is>
       </c>
       <c r="C315" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D315" s="7" t="inlineStr">
         <is>
@@ -21084,7 +21084,7 @@
         </is>
       </c>
       <c r="C316" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D316" s="7" t="inlineStr">
         <is>
@@ -21151,7 +21151,7 @@
         </is>
       </c>
       <c r="C317" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D317" s="7" t="inlineStr">
         <is>
@@ -21218,7 +21218,7 @@
         </is>
       </c>
       <c r="C318" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D318" s="7" t="inlineStr">
         <is>
@@ -21285,7 +21285,7 @@
         </is>
       </c>
       <c r="C319" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D319" s="7" t="inlineStr">
         <is>
@@ -21352,7 +21352,7 @@
         </is>
       </c>
       <c r="C320" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D320" s="7" t="inlineStr">
         <is>
@@ -21419,7 +21419,7 @@
         </is>
       </c>
       <c r="C321" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D321" s="7" t="inlineStr">
         <is>
@@ -21486,7 +21486,7 @@
         </is>
       </c>
       <c r="C322" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D322" s="7" t="inlineStr">
         <is>
@@ -21553,7 +21553,7 @@
         </is>
       </c>
       <c r="C323" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D323" s="7" t="inlineStr">
         <is>
@@ -21620,7 +21620,7 @@
         </is>
       </c>
       <c r="C324" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D324" s="7" t="inlineStr">
         <is>
@@ -21687,7 +21687,7 @@
         </is>
       </c>
       <c r="C325" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D325" s="7" t="inlineStr">
         <is>
@@ -21754,7 +21754,7 @@
         </is>
       </c>
       <c r="C326" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D326" s="7" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         </is>
       </c>
       <c r="C327" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D327" s="7" t="inlineStr">
         <is>
@@ -21888,7 +21888,7 @@
         </is>
       </c>
       <c r="C328" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D328" s="7" t="inlineStr">
         <is>
@@ -21955,7 +21955,7 @@
         </is>
       </c>
       <c r="C329" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D329" s="7" t="inlineStr">
         <is>
@@ -22022,7 +22022,7 @@
         </is>
       </c>
       <c r="C330" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D330" s="7" t="inlineStr">
         <is>
@@ -22089,7 +22089,7 @@
         </is>
       </c>
       <c r="C331" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D331" s="7" t="inlineStr">
         <is>
@@ -22156,7 +22156,7 @@
         </is>
       </c>
       <c r="C332" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D332" s="7" t="inlineStr">
         <is>
@@ -22223,7 +22223,7 @@
         </is>
       </c>
       <c r="C333" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D333" s="7" t="inlineStr">
         <is>
@@ -22290,7 +22290,7 @@
         </is>
       </c>
       <c r="C334" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D334" s="7" t="inlineStr">
         <is>
@@ -22357,7 +22357,7 @@
         </is>
       </c>
       <c r="C335" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D335" s="7" t="inlineStr">
         <is>
@@ -22424,7 +22424,7 @@
         </is>
       </c>
       <c r="C336" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D336" s="7" t="inlineStr">
         <is>
@@ -22491,7 +22491,7 @@
         </is>
       </c>
       <c r="C337" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D337" s="7" t="inlineStr">
         <is>
@@ -22558,7 +22558,7 @@
         </is>
       </c>
       <c r="C338" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D338" s="7" t="inlineStr">
         <is>
@@ -22625,7 +22625,7 @@
         </is>
       </c>
       <c r="C339" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D339" s="7" t="inlineStr">
         <is>
@@ -22692,7 +22692,7 @@
         </is>
       </c>
       <c r="C340" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D340" s="7" t="inlineStr">
         <is>
@@ -22752,7 +22752,7 @@
         </is>
       </c>
       <c r="C341" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D341" s="7" t="inlineStr">
         <is>
@@ -22812,7 +22812,7 @@
         </is>
       </c>
       <c r="C342" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D342" s="7" t="inlineStr">
         <is>
@@ -22872,7 +22872,7 @@
         </is>
       </c>
       <c r="C343" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D343" s="7" t="inlineStr">
         <is>
@@ -22932,7 +22932,7 @@
         </is>
       </c>
       <c r="C344" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D344" s="7" t="inlineStr">
         <is>
@@ -22992,7 +22992,7 @@
         </is>
       </c>
       <c r="C345" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D345" s="7" t="inlineStr">
         <is>
@@ -23052,7 +23052,7 @@
         </is>
       </c>
       <c r="C346" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D346" s="1" t="inlineStr">
         <is>
@@ -23112,7 +23112,7 @@
         </is>
       </c>
       <c r="C347" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D347" s="7" t="inlineStr">
         <is>
@@ -23172,7 +23172,7 @@
         </is>
       </c>
       <c r="C348" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D348" s="7" t="inlineStr">
         <is>
@@ -23232,7 +23232,7 @@
         </is>
       </c>
       <c r="C349" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D349" s="7" t="inlineStr">
         <is>
@@ -23292,7 +23292,7 @@
         </is>
       </c>
       <c r="C350" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D350" s="7" t="inlineStr">
         <is>
@@ -23352,7 +23352,7 @@
         </is>
       </c>
       <c r="C351" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D351" s="7" t="inlineStr">
         <is>
@@ -23412,7 +23412,7 @@
         </is>
       </c>
       <c r="C352" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D352" s="7" t="inlineStr">
         <is>
@@ -23472,7 +23472,7 @@
         </is>
       </c>
       <c r="C353" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D353" s="7" t="inlineStr">
         <is>
@@ -23532,7 +23532,7 @@
         </is>
       </c>
       <c r="C354" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D354" s="7" t="inlineStr">
         <is>
@@ -23592,7 +23592,7 @@
         </is>
       </c>
       <c r="C355" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D355" s="7" t="inlineStr">
         <is>
@@ -23652,7 +23652,7 @@
         </is>
       </c>
       <c r="C356" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D356" s="7" t="inlineStr">
         <is>
@@ -23712,7 +23712,7 @@
         </is>
       </c>
       <c r="C357" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D357" s="7" t="inlineStr">
         <is>
@@ -23772,7 +23772,7 @@
         </is>
       </c>
       <c r="C358" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D358" s="7" t="inlineStr">
         <is>
@@ -23832,7 +23832,7 @@
         </is>
       </c>
       <c r="C359" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D359" s="7" t="inlineStr">
         <is>
@@ -23892,7 +23892,7 @@
         </is>
       </c>
       <c r="C360" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D360" s="7" t="inlineStr">
         <is>
@@ -23952,7 +23952,7 @@
         </is>
       </c>
       <c r="C361" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D361" s="7" t="inlineStr">
         <is>
@@ -24019,7 +24019,7 @@
         </is>
       </c>
       <c r="C362" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D362" s="7" t="inlineStr">
         <is>
@@ -24079,7 +24079,7 @@
         </is>
       </c>
       <c r="C363" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D363" s="7" t="inlineStr">
         <is>
@@ -24139,7 +24139,7 @@
         </is>
       </c>
       <c r="C364" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D364" s="7" t="inlineStr">
         <is>
@@ -24199,7 +24199,7 @@
         </is>
       </c>
       <c r="C365" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D365" s="7" t="inlineStr">
         <is>
@@ -24259,7 +24259,7 @@
         </is>
       </c>
       <c r="C366" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D366" s="7" t="inlineStr">
         <is>
@@ -24319,7 +24319,7 @@
         </is>
       </c>
       <c r="C367" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D367" s="7" t="inlineStr">
         <is>
@@ -24379,7 +24379,7 @@
         </is>
       </c>
       <c r="C368" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D368" s="7" t="inlineStr">
         <is>
@@ -24439,7 +24439,7 @@
         </is>
       </c>
       <c r="C369" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D369" s="7" t="inlineStr">
         <is>
@@ -24499,7 +24499,7 @@
         </is>
       </c>
       <c r="C370" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D370" s="7" t="inlineStr">
         <is>
@@ -24559,7 +24559,7 @@
         </is>
       </c>
       <c r="C371" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D371" s="7" t="inlineStr">
         <is>
@@ -24619,7 +24619,7 @@
         </is>
       </c>
       <c r="C372" s="10" t="n">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="D372" s="7" t="inlineStr">
         <is>
@@ -24680,7 +24680,7 @@
         </is>
       </c>
       <c r="C373" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D373" s="7" t="inlineStr">
         <is>
@@ -24743,7 +24743,7 @@
         </is>
       </c>
       <c r="C374" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D374" s="7" t="inlineStr">
         <is>
@@ -24806,7 +24806,7 @@
         </is>
       </c>
       <c r="C375" s="22" t="n">
-        <v>46055</v>
+        <v>46086</v>
       </c>
       <c r="D375" s="7" t="inlineStr">
         <is>
@@ -24869,7 +24869,7 @@
         </is>
       </c>
       <c r="C376" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D376" s="7" t="inlineStr">
         <is>
@@ -24932,7 +24932,7 @@
         </is>
       </c>
       <c r="C377" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D377" s="7" t="inlineStr">
         <is>
@@ -24995,7 +24995,7 @@
         </is>
       </c>
       <c r="C378" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D378" s="7" t="inlineStr">
         <is>
@@ -25058,7 +25058,7 @@
         </is>
       </c>
       <c r="C379" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D379" s="7" t="inlineStr">
         <is>
@@ -25121,7 +25121,7 @@
         </is>
       </c>
       <c r="C380" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D380" s="7" t="inlineStr">
         <is>
@@ -25184,7 +25184,7 @@
         </is>
       </c>
       <c r="C381" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D381" s="7" t="inlineStr">
         <is>
@@ -25247,7 +25247,7 @@
         </is>
       </c>
       <c r="C382" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D382" s="7" t="inlineStr">
         <is>
@@ -25310,7 +25310,7 @@
         </is>
       </c>
       <c r="C383" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D383" s="7" t="inlineStr">
         <is>
@@ -25373,7 +25373,7 @@
         </is>
       </c>
       <c r="C384" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D384" s="7" t="inlineStr">
         <is>
@@ -25436,7 +25436,7 @@
         </is>
       </c>
       <c r="C385" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D385" s="7" t="inlineStr">
         <is>
@@ -25499,7 +25499,7 @@
         </is>
       </c>
       <c r="C386" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D386" s="7" t="inlineStr">
         <is>
@@ -25562,7 +25562,7 @@
         </is>
       </c>
       <c r="C387" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D387" s="7" t="inlineStr">
         <is>
@@ -25625,7 +25625,7 @@
         </is>
       </c>
       <c r="C388" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D388" s="7" t="inlineStr">
         <is>
@@ -25688,7 +25688,7 @@
         </is>
       </c>
       <c r="C389" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D389" s="7" t="inlineStr">
         <is>
@@ -25751,7 +25751,7 @@
         </is>
       </c>
       <c r="C390" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D390" s="7" t="inlineStr">
         <is>
@@ -25814,7 +25814,7 @@
         </is>
       </c>
       <c r="C391" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D391" s="7" t="inlineStr">
         <is>
@@ -25877,7 +25877,7 @@
         </is>
       </c>
       <c r="C392" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D392" s="7" t="inlineStr">
         <is>
@@ -25940,7 +25940,7 @@
         </is>
       </c>
       <c r="C393" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D393" s="7" t="inlineStr">
         <is>
@@ -26003,7 +26003,7 @@
         </is>
       </c>
       <c r="C394" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D394" s="7" t="inlineStr">
         <is>
@@ -26066,7 +26066,7 @@
         </is>
       </c>
       <c r="C395" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D395" s="7" t="inlineStr">
         <is>
@@ -26129,7 +26129,7 @@
         </is>
       </c>
       <c r="C396" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D396" s="7" t="inlineStr">
         <is>
@@ -26192,7 +26192,7 @@
         </is>
       </c>
       <c r="C397" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D397" s="7" t="inlineStr">
         <is>
@@ -26255,7 +26255,7 @@
         </is>
       </c>
       <c r="C398" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D398" s="7" t="inlineStr">
         <is>
@@ -26318,7 +26318,7 @@
         </is>
       </c>
       <c r="C399" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D399" s="7" t="inlineStr">
         <is>
@@ -26381,7 +26381,7 @@
         </is>
       </c>
       <c r="C400" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D400" s="7" t="inlineStr">
         <is>
@@ -26444,7 +26444,7 @@
         </is>
       </c>
       <c r="C401" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D401" s="7" t="inlineStr">
         <is>
@@ -26507,7 +26507,7 @@
         </is>
       </c>
       <c r="C402" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D402" s="7" t="inlineStr">
         <is>
@@ -26570,7 +26570,7 @@
         </is>
       </c>
       <c r="C403" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D403" s="7" t="inlineStr">
         <is>
@@ -26633,7 +26633,7 @@
         </is>
       </c>
       <c r="C404" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D404" s="7" t="inlineStr">
         <is>
@@ -26696,7 +26696,7 @@
         </is>
       </c>
       <c r="C405" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D405" s="7" t="inlineStr">
         <is>
@@ -26759,7 +26759,7 @@
         </is>
       </c>
       <c r="C406" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D406" s="7" t="inlineStr">
         <is>
@@ -26822,7 +26822,7 @@
         </is>
       </c>
       <c r="C407" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D407" s="7" t="inlineStr">
         <is>
@@ -26885,7 +26885,7 @@
         </is>
       </c>
       <c r="C408" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D408" s="7" t="inlineStr">
         <is>
@@ -26948,7 +26948,7 @@
         </is>
       </c>
       <c r="C409" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D409" s="7" t="inlineStr">
         <is>
@@ -27011,7 +27011,7 @@
         </is>
       </c>
       <c r="C410" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D410" s="7" t="inlineStr">
         <is>
@@ -27074,7 +27074,7 @@
         </is>
       </c>
       <c r="C411" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D411" s="7" t="inlineStr">
         <is>
@@ -27137,7 +27137,7 @@
         </is>
       </c>
       <c r="C412" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D412" s="7" t="inlineStr">
         <is>
@@ -27200,7 +27200,7 @@
         </is>
       </c>
       <c r="C413" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D413" s="7" t="inlineStr">
         <is>
@@ -27263,7 +27263,7 @@
         </is>
       </c>
       <c r="C414" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D414" s="7" t="inlineStr">
         <is>
@@ -27326,7 +27326,7 @@
         </is>
       </c>
       <c r="C415" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D415" s="7" t="inlineStr">
         <is>
@@ -27389,7 +27389,7 @@
         </is>
       </c>
       <c r="C416" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D416" s="7" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
         </is>
       </c>
       <c r="C417" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D417" s="7" t="inlineStr">
         <is>
@@ -27515,7 +27515,7 @@
         </is>
       </c>
       <c r="C418" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D418" s="7" t="inlineStr">
         <is>
@@ -27578,7 +27578,7 @@
         </is>
       </c>
       <c r="C419" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D419" s="7" t="inlineStr">
         <is>
@@ -27641,7 +27641,7 @@
         </is>
       </c>
       <c r="C420" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D420" s="7" t="inlineStr">
         <is>
@@ -27704,7 +27704,7 @@
         </is>
       </c>
       <c r="C421" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D421" s="7" t="inlineStr">
         <is>
@@ -27767,7 +27767,7 @@
         </is>
       </c>
       <c r="C422" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D422" s="7" t="inlineStr">
         <is>
@@ -27830,7 +27830,7 @@
         </is>
       </c>
       <c r="C423" s="22" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D423" s="7" t="inlineStr">
         <is>
@@ -27893,7 +27893,7 @@
         </is>
       </c>
       <c r="C424" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D424" s="7" t="inlineStr">
         <is>
@@ -27961,7 +27961,7 @@
         </is>
       </c>
       <c r="C425" s="22" t="n">
-        <v>46066</v>
+        <v>46086</v>
       </c>
       <c r="D425" s="7" t="inlineStr">
         <is>
@@ -28024,7 +28024,7 @@
         </is>
       </c>
       <c r="C426" s="22" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="D426" s="7" t="inlineStr">
         <is>
@@ -28087,7 +28087,7 @@
         </is>
       </c>
       <c r="C427" s="24" t="n">
-        <v>46067</v>
+        <v>46086</v>
       </c>
       <c r="D427" s="7" t="inlineStr">
         <is>
@@ -28157,7 +28157,7 @@
         </is>
       </c>
       <c r="C428" s="24" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D428" s="7" t="inlineStr">
         <is>
@@ -28216,11 +28216,11 @@
       </c>
       <c r="B429" s="7" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>published</t>
         </is>
       </c>
       <c r="C429" s="24" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D429" s="7" t="inlineStr">
         <is>
@@ -28283,7 +28283,7 @@
         </is>
       </c>
       <c r="C430" s="24" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D430" s="7" t="inlineStr">
         <is>
@@ -28346,7 +28346,7 @@
         </is>
       </c>
       <c r="C431" s="24" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D431" s="7" t="inlineStr">
         <is>
@@ -28409,7 +28409,7 @@
         </is>
       </c>
       <c r="C432" s="24" t="n">
-        <v>46069</v>
+        <v>46086</v>
       </c>
       <c r="D432" s="7" t="inlineStr">
         <is>
@@ -28472,7 +28472,7 @@
         </is>
       </c>
       <c r="C433" s="22" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D433" s="7" t="inlineStr">
         <is>
@@ -28537,7 +28537,7 @@
         </is>
       </c>
       <c r="C434" s="24" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D434" s="7" t="inlineStr">
         <is>
@@ -28600,7 +28600,7 @@
         </is>
       </c>
       <c r="C435" s="24" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D435" s="7" t="inlineStr">
         <is>
@@ -28663,7 +28663,7 @@
         </is>
       </c>
       <c r="C436" s="24" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D436" s="7" t="inlineStr">
         <is>
@@ -28726,7 +28726,7 @@
         </is>
       </c>
       <c r="C437" s="24" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D437" s="7" t="inlineStr">
         <is>
@@ -28789,7 +28789,7 @@
         </is>
       </c>
       <c r="C438" s="24" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D438" s="7" t="inlineStr">
         <is>
@@ -28852,7 +28852,7 @@
         </is>
       </c>
       <c r="C439" s="24" t="n">
-        <v>46070</v>
+        <v>46086</v>
       </c>
       <c r="D439" s="7" t="inlineStr">
         <is>
@@ -28915,7 +28915,7 @@
         </is>
       </c>
       <c r="C440" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D440" s="7" t="inlineStr">
         <is>
@@ -28978,7 +28978,7 @@
         </is>
       </c>
       <c r="C441" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D441" s="7" t="inlineStr">
         <is>
@@ -29041,7 +29041,7 @@
         </is>
       </c>
       <c r="C442" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D442" s="7" t="inlineStr">
         <is>
@@ -29104,7 +29104,7 @@
         </is>
       </c>
       <c r="C443" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D443" s="7" t="inlineStr">
         <is>
@@ -29167,7 +29167,7 @@
         </is>
       </c>
       <c r="C444" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D444" s="7" t="inlineStr">
         <is>
@@ -29230,7 +29230,7 @@
         </is>
       </c>
       <c r="C445" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D445" s="7" t="inlineStr">
         <is>
@@ -29293,7 +29293,7 @@
         </is>
       </c>
       <c r="C446" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D446" s="7" t="inlineStr">
         <is>
@@ -29356,7 +29356,7 @@
         </is>
       </c>
       <c r="C447" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D447" s="7" t="inlineStr">
         <is>
@@ -29419,7 +29419,7 @@
         </is>
       </c>
       <c r="C448" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D448" s="7" t="inlineStr">
         <is>
@@ -29482,7 +29482,7 @@
         </is>
       </c>
       <c r="C449" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D449" s="7" t="inlineStr">
         <is>
@@ -29545,7 +29545,7 @@
         </is>
       </c>
       <c r="C450" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D450" s="7" t="inlineStr">
         <is>
@@ -29608,7 +29608,7 @@
         </is>
       </c>
       <c r="C451" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D451" s="7" t="inlineStr">
         <is>
@@ -29671,7 +29671,7 @@
         </is>
       </c>
       <c r="C452" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D452" s="7" t="inlineStr">
         <is>
@@ -29734,7 +29734,7 @@
         </is>
       </c>
       <c r="C453" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D453" s="7" t="inlineStr">
         <is>
@@ -29797,7 +29797,7 @@
         </is>
       </c>
       <c r="C454" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D454" s="7" t="inlineStr">
         <is>
@@ -29860,7 +29860,7 @@
         </is>
       </c>
       <c r="C455" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D455" s="7" t="inlineStr">
         <is>
@@ -29923,7 +29923,7 @@
         </is>
       </c>
       <c r="C456" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D456" s="7" t="inlineStr">
         <is>
@@ -29986,7 +29986,7 @@
         </is>
       </c>
       <c r="C457" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D457" s="7" t="inlineStr">
         <is>
@@ -30049,7 +30049,7 @@
         </is>
       </c>
       <c r="C458" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D458" s="7" t="inlineStr">
         <is>
@@ -30112,7 +30112,7 @@
         </is>
       </c>
       <c r="C459" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D459" s="7" t="inlineStr">
         <is>
@@ -30175,7 +30175,7 @@
         </is>
       </c>
       <c r="C460" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D460" s="7" t="inlineStr">
         <is>
@@ -30238,7 +30238,7 @@
         </is>
       </c>
       <c r="C461" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D461" s="7" t="inlineStr">
         <is>
@@ -30301,7 +30301,7 @@
         </is>
       </c>
       <c r="C462" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D462" s="7" t="inlineStr">
         <is>
@@ -30364,7 +30364,7 @@
         </is>
       </c>
       <c r="C463" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D463" s="7" t="inlineStr">
         <is>
@@ -30427,7 +30427,7 @@
         </is>
       </c>
       <c r="C464" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D464" s="7" t="inlineStr">
         <is>
@@ -30490,7 +30490,7 @@
         </is>
       </c>
       <c r="C465" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D465" s="7" t="inlineStr">
         <is>
@@ -30553,7 +30553,7 @@
         </is>
       </c>
       <c r="C466" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D466" s="7" t="inlineStr">
         <is>
@@ -30616,7 +30616,7 @@
         </is>
       </c>
       <c r="C467" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D467" s="7" t="inlineStr">
         <is>
@@ -30679,7 +30679,7 @@
         </is>
       </c>
       <c r="C468" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D468" s="7" t="inlineStr">
         <is>
@@ -30742,7 +30742,7 @@
         </is>
       </c>
       <c r="C469" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D469" s="7" t="inlineStr">
         <is>
@@ -30805,7 +30805,7 @@
         </is>
       </c>
       <c r="C470" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D470" s="7" t="inlineStr">
         <is>
@@ -30868,7 +30868,7 @@
         </is>
       </c>
       <c r="C471" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D471" s="7" t="inlineStr">
         <is>
@@ -30931,7 +30931,7 @@
         </is>
       </c>
       <c r="C472" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D472" s="7" t="inlineStr">
         <is>
@@ -30994,7 +30994,7 @@
         </is>
       </c>
       <c r="C473" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D473" s="7" t="inlineStr">
         <is>
@@ -31057,7 +31057,7 @@
         </is>
       </c>
       <c r="C474" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D474" s="7" t="inlineStr">
         <is>
@@ -31120,7 +31120,7 @@
         </is>
       </c>
       <c r="C475" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D475" s="7" t="inlineStr">
         <is>
@@ -31183,7 +31183,7 @@
         </is>
       </c>
       <c r="C476" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D476" s="7" t="inlineStr">
         <is>
@@ -31246,7 +31246,7 @@
         </is>
       </c>
       <c r="C477" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D477" s="7" t="inlineStr">
         <is>
@@ -31309,7 +31309,7 @@
         </is>
       </c>
       <c r="C478" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D478" s="7" t="inlineStr">
         <is>
@@ -31372,7 +31372,7 @@
         </is>
       </c>
       <c r="C479" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D479" s="7" t="inlineStr">
         <is>
@@ -31435,7 +31435,7 @@
         </is>
       </c>
       <c r="C480" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D480" s="7" t="inlineStr">
         <is>
@@ -31498,7 +31498,7 @@
         </is>
       </c>
       <c r="C481" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D481" s="7" t="inlineStr">
         <is>
@@ -31561,7 +31561,7 @@
         </is>
       </c>
       <c r="C482" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D482" s="7" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         </is>
       </c>
       <c r="C483" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D483" s="7" t="inlineStr">
         <is>
@@ -31687,7 +31687,7 @@
         </is>
       </c>
       <c r="C484" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D484" s="7" t="inlineStr">
         <is>
@@ -31750,7 +31750,7 @@
         </is>
       </c>
       <c r="C485" s="22" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D485" s="7" t="inlineStr">
         <is>
@@ -31813,7 +31813,7 @@
         </is>
       </c>
       <c r="C486" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D486" s="26" t="inlineStr">
         <is>
@@ -31876,7 +31876,7 @@
         </is>
       </c>
       <c r="C487" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D487" s="26" t="inlineStr">
         <is>
@@ -31939,7 +31939,7 @@
         </is>
       </c>
       <c r="C488" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D488" s="26" t="inlineStr">
         <is>
@@ -32002,7 +32002,7 @@
         </is>
       </c>
       <c r="C489" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D489" s="1" t="inlineStr">
         <is>
@@ -32067,7 +32067,7 @@
         </is>
       </c>
       <c r="C490" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D490" s="1" t="inlineStr">
         <is>
@@ -32126,7 +32126,7 @@
         </is>
       </c>
       <c r="C491" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D491" s="1" t="inlineStr">
         <is>
@@ -32185,7 +32185,7 @@
         </is>
       </c>
       <c r="C492" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D492" s="1" t="inlineStr">
         <is>
@@ -32244,7 +32244,7 @@
         </is>
       </c>
       <c r="C493" s="10" t="n">
-        <v>46071</v>
+        <v>46086</v>
       </c>
       <c r="D493" s="1" t="inlineStr">
         <is>
@@ -32303,7 +32303,7 @@
         </is>
       </c>
       <c r="C494" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D494" s="7" t="inlineStr">
         <is>
@@ -34279,7 +34279,7 @@
         </is>
       </c>
       <c r="C536" s="10" t="n">
-        <v>46074</v>
+        <v>46086</v>
       </c>
       <c r="D536" s="7" t="inlineStr">
         <is>

</xml_diff>